<commit_message>
atualiza dados e config para ploa 2024
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_QDD_INVESTIMENTO.xlsx
+++ b/bancos/SISOR/BASE_QDD_INVESTIMENTO.xlsx
@@ -534,29 +534,29 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B2" t="n">
-        <v>1190</v>
+        <v>1220</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE FAZENDA - SEF</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>5191</v>
+        <v>5011</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
+          <t>COMPANHIA DE DESENVOLVIMENTO ECONÔMICO DE MINAS GERAIS - CODEMIG</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>9796</v>
+        <v>10929</v>
       </c>
       <c r="H2" t="n">
         <v>4</v>
@@ -565,39 +565,39 @@
         <v>122</v>
       </c>
       <c r="J2" t="n">
-        <v>13</v>
+        <v>133</v>
       </c>
       <c r="K2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L2" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="M2" t="n">
-        <v>6011</v>
+        <v>3017</v>
       </c>
       <c r="N2" t="n">
-        <v>90000</v>
+        <v>1000</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>MANUTENÇÃO E AQUISIÇÕES DA CODEMIG</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R2" t="n">
-        <v>4817</v>
+        <v>4614</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>EQUIPAMENTOS E SOFTWARE</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T2" t="n">
@@ -610,81 +610,81 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>MANUTENÇÃO E AQUISIÇÕES DA CODEMIG</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>MINAS GERAÇÃO DE VALOR</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B3" t="n">
-        <v>1190</v>
+        <v>1220</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE FAZENDA - SEF</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D3" t="n">
         <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>5191</v>
+        <v>5031</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
+          <t>COMPANHIA DE DESENVOLVIMENTO DE MINAS GERAIS - CODEMG</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>9082</v>
+        <v>10927</v>
       </c>
       <c r="H3" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="I3" t="n">
-        <v>122</v>
+        <v>572</v>
       </c>
       <c r="J3" t="n">
-        <v>24</v>
+        <v>133</v>
       </c>
       <c r="K3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L3" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="M3" t="n">
-        <v>6003</v>
+        <v>3015</v>
       </c>
       <c r="N3" t="n">
-        <v>15882556</v>
+        <v>12580000</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
+          <t>GESTÃO DE INFRAESTRUTURA, CONSÓRCIOS E EQUIPAMENTOS CULTURAIS E TURÍSTICOS</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R3" t="n">
-        <v>4819</v>
+        <v>4613</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T3" t="n">
@@ -697,192 +697,192 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
+          <t>GESTÃO DE INFRAESTRUTURA, CONSÓRCIOS E EQUIPAMENTOS CULTURAIS E TURÍSTICOS</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>APOIO AO DESENVOLVIMENTO MUNICIPAL, À CAPTAÇÃO E À COORDENAÇÃO DA TRANSFERÊNCIA DE RECURSOS</t>
+          <t>MINAS GERAÇÃO DE VALOR</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B4" t="n">
-        <v>1190</v>
+        <v>1220</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE FAZENDA - SEF</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D4" t="n">
         <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>5191</v>
+        <v>5071</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
+          <t>COMPANHIA DE HABITAÇÃO DO ESTADO DE MINAS GERAIS - COHAB</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>9058</v>
+        <v>9775</v>
       </c>
       <c r="H4" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="I4" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J4" t="n">
-        <v>13</v>
+        <v>705</v>
       </c>
       <c r="K4" t="n">
         <v>6</v>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="M4" t="n">
-        <v>6001</v>
+        <v>6010</v>
       </c>
       <c r="N4" t="n">
-        <v>1000</v>
+        <v>120000</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA - COHAB</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R4" t="n">
-        <v>4511</v>
+        <v>4614</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T4" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA - COHAB</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B5" t="n">
-        <v>1190</v>
+        <v>1220</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE FAZENDA - SEF</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D5" t="n">
         <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>5191</v>
+        <v>5081</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
+          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>9058</v>
+        <v>11021</v>
       </c>
       <c r="H5" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I5" t="n">
-        <v>123</v>
+        <v>512</v>
       </c>
       <c r="J5" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="K5" t="n">
         <v>6</v>
       </c>
       <c r="L5" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="M5" t="n">
-        <v>6001</v>
+        <v>6009</v>
       </c>
       <c r="N5" t="n">
-        <v>1000</v>
+        <v>50000000</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R5" t="n">
-        <v>4511</v>
+        <v>4614</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T5" t="n">
-        <v>51000</v>
+        <v>22199</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B6" t="n">
         <v>1220</v>
@@ -896,56 +896,56 @@
         <v>3</v>
       </c>
       <c r="E6" t="n">
-        <v>5011</v>
+        <v>5081</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>COMPANHIA DE DESENVOLVIMENTO ECONÔMICO DE MINAS GERAIS - CODEMIG</t>
+          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>10011</v>
+        <v>11021</v>
       </c>
       <c r="H6" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I6" t="n">
-        <v>122</v>
+        <v>512</v>
       </c>
       <c r="J6" t="n">
-        <v>63</v>
+        <v>21</v>
       </c>
       <c r="K6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L6" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="M6" t="n">
-        <v>3014</v>
+        <v>6009</v>
       </c>
       <c r="N6" t="n">
-        <v>1000</v>
+        <v>50000000</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E AQUISIÇÕES DA CODEMIG</t>
+          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R6" t="n">
-        <v>4819</v>
+        <v>4614</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T6" t="n">
@@ -958,18 +958,18 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E AQUISIÇÕES DA CODEMIG</t>
+          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>MINAS + GERAIS - DIVERSIFICAÇÃO E FORTALECIMENTO DA ECONOMIA</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B7" t="n">
         <v>1220</v>
@@ -983,56 +983,56 @@
         <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>5031</v>
+        <v>5081</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>COMPANHIA DE DESENVOLVIMENTO DE MINAS GERAIS - CODEMG</t>
+          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>9617</v>
+        <v>11022</v>
       </c>
       <c r="H7" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="I7" t="n">
-        <v>572</v>
+        <v>512</v>
       </c>
       <c r="J7" t="n">
-        <v>63</v>
+        <v>21</v>
       </c>
       <c r="K7" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L7" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="M7" t="n">
-        <v>3017</v>
+        <v>8008</v>
       </c>
       <c r="N7" t="n">
-        <v>14119841</v>
+        <v>100000000</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>GESTÃO DE PARTICIPAÇÕES, FUNDOS, CONSÓRCIOS, P&amp;D E EQUIPAMENTOS CULTURAIS E TURÍSTICOS</t>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R7" t="n">
-        <v>4819</v>
+        <v>4611</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>TERRENOS</t>
         </is>
       </c>
       <c r="T7" t="n">
@@ -1045,18 +1045,18 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>GESTÃO DE PARTICIPAÇÕES, FUNDOS, CONSÓRCIOS, P&amp;D E EQUIPAMENTOS CULTURAIS E TURÍSTICOS</t>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>MINAS + GERAIS - DIVERSIFICAÇÃO E FORTALECIMENTO DA ECONOMIA</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B8" t="n">
         <v>1220</v>
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>9897</v>
+        <v>11022</v>
       </c>
       <c r="H8" t="n">
         <v>17</v>
@@ -1087,19 +1087,19 @@
         <v>512</v>
       </c>
       <c r="J8" t="n">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="K8" t="n">
         <v>8</v>
       </c>
       <c r="L8" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M8" t="n">
-        <v>8004</v>
+        <v>8008</v>
       </c>
       <c r="N8" t="n">
-        <v>80000000</v>
+        <v>250000000</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
@@ -1115,19 +1115,19 @@
         </is>
       </c>
       <c r="R8" t="n">
-        <v>4611</v>
+        <v>4613</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>TERRENOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T8" t="n">
-        <v>51000</v>
+        <v>21204</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OP CRÉD CONTRAT EXTERNA - KFW</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1137,13 +1137,13 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B9" t="n">
         <v>1220</v>
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>9897</v>
+        <v>11022</v>
       </c>
       <c r="H9" t="n">
         <v>17</v>
@@ -1174,19 +1174,19 @@
         <v>512</v>
       </c>
       <c r="J9" t="n">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="K9" t="n">
         <v>8</v>
       </c>
       <c r="L9" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M9" t="n">
-        <v>8004</v>
+        <v>8008</v>
       </c>
       <c r="N9" t="n">
-        <v>250000000</v>
+        <v>1062500000</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
@@ -1210,11 +1210,11 @@
         </is>
       </c>
       <c r="T9" t="n">
-        <v>21204</v>
+        <v>22199</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>OP CRÉD CONTRAT EXTERNA - KFW</t>
+          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1224,13 +1224,13 @@
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B10" t="n">
         <v>1220</v>
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>9897</v>
+        <v>11022</v>
       </c>
       <c r="H10" t="n">
         <v>17</v>
@@ -1261,19 +1261,19 @@
         <v>512</v>
       </c>
       <c r="J10" t="n">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="K10" t="n">
         <v>8</v>
       </c>
       <c r="L10" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M10" t="n">
-        <v>8004</v>
+        <v>8008</v>
       </c>
       <c r="N10" t="n">
-        <v>885250000</v>
+        <v>97500000</v>
       </c>
       <c r="O10" t="n">
         <v>0</v>
@@ -1297,11 +1297,11 @@
         </is>
       </c>
       <c r="T10" t="n">
-        <v>22199</v>
+        <v>51000</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1311,13 +1311,13 @@
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B11" t="n">
         <v>1220</v>
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>9897</v>
+        <v>11022</v>
       </c>
       <c r="H11" t="n">
         <v>17</v>
@@ -1348,19 +1348,19 @@
         <v>512</v>
       </c>
       <c r="J11" t="n">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="K11" t="n">
         <v>8</v>
       </c>
       <c r="L11" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M11" t="n">
-        <v>8004</v>
+        <v>8008</v>
       </c>
       <c r="N11" t="n">
-        <v>74750000</v>
+        <v>40000000</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
@@ -1376,19 +1376,19 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>4613</v>
+        <v>4614</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T11" t="n">
-        <v>51000</v>
+        <v>22199</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -1398,13 +1398,13 @@
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B12" t="n">
         <v>1220</v>
@@ -1426,7 +1426,7 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>9897</v>
+        <v>11023</v>
       </c>
       <c r="H12" t="n">
         <v>17</v>
@@ -1435,26 +1435,26 @@
         <v>512</v>
       </c>
       <c r="J12" t="n">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="K12" t="n">
         <v>8</v>
       </c>
       <c r="L12" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="M12" t="n">
-        <v>8004</v>
+        <v>8009</v>
       </c>
       <c r="N12" t="n">
-        <v>40000000</v>
+        <v>45752420</v>
       </c>
       <c r="O12" t="n">
         <v>0</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
+          <t>PPP SISTEMA ADUTOR RIO MANSO</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -1463,35 +1463,35 @@
         </is>
       </c>
       <c r="R12" t="n">
-        <v>4614</v>
+        <v>4613</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T12" t="n">
-        <v>22199</v>
+        <v>51000</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
+          <t>PPP SISTEMA ADUTOR RIO MANSO</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B13" t="n">
         <v>1220</v>
@@ -1505,56 +1505,56 @@
         <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>5081</v>
+        <v>5121</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
+          <t>COMPANHIA ENERGÉTICA DE MINAS GERAIS - CEMIG HOLDING</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>9898</v>
+        <v>10542</v>
       </c>
       <c r="H13" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I13" t="n">
-        <v>512</v>
+        <v>752</v>
       </c>
       <c r="J13" t="n">
-        <v>120</v>
+        <v>35</v>
       </c>
       <c r="K13" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L13" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="M13" t="n">
-        <v>8005</v>
+        <v>3010</v>
       </c>
       <c r="N13" t="n">
-        <v>49915500</v>
+        <v>344720630</v>
       </c>
       <c r="O13" t="n">
         <v>0</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>PPP - SISTEMA ADUTOR RIO MANSO</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>4613</v>
+        <v>4511</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T13" t="n">
@@ -1567,18 +1567,18 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>PPP - SISTEMA ADUTOR RIO MANSO</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>INVESTIMENTOS CEMIG</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B14" t="n">
         <v>1220</v>
@@ -1592,80 +1592,80 @@
         <v>3</v>
       </c>
       <c r="E14" t="n">
-        <v>5081</v>
+        <v>5121</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
+          <t>COMPANHIA ENERGÉTICA DE MINAS GERAIS - CEMIG HOLDING</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>9901</v>
+        <v>9994</v>
       </c>
       <c r="H14" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I14" t="n">
-        <v>512</v>
+        <v>752</v>
       </c>
       <c r="J14" t="n">
-        <v>120</v>
+        <v>35</v>
       </c>
       <c r="K14" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L14" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="M14" t="n">
-        <v>8008</v>
+        <v>3011</v>
       </c>
       <c r="N14" t="n">
-        <v>31000000</v>
+        <v>40000</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R14" t="n">
-        <v>4614</v>
+        <v>4817</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
         </is>
       </c>
       <c r="T14" t="n">
-        <v>22199</v>
+        <v>51000</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>INVESTIMENTOS CEMIG</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B15" t="n">
         <v>1220</v>
@@ -1679,43 +1679,43 @@
         <v>3</v>
       </c>
       <c r="E15" t="n">
-        <v>5081</v>
+        <v>5131</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
+          <t>AGÊNCIA DE PROMOÇÃO DE INVESTIMENTOS DE MINAS GERAIS - INVEST MINAS</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>9901</v>
+        <v>9723</v>
       </c>
       <c r="H15" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="I15" t="n">
-        <v>512</v>
+        <v>122</v>
       </c>
       <c r="J15" t="n">
-        <v>120</v>
+        <v>142</v>
       </c>
       <c r="K15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L15" t="n">
         <v>8</v>
       </c>
       <c r="M15" t="n">
-        <v>8008</v>
+        <v>6008</v>
       </c>
       <c r="N15" t="n">
-        <v>50000000</v>
+        <v>500000</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -1741,18 +1741,18 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL - INDI</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B16" t="n">
         <v>1220</v>
@@ -1766,56 +1766,56 @@
         <v>3</v>
       </c>
       <c r="E16" t="n">
-        <v>5121</v>
+        <v>5131</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>COMPANHIA ENERGÉTICA DE MINAS GERAIS - CEMIG HOLDING</t>
+          <t>AGÊNCIA DE PROMOÇÃO DE INVESTIMENTOS DE MINAS GERAIS - INVEST MINAS</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>9994</v>
+        <v>9723</v>
       </c>
       <c r="H16" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I16" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J16" t="n">
-        <v>35</v>
+        <v>142</v>
       </c>
       <c r="K16" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L16" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="M16" t="n">
-        <v>3011</v>
+        <v>6008</v>
       </c>
       <c r="N16" t="n">
-        <v>30608</v>
+        <v>0</v>
       </c>
       <c r="O16" t="n">
         <v>0</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R16" t="n">
-        <v>4614</v>
+        <v>4817</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
         </is>
       </c>
       <c r="T16" t="n">
@@ -1828,18 +1828,18 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS CEMIG</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL - INDI</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B17" t="n">
         <v>1220</v>
@@ -1853,80 +1853,80 @@
         <v>3</v>
       </c>
       <c r="E17" t="n">
-        <v>5121</v>
+        <v>5191</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>COMPANHIA ENERGÉTICA DE MINAS GERAIS - CEMIG HOLDING</t>
+          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>9995</v>
+        <v>9796</v>
       </c>
       <c r="H17" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I17" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J17" t="n">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="K17" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L17" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M17" t="n">
-        <v>3012</v>
+        <v>6011</v>
       </c>
       <c r="N17" t="n">
-        <v>629198369</v>
+        <v>670000</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL - PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R17" t="n">
-        <v>4512</v>
+        <v>4817</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>SOCIEDADES COLIGADAS</t>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
         </is>
       </c>
       <c r="T17" t="n">
-        <v>12100</v>
+        <v>51000</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>OUTRAS ENTIDADES - CEMIG</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL - PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS CEMIG</t>
+          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B18" t="n">
         <v>1220</v>
@@ -1940,80 +1940,80 @@
         <v>3</v>
       </c>
       <c r="E18" t="n">
-        <v>5131</v>
+        <v>5191</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>INSTITUTO DE DESENVOLVIMENTO INTEGRADO DE MINAS GERAIS - INDI</t>
+          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>9723</v>
+        <v>10513</v>
       </c>
       <c r="H18" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="I18" t="n">
         <v>122</v>
       </c>
       <c r="J18" t="n">
-        <v>142</v>
+        <v>24</v>
       </c>
       <c r="K18" t="n">
         <v>6</v>
       </c>
       <c r="L18" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="M18" t="n">
-        <v>6008</v>
+        <v>6002</v>
       </c>
       <c r="N18" t="n">
-        <v>500000</v>
+        <v>1000</v>
       </c>
       <c r="O18" t="n">
         <v>0</v>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DO INDI</t>
+          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R18" t="n">
-        <v>4614</v>
+        <v>4819</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T18" t="n">
-        <v>51000</v>
+        <v>11101</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DO INDI</t>
+          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL - INDI</t>
+          <t>DESENVOLVIMENTO SOCIOECONÔMICO</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B19" t="n">
         <v>1220</v>
@@ -2027,43 +2027,43 @@
         <v>3</v>
       </c>
       <c r="E19" t="n">
-        <v>5201</v>
+        <v>5191</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
+          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>9087</v>
+        <v>10513</v>
       </c>
       <c r="H19" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="I19" t="n">
         <v>122</v>
       </c>
       <c r="J19" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="K19" t="n">
         <v>6</v>
       </c>
       <c r="L19" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M19" t="n">
-        <v>6004</v>
+        <v>6002</v>
       </c>
       <c r="N19" t="n">
-        <v>21267000</v>
+        <v>186000</v>
       </c>
       <c r="O19" t="n">
         <v>0</v>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
+          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -2072,35 +2072,35 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>4813</v>
+        <v>4819</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>INTANGÍVEIS E OUTROS INVESTIMENTOS</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T19" t="n">
-        <v>12400</v>
+        <v>51000</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>OUTRAS ENTIDADES - BDMG</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
+          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>INVESTIMENTO NA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
+          <t>DESENVOLVIMENTO SOCIOECONÔMICO</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B20" t="n">
         <v>1220</v>
@@ -2114,80 +2114,80 @@
         <v>3</v>
       </c>
       <c r="E20" t="n">
-        <v>5251</v>
+        <v>5191</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>COMPANHIA DE GÁS DE MINAS GERAIS - GASMIG</t>
+          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>9629</v>
+        <v>9058</v>
       </c>
       <c r="H20" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I20" t="n">
-        <v>451</v>
+        <v>123</v>
       </c>
       <c r="J20" t="n">
-        <v>66</v>
+        <v>13</v>
       </c>
       <c r="K20" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>8003</v>
+        <v>6001</v>
       </c>
       <c r="N20" t="n">
-        <v>244358023</v>
+        <v>1000</v>
       </c>
       <c r="O20" t="n">
         <v>0</v>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
+          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R20" t="n">
-        <v>4613</v>
+        <v>4511</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T20" t="n">
-        <v>12900</v>
+        <v>51000</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>OUTRAS ENTIDADES - OUTRAS</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
+          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>#VEMPRAMINAS - ATRAÇÃO DE INVESTIMENTOS</t>
+          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B21" t="n">
         <v>1220</v>
@@ -2201,80 +2201,80 @@
         <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>5391</v>
+        <v>5201</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>9420</v>
+        <v>9087</v>
       </c>
       <c r="H21" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I21" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J21" t="n">
-        <v>92</v>
+        <v>17</v>
       </c>
       <c r="K21" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L21" t="n">
         <v>4</v>
       </c>
       <c r="M21" t="n">
-        <v>3004</v>
+        <v>6004</v>
       </c>
       <c r="N21" t="n">
-        <v>308709015</v>
+        <v>23908160</v>
       </c>
       <c r="O21" t="n">
         <v>0</v>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R21" t="n">
-        <v>4613</v>
+        <v>4813</v>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>INTANGÍVEIS E OUTROS INVESTIMENTOS</t>
         </is>
       </c>
       <c r="T21" t="n">
-        <v>51000</v>
+        <v>12400</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OUTRAS ENTIDADES - BDMG</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
+          <t>INVESTIMENTO NA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B22" t="n">
         <v>1220</v>
@@ -2288,80 +2288,80 @@
         <v>3</v>
       </c>
       <c r="E22" t="n">
-        <v>5391</v>
+        <v>5201</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>9421</v>
+        <v>10991</v>
       </c>
       <c r="H22" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I22" t="n">
-        <v>752</v>
+        <v>694</v>
       </c>
       <c r="J22" t="n">
-        <v>92</v>
+        <v>171</v>
       </c>
       <c r="K22" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M22" t="n">
-        <v>3005</v>
+        <v>8006</v>
       </c>
       <c r="N22" t="n">
-        <v>120452442</v>
+        <v>600000000</v>
       </c>
       <c r="O22" t="n">
         <v>0</v>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
+          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R22" t="n">
-        <v>4613</v>
+        <v>4819</v>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T22" t="n">
-        <v>51000</v>
+        <v>12400</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OUTRAS ENTIDADES - BDMG</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
+          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
+          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B23" t="n">
         <v>1220</v>
@@ -2375,43 +2375,43 @@
         <v>3</v>
       </c>
       <c r="E23" t="n">
-        <v>5391</v>
+        <v>5251</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>COMPANHIA DE GÁS DE MINAS GERAIS - GASMIG</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>9430</v>
+        <v>11027</v>
       </c>
       <c r="H23" t="n">
         <v>25</v>
       </c>
       <c r="I23" t="n">
-        <v>752</v>
+        <v>121</v>
       </c>
       <c r="J23" t="n">
-        <v>92</v>
+        <v>133</v>
       </c>
       <c r="K23" t="n">
         <v>3</v>
       </c>
       <c r="L23" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="M23" t="n">
-        <v>3006</v>
+        <v>3018</v>
       </c>
       <c r="N23" t="n">
-        <v>4693805</v>
+        <v>409881263</v>
       </c>
       <c r="O23" t="n">
         <v>0</v>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
+          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -2428,27 +2428,27 @@
         </is>
       </c>
       <c r="T23" t="n">
-        <v>51000</v>
+        <v>61000</v>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OUTRAS ORIGENS</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
+          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
+          <t>MINAS GERAÇÃO DE VALOR</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B24" t="n">
         <v>1220</v>
@@ -2462,43 +2462,43 @@
         <v>3</v>
       </c>
       <c r="E24" t="n">
-        <v>5391</v>
+        <v>5381</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>10062</v>
+        <v>9239</v>
       </c>
       <c r="H24" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J24" t="n">
-        <v>94</v>
+        <v>57</v>
       </c>
       <c r="K24" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M24" t="n">
-        <v>3001</v>
+        <v>8002</v>
       </c>
       <c r="N24" t="n">
-        <v>1880000000</v>
+        <v>4300000</v>
       </c>
       <c r="O24" t="n">
         <v>0</v>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -2507,11 +2507,11 @@
         </is>
       </c>
       <c r="R24" t="n">
-        <v>4613</v>
+        <v>4614</v>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T24" t="n">
@@ -2524,18 +2524,18 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B25" t="n">
         <v>1220</v>
@@ -2549,43 +2549,43 @@
         <v>3</v>
       </c>
       <c r="E25" t="n">
-        <v>5391</v>
+        <v>5381</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>9440</v>
+        <v>9239</v>
       </c>
       <c r="H25" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I25" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J25" t="n">
-        <v>94</v>
+        <v>57</v>
       </c>
       <c r="K25" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L25" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="M25" t="n">
-        <v>3007</v>
+        <v>8002</v>
       </c>
       <c r="N25" t="n">
-        <v>17888000</v>
+        <v>200000</v>
       </c>
       <c r="O25" t="n">
         <v>0</v>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -2594,11 +2594,11 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>4614</v>
+        <v>4615</v>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>MÓVEIS E UTENSÍLIOS</t>
         </is>
       </c>
       <c r="T25" t="n">
@@ -2611,18 +2611,18 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B26" t="n">
         <v>1220</v>
@@ -2636,56 +2636,56 @@
         <v>3</v>
       </c>
       <c r="E26" t="n">
-        <v>5391</v>
+        <v>5381</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>9450</v>
+        <v>9239</v>
       </c>
       <c r="H26" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I26" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J26" t="n">
-        <v>94</v>
+        <v>57</v>
       </c>
       <c r="K26" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L26" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="M26" t="n">
-        <v>3008</v>
+        <v>8002</v>
       </c>
       <c r="N26" t="n">
-        <v>15165514</v>
+        <v>4000000</v>
       </c>
       <c r="O26" t="n">
         <v>0</v>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R26" t="n">
-        <v>4614</v>
+        <v>4817</v>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
         </is>
       </c>
       <c r="T26" t="n">
@@ -2698,18 +2698,18 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B27" t="n">
         <v>1220</v>
@@ -2723,80 +2723,80 @@
         <v>3</v>
       </c>
       <c r="E27" t="n">
-        <v>5391</v>
+        <v>5381</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>10161</v>
+        <v>9239</v>
       </c>
       <c r="H27" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I27" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J27" t="n">
-        <v>94</v>
+        <v>57</v>
       </c>
       <c r="K27" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L27" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="M27" t="n">
-        <v>3009</v>
+        <v>8002</v>
       </c>
       <c r="N27" t="n">
-        <v>12241405</v>
+        <v>1000</v>
       </c>
       <c r="O27" t="n">
         <v>0</v>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL - PARTICIPAÇÕES SOCIETÁRIAS CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R27" t="n">
-        <v>4511</v>
+        <v>4819</v>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T27" t="n">
-        <v>12100</v>
+        <v>11101</v>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>OUTRAS ENTIDADES - CEMIG</t>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL - PARTICIPAÇÕES SOCIETÁRIAS CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B28" t="n">
         <v>1220</v>
@@ -2810,15 +2810,15 @@
         <v>3</v>
       </c>
       <c r="E28" t="n">
-        <v>5401</v>
+        <v>5391</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>9332</v>
+        <v>9420</v>
       </c>
       <c r="H28" t="n">
         <v>25</v>
@@ -2827,26 +2827,26 @@
         <v>752</v>
       </c>
       <c r="J28" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="K28" t="n">
         <v>3</v>
       </c>
       <c r="L28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M28" t="n">
-        <v>3002</v>
+        <v>3004</v>
       </c>
       <c r="N28" t="n">
-        <v>2901796000</v>
+        <v>198940203</v>
       </c>
       <c r="O28" t="n">
         <v>0</v>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
+          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -2872,18 +2872,18 @@
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
+          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B29" t="n">
         <v>1220</v>
@@ -2897,15 +2897,15 @@
         <v>3</v>
       </c>
       <c r="E29" t="n">
-        <v>5401</v>
+        <v>5391</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>9408</v>
+        <v>9421</v>
       </c>
       <c r="H29" t="n">
         <v>25</v>
@@ -2914,26 +2914,26 @@
         <v>752</v>
       </c>
       <c r="J29" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="K29" t="n">
         <v>3</v>
       </c>
       <c r="L29" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M29" t="n">
-        <v>3003</v>
+        <v>3005</v>
       </c>
       <c r="N29" t="n">
-        <v>162092993</v>
+        <v>241821909</v>
       </c>
       <c r="O29" t="n">
         <v>0</v>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
+          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -2942,11 +2942,11 @@
         </is>
       </c>
       <c r="R29" t="n">
-        <v>4614</v>
+        <v>4613</v>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T29" t="n">
@@ -2959,18 +2959,18 @@
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
+          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B30" t="n">
         <v>1220</v>
@@ -2984,43 +2984,43 @@
         <v>3</v>
       </c>
       <c r="E30" t="n">
-        <v>5511</v>
+        <v>5391</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>9899</v>
+        <v>9430</v>
       </c>
       <c r="H30" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I30" t="n">
-        <v>512</v>
+        <v>752</v>
       </c>
       <c r="J30" t="n">
-        <v>120</v>
+        <v>92</v>
       </c>
       <c r="K30" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L30" t="n">
         <v>6</v>
       </c>
       <c r="M30" t="n">
-        <v>8006</v>
+        <v>3006</v>
       </c>
       <c r="N30" t="n">
-        <v>45000000</v>
+        <v>30805275</v>
       </c>
       <c r="O30" t="n">
         <v>0</v>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPANOR</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -3029,11 +3029,11 @@
         </is>
       </c>
       <c r="R30" t="n">
-        <v>4613</v>
+        <v>4614</v>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T30" t="n">
@@ -3046,18 +3046,18 @@
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPANOR</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B31" t="n">
         <v>1220</v>
@@ -3071,43 +3071,43 @@
         <v>3</v>
       </c>
       <c r="E31" t="n">
-        <v>5511</v>
+        <v>5391</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>9900</v>
+        <v>10062</v>
       </c>
       <c r="H31" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I31" t="n">
-        <v>512</v>
+        <v>752</v>
       </c>
       <c r="J31" t="n">
-        <v>120</v>
+        <v>94</v>
       </c>
       <c r="K31" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L31" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>8007</v>
+        <v>3001</v>
       </c>
       <c r="N31" t="n">
-        <v>2000000</v>
+        <v>49096963</v>
       </c>
       <c r="O31" t="n">
         <v>0</v>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
+          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -3133,155 +3133,155 @@
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
+          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
         </is>
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B32" t="n">
-        <v>1300</v>
+        <v>1220</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA E MOBILIDADE - SEINFRA</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D32" t="n">
         <v>3</v>
       </c>
       <c r="E32" t="n">
-        <v>5261</v>
+        <v>5391</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>TREM METROPOLITANO DE BELO HORIZONTE S.A - TREM METROPOLITANO</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>9927</v>
+        <v>9440</v>
       </c>
       <c r="H32" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I32" t="n">
-        <v>783</v>
+        <v>752</v>
       </c>
       <c r="J32" t="n">
-        <v>705</v>
+        <v>94</v>
       </c>
       <c r="K32" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L32" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="M32" t="n">
-        <v>8011</v>
+        <v>3007</v>
       </c>
       <c r="N32" t="n">
-        <v>1000</v>
+        <v>130600000</v>
       </c>
       <c r="O32" t="n">
         <v>0</v>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R32" t="n">
-        <v>4511</v>
+        <v>4614</v>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T32" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
         </is>
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
+          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B33" t="n">
-        <v>1480</v>
+        <v>1220</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO SOCIAL - SEDESE</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D33" t="n">
         <v>3</v>
       </c>
       <c r="E33" t="n">
-        <v>5071</v>
+        <v>5391</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>COMPANHIA DE HABITAÇÃO DO ESTADO DE MINAS GERAIS - COHAB</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>9775</v>
+        <v>9450</v>
       </c>
       <c r="H33" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I33" t="n">
-        <v>122</v>
+        <v>752</v>
       </c>
       <c r="J33" t="n">
-        <v>705</v>
+        <v>94</v>
       </c>
       <c r="K33" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L33" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="M33" t="n">
-        <v>6010</v>
+        <v>3008</v>
       </c>
       <c r="N33" t="n">
-        <v>120000</v>
+        <v>13194360</v>
       </c>
       <c r="O33" t="n">
         <v>0</v>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA - COHAB</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -3307,81 +3307,81 @@
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA - COHAB</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
         </is>
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
+          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B34" t="n">
-        <v>1500</v>
+        <v>1220</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D34" t="n">
         <v>3</v>
       </c>
       <c r="E34" t="n">
-        <v>5141</v>
+        <v>5391</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>9116</v>
+        <v>10677</v>
       </c>
       <c r="H34" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="I34" t="n">
-        <v>126</v>
+        <v>752</v>
       </c>
       <c r="J34" t="n">
-        <v>30</v>
+        <v>94</v>
       </c>
       <c r="K34" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L34" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="M34" t="n">
-        <v>8001</v>
+        <v>3014</v>
       </c>
       <c r="N34" t="n">
-        <v>45914908</v>
+        <v>508846661</v>
       </c>
       <c r="O34" t="n">
         <v>0</v>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R34" t="n">
-        <v>4817</v>
+        <v>4511</v>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>EQUIPAMENTOS E SOFTWARE</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T34" t="n">
@@ -3394,68 +3394,68 @@
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B35" t="n">
-        <v>1500</v>
+        <v>1220</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D35" t="n">
         <v>3</v>
       </c>
       <c r="E35" t="n">
-        <v>5381</v>
+        <v>5401</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
+          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>9239</v>
+        <v>9332</v>
       </c>
       <c r="H35" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="I35" t="n">
-        <v>122</v>
+        <v>752</v>
       </c>
       <c r="J35" t="n">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="K35" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L35" t="n">
         <v>2</v>
       </c>
       <c r="M35" t="n">
-        <v>8002</v>
+        <v>3002</v>
       </c>
       <c r="N35" t="n">
-        <v>3300000</v>
+        <v>3487433034</v>
       </c>
       <c r="O35" t="n">
         <v>0</v>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -3464,11 +3464,11 @@
         </is>
       </c>
       <c r="R35" t="n">
-        <v>4614</v>
+        <v>4613</v>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T35" t="n">
@@ -3481,68 +3481,68 @@
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
         </is>
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
+          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B36" t="n">
-        <v>1500</v>
+        <v>1220</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D36" t="n">
         <v>3</v>
       </c>
       <c r="E36" t="n">
-        <v>5381</v>
+        <v>5401</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
+          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>9239</v>
+        <v>9408</v>
       </c>
       <c r="H36" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="I36" t="n">
-        <v>122</v>
+        <v>752</v>
       </c>
       <c r="J36" t="n">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="K36" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M36" t="n">
-        <v>8002</v>
+        <v>3003</v>
       </c>
       <c r="N36" t="n">
-        <v>200000</v>
+        <v>247223810</v>
       </c>
       <c r="O36" t="n">
         <v>0</v>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -3551,11 +3551,11 @@
         </is>
       </c>
       <c r="R36" t="n">
-        <v>4615</v>
+        <v>4614</v>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>MÓVEIS E UTENSÍLIOS</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T36" t="n">
@@ -3568,81 +3568,81 @@
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
+          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B37" t="n">
-        <v>1500</v>
+        <v>1220</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D37" t="n">
         <v>3</v>
       </c>
       <c r="E37" t="n">
-        <v>5381</v>
+        <v>5511</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
+          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>9239</v>
+        <v>11024</v>
       </c>
       <c r="H37" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I37" t="n">
-        <v>122</v>
+        <v>512</v>
       </c>
       <c r="J37" t="n">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="K37" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L37" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="M37" t="n">
-        <v>8002</v>
+        <v>6012</v>
       </c>
       <c r="N37" t="n">
-        <v>4500000</v>
+        <v>2000000</v>
       </c>
       <c r="O37" t="n">
         <v>0</v>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R37" t="n">
-        <v>4817</v>
+        <v>4614</v>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>EQUIPAMENTOS E SOFTWARE</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T37" t="n">
@@ -3655,99 +3655,360 @@
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
         </is>
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B38" t="n">
-        <v>1500</v>
+        <v>1220</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D38" t="n">
         <v>3</v>
       </c>
       <c r="E38" t="n">
-        <v>5381</v>
+        <v>5511</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
+          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>9239</v>
+        <v>11026</v>
       </c>
       <c r="H38" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I38" t="n">
-        <v>122</v>
+        <v>512</v>
       </c>
       <c r="J38" t="n">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="K38" t="n">
         <v>8</v>
       </c>
       <c r="L38" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="M38" t="n">
-        <v>8002</v>
+        <v>8012</v>
       </c>
       <c r="N38" t="n">
-        <v>1000</v>
+        <v>45000000</v>
       </c>
       <c r="O38" t="n">
         <v>0</v>
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
+          <t>4610 - IMOBILIZAÇÕES</t>
+        </is>
+      </c>
+      <c r="R38" t="n">
+        <v>4613</v>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>OBRAS E INSTALAÇÕES</t>
+        </is>
+      </c>
+      <c r="T38" t="n">
+        <v>51000</v>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>RECURSOS PRÓPRIOS</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B39" t="n">
+        <v>1300</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA, MOBILIDADE E PARCERIA - SEINFRA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>3</v>
+      </c>
+      <c r="E39" t="n">
+        <v>5261</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>TREM METROPOLITANO DE BELO HORIZONTE S.A - TREM METROPOLITANO</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>9927</v>
+      </c>
+      <c r="H39" t="n">
+        <v>26</v>
+      </c>
+      <c r="I39" t="n">
+        <v>783</v>
+      </c>
+      <c r="J39" t="n">
+        <v>705</v>
+      </c>
+      <c r="K39" t="n">
+        <v>8</v>
+      </c>
+      <c r="L39" t="n">
+        <v>11</v>
+      </c>
+      <c r="M39" t="n">
+        <v>8011</v>
+      </c>
+      <c r="N39" t="n">
+        <v>1000</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+        </is>
+      </c>
+      <c r="R39" t="n">
+        <v>4511</v>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>SOCIEDADES CONTROLADAS</t>
+        </is>
+      </c>
+      <c r="T39" t="n">
+        <v>11101</v>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B40" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" t="n">
+        <v>5141</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>10882</v>
+      </c>
+      <c r="H40" t="n">
+        <v>4</v>
+      </c>
+      <c r="I40" t="n">
+        <v>126</v>
+      </c>
+      <c r="J40" t="n">
+        <v>30</v>
+      </c>
+      <c r="K40" t="n">
+        <v>6</v>
+      </c>
+      <c r="L40" t="n">
+        <v>6</v>
+      </c>
+      <c r="M40" t="n">
+        <v>6006</v>
+      </c>
+      <c r="N40" t="n">
+        <v>3280000</v>
+      </c>
+      <c r="O40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>4610 - IMOBILIZAÇÕES</t>
+        </is>
+      </c>
+      <c r="R40" t="n">
+        <v>4613</v>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>OBRAS E INSTALAÇÕES</t>
+        </is>
+      </c>
+      <c r="T40" t="n">
+        <v>51000</v>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>RECURSOS PRÓPRIOS</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B41" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" t="n">
+        <v>5141</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>9116</v>
+      </c>
+      <c r="H41" t="n">
+        <v>4</v>
+      </c>
+      <c r="I41" t="n">
+        <v>126</v>
+      </c>
+      <c r="J41" t="n">
+        <v>30</v>
+      </c>
+      <c r="K41" t="n">
+        <v>8</v>
+      </c>
+      <c r="L41" t="n">
+        <v>1</v>
+      </c>
+      <c r="M41" t="n">
+        <v>8001</v>
+      </c>
+      <c r="N41" t="n">
+        <v>35386354</v>
+      </c>
+      <c r="O41" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
           <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
-      <c r="R38" t="n">
-        <v>4819</v>
-      </c>
-      <c r="S38" t="inlineStr">
-        <is>
-          <t>OUTRAS APLICAÇÕES</t>
-        </is>
-      </c>
-      <c r="T38" t="n">
-        <v>11101</v>
-      </c>
-      <c r="U38" t="inlineStr">
-        <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
-        </is>
-      </c>
-      <c r="V38" t="inlineStr">
-        <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
-        </is>
-      </c>
-      <c r="W38" t="inlineStr">
-        <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
+      <c r="R41" t="n">
+        <v>4817</v>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
+        </is>
+      </c>
+      <c r="T41" t="n">
+        <v>51000</v>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>RECURSOS PRÓPRIOS</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Migra repo para geracao ploa 2024 (#71)
* atualiza dados e config para ploa 2024

* atualiza CapaLoa na pasta de cada volume

* remove logs

* fix bugs
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_QDD_INVESTIMENTO.xlsx
+++ b/bancos/SISOR/BASE_QDD_INVESTIMENTO.xlsx
@@ -534,29 +534,29 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B2" t="n">
-        <v>1190</v>
+        <v>1220</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE FAZENDA - SEF</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>5191</v>
+        <v>5011</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
+          <t>COMPANHIA DE DESENVOLVIMENTO ECONÔMICO DE MINAS GERAIS - CODEMIG</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>9796</v>
+        <v>10929</v>
       </c>
       <c r="H2" t="n">
         <v>4</v>
@@ -565,39 +565,39 @@
         <v>122</v>
       </c>
       <c r="J2" t="n">
-        <v>13</v>
+        <v>133</v>
       </c>
       <c r="K2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L2" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="M2" t="n">
-        <v>6011</v>
+        <v>3017</v>
       </c>
       <c r="N2" t="n">
-        <v>90000</v>
+        <v>1000</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>MANUTENÇÃO E AQUISIÇÕES DA CODEMIG</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R2" t="n">
-        <v>4817</v>
+        <v>4614</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>EQUIPAMENTOS E SOFTWARE</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T2" t="n">
@@ -610,81 +610,81 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>MANUTENÇÃO E AQUISIÇÕES DA CODEMIG</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>MINAS GERAÇÃO DE VALOR</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B3" t="n">
-        <v>1190</v>
+        <v>1220</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE FAZENDA - SEF</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D3" t="n">
         <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>5191</v>
+        <v>5031</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
+          <t>COMPANHIA DE DESENVOLVIMENTO DE MINAS GERAIS - CODEMG</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>9082</v>
+        <v>10927</v>
       </c>
       <c r="H3" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="I3" t="n">
-        <v>122</v>
+        <v>572</v>
       </c>
       <c r="J3" t="n">
-        <v>24</v>
+        <v>133</v>
       </c>
       <c r="K3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L3" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="M3" t="n">
-        <v>6003</v>
+        <v>3015</v>
       </c>
       <c r="N3" t="n">
-        <v>15882556</v>
+        <v>12580000</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
+          <t>GESTÃO DE INFRAESTRUTURA, CONSÓRCIOS E EQUIPAMENTOS CULTURAIS E TURÍSTICOS</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R3" t="n">
-        <v>4819</v>
+        <v>4613</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T3" t="n">
@@ -697,192 +697,192 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
+          <t>GESTÃO DE INFRAESTRUTURA, CONSÓRCIOS E EQUIPAMENTOS CULTURAIS E TURÍSTICOS</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>APOIO AO DESENVOLVIMENTO MUNICIPAL, À CAPTAÇÃO E À COORDENAÇÃO DA TRANSFERÊNCIA DE RECURSOS</t>
+          <t>MINAS GERAÇÃO DE VALOR</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B4" t="n">
-        <v>1190</v>
+        <v>1220</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE FAZENDA - SEF</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D4" t="n">
         <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>5191</v>
+        <v>5071</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
+          <t>COMPANHIA DE HABITAÇÃO DO ESTADO DE MINAS GERAIS - COHAB</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>9058</v>
+        <v>9775</v>
       </c>
       <c r="H4" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="I4" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J4" t="n">
-        <v>13</v>
+        <v>705</v>
       </c>
       <c r="K4" t="n">
         <v>6</v>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="M4" t="n">
-        <v>6001</v>
+        <v>6010</v>
       </c>
       <c r="N4" t="n">
-        <v>1000</v>
+        <v>120000</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA - COHAB</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R4" t="n">
-        <v>4511</v>
+        <v>4614</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T4" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA - COHAB</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B5" t="n">
-        <v>1190</v>
+        <v>1220</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE FAZENDA - SEF</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D5" t="n">
         <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>5191</v>
+        <v>5081</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
+          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>9058</v>
+        <v>11021</v>
       </c>
       <c r="H5" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I5" t="n">
-        <v>123</v>
+        <v>512</v>
       </c>
       <c r="J5" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="K5" t="n">
         <v>6</v>
       </c>
       <c r="L5" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="M5" t="n">
-        <v>6001</v>
+        <v>6009</v>
       </c>
       <c r="N5" t="n">
-        <v>1000</v>
+        <v>50000000</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R5" t="n">
-        <v>4511</v>
+        <v>4614</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T5" t="n">
-        <v>51000</v>
+        <v>22199</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B6" t="n">
         <v>1220</v>
@@ -896,56 +896,56 @@
         <v>3</v>
       </c>
       <c r="E6" t="n">
-        <v>5011</v>
+        <v>5081</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>COMPANHIA DE DESENVOLVIMENTO ECONÔMICO DE MINAS GERAIS - CODEMIG</t>
+          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>10011</v>
+        <v>11021</v>
       </c>
       <c r="H6" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I6" t="n">
-        <v>122</v>
+        <v>512</v>
       </c>
       <c r="J6" t="n">
-        <v>63</v>
+        <v>21</v>
       </c>
       <c r="K6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L6" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="M6" t="n">
-        <v>3014</v>
+        <v>6009</v>
       </c>
       <c r="N6" t="n">
-        <v>1000</v>
+        <v>50000000</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E AQUISIÇÕES DA CODEMIG</t>
+          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R6" t="n">
-        <v>4819</v>
+        <v>4614</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T6" t="n">
@@ -958,18 +958,18 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E AQUISIÇÕES DA CODEMIG</t>
+          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>MINAS + GERAIS - DIVERSIFICAÇÃO E FORTALECIMENTO DA ECONOMIA</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B7" t="n">
         <v>1220</v>
@@ -983,56 +983,56 @@
         <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>5031</v>
+        <v>5081</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>COMPANHIA DE DESENVOLVIMENTO DE MINAS GERAIS - CODEMG</t>
+          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>9617</v>
+        <v>11022</v>
       </c>
       <c r="H7" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="I7" t="n">
-        <v>572</v>
+        <v>512</v>
       </c>
       <c r="J7" t="n">
-        <v>63</v>
+        <v>21</v>
       </c>
       <c r="K7" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L7" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="M7" t="n">
-        <v>3017</v>
+        <v>8008</v>
       </c>
       <c r="N7" t="n">
-        <v>14119841</v>
+        <v>100000000</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>GESTÃO DE PARTICIPAÇÕES, FUNDOS, CONSÓRCIOS, P&amp;D E EQUIPAMENTOS CULTURAIS E TURÍSTICOS</t>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R7" t="n">
-        <v>4819</v>
+        <v>4611</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>TERRENOS</t>
         </is>
       </c>
       <c r="T7" t="n">
@@ -1045,18 +1045,18 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>GESTÃO DE PARTICIPAÇÕES, FUNDOS, CONSÓRCIOS, P&amp;D E EQUIPAMENTOS CULTURAIS E TURÍSTICOS</t>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>MINAS + GERAIS - DIVERSIFICAÇÃO E FORTALECIMENTO DA ECONOMIA</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B8" t="n">
         <v>1220</v>
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>9897</v>
+        <v>11022</v>
       </c>
       <c r="H8" t="n">
         <v>17</v>
@@ -1087,19 +1087,19 @@
         <v>512</v>
       </c>
       <c r="J8" t="n">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="K8" t="n">
         <v>8</v>
       </c>
       <c r="L8" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M8" t="n">
-        <v>8004</v>
+        <v>8008</v>
       </c>
       <c r="N8" t="n">
-        <v>80000000</v>
+        <v>250000000</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
@@ -1115,19 +1115,19 @@
         </is>
       </c>
       <c r="R8" t="n">
-        <v>4611</v>
+        <v>4613</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>TERRENOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T8" t="n">
-        <v>51000</v>
+        <v>21204</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OP CRÉD CONTRAT EXTERNA - KFW</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1137,13 +1137,13 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B9" t="n">
         <v>1220</v>
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>9897</v>
+        <v>11022</v>
       </c>
       <c r="H9" t="n">
         <v>17</v>
@@ -1174,19 +1174,19 @@
         <v>512</v>
       </c>
       <c r="J9" t="n">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="K9" t="n">
         <v>8</v>
       </c>
       <c r="L9" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M9" t="n">
-        <v>8004</v>
+        <v>8008</v>
       </c>
       <c r="N9" t="n">
-        <v>250000000</v>
+        <v>1062500000</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
@@ -1210,11 +1210,11 @@
         </is>
       </c>
       <c r="T9" t="n">
-        <v>21204</v>
+        <v>22199</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>OP CRÉD CONTRAT EXTERNA - KFW</t>
+          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1224,13 +1224,13 @@
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B10" t="n">
         <v>1220</v>
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>9897</v>
+        <v>11022</v>
       </c>
       <c r="H10" t="n">
         <v>17</v>
@@ -1261,19 +1261,19 @@
         <v>512</v>
       </c>
       <c r="J10" t="n">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="K10" t="n">
         <v>8</v>
       </c>
       <c r="L10" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M10" t="n">
-        <v>8004</v>
+        <v>8008</v>
       </c>
       <c r="N10" t="n">
-        <v>885250000</v>
+        <v>97500000</v>
       </c>
       <c r="O10" t="n">
         <v>0</v>
@@ -1297,11 +1297,11 @@
         </is>
       </c>
       <c r="T10" t="n">
-        <v>22199</v>
+        <v>51000</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1311,13 +1311,13 @@
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B11" t="n">
         <v>1220</v>
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>9897</v>
+        <v>11022</v>
       </c>
       <c r="H11" t="n">
         <v>17</v>
@@ -1348,19 +1348,19 @@
         <v>512</v>
       </c>
       <c r="J11" t="n">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="K11" t="n">
         <v>8</v>
       </c>
       <c r="L11" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M11" t="n">
-        <v>8004</v>
+        <v>8008</v>
       </c>
       <c r="N11" t="n">
-        <v>74750000</v>
+        <v>40000000</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
@@ -1376,19 +1376,19 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>4613</v>
+        <v>4614</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T11" t="n">
-        <v>51000</v>
+        <v>22199</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -1398,13 +1398,13 @@
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B12" t="n">
         <v>1220</v>
@@ -1426,7 +1426,7 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>9897</v>
+        <v>11023</v>
       </c>
       <c r="H12" t="n">
         <v>17</v>
@@ -1435,26 +1435,26 @@
         <v>512</v>
       </c>
       <c r="J12" t="n">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="K12" t="n">
         <v>8</v>
       </c>
       <c r="L12" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="M12" t="n">
-        <v>8004</v>
+        <v>8009</v>
       </c>
       <c r="N12" t="n">
-        <v>40000000</v>
+        <v>45752420</v>
       </c>
       <c r="O12" t="n">
         <v>0</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
+          <t>PPP SISTEMA ADUTOR RIO MANSO</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -1463,35 +1463,35 @@
         </is>
       </c>
       <c r="R12" t="n">
-        <v>4614</v>
+        <v>4613</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T12" t="n">
-        <v>22199</v>
+        <v>51000</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
+          <t>PPP SISTEMA ADUTOR RIO MANSO</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B13" t="n">
         <v>1220</v>
@@ -1505,56 +1505,56 @@
         <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>5081</v>
+        <v>5121</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
+          <t>COMPANHIA ENERGÉTICA DE MINAS GERAIS - CEMIG HOLDING</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>9898</v>
+        <v>10542</v>
       </c>
       <c r="H13" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I13" t="n">
-        <v>512</v>
+        <v>752</v>
       </c>
       <c r="J13" t="n">
-        <v>120</v>
+        <v>35</v>
       </c>
       <c r="K13" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L13" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="M13" t="n">
-        <v>8005</v>
+        <v>3010</v>
       </c>
       <c r="N13" t="n">
-        <v>49915500</v>
+        <v>344720630</v>
       </c>
       <c r="O13" t="n">
         <v>0</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>PPP - SISTEMA ADUTOR RIO MANSO</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>4613</v>
+        <v>4511</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T13" t="n">
@@ -1567,18 +1567,18 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>PPP - SISTEMA ADUTOR RIO MANSO</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>INVESTIMENTOS CEMIG</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B14" t="n">
         <v>1220</v>
@@ -1592,80 +1592,80 @@
         <v>3</v>
       </c>
       <c r="E14" t="n">
-        <v>5081</v>
+        <v>5121</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
+          <t>COMPANHIA ENERGÉTICA DE MINAS GERAIS - CEMIG HOLDING</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>9901</v>
+        <v>9994</v>
       </c>
       <c r="H14" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I14" t="n">
-        <v>512</v>
+        <v>752</v>
       </c>
       <c r="J14" t="n">
-        <v>120</v>
+        <v>35</v>
       </c>
       <c r="K14" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L14" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="M14" t="n">
-        <v>8008</v>
+        <v>3011</v>
       </c>
       <c r="N14" t="n">
-        <v>31000000</v>
+        <v>40000</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R14" t="n">
-        <v>4614</v>
+        <v>4817</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
         </is>
       </c>
       <c r="T14" t="n">
-        <v>22199</v>
+        <v>51000</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>INVESTIMENTOS CEMIG</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B15" t="n">
         <v>1220</v>
@@ -1679,43 +1679,43 @@
         <v>3</v>
       </c>
       <c r="E15" t="n">
-        <v>5081</v>
+        <v>5131</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
+          <t>AGÊNCIA DE PROMOÇÃO DE INVESTIMENTOS DE MINAS GERAIS - INVEST MINAS</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>9901</v>
+        <v>9723</v>
       </c>
       <c r="H15" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="I15" t="n">
-        <v>512</v>
+        <v>122</v>
       </c>
       <c r="J15" t="n">
-        <v>120</v>
+        <v>142</v>
       </c>
       <c r="K15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L15" t="n">
         <v>8</v>
       </c>
       <c r="M15" t="n">
-        <v>8008</v>
+        <v>6008</v>
       </c>
       <c r="N15" t="n">
-        <v>50000000</v>
+        <v>500000</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -1741,18 +1741,18 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL - INDI</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B16" t="n">
         <v>1220</v>
@@ -1766,56 +1766,56 @@
         <v>3</v>
       </c>
       <c r="E16" t="n">
-        <v>5121</v>
+        <v>5131</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>COMPANHIA ENERGÉTICA DE MINAS GERAIS - CEMIG HOLDING</t>
+          <t>AGÊNCIA DE PROMOÇÃO DE INVESTIMENTOS DE MINAS GERAIS - INVEST MINAS</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>9994</v>
+        <v>9723</v>
       </c>
       <c r="H16" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I16" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J16" t="n">
-        <v>35</v>
+        <v>142</v>
       </c>
       <c r="K16" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L16" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="M16" t="n">
-        <v>3011</v>
+        <v>6008</v>
       </c>
       <c r="N16" t="n">
-        <v>30608</v>
+        <v>0</v>
       </c>
       <c r="O16" t="n">
         <v>0</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R16" t="n">
-        <v>4614</v>
+        <v>4817</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
         </is>
       </c>
       <c r="T16" t="n">
@@ -1828,18 +1828,18 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS CEMIG</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL - INDI</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B17" t="n">
         <v>1220</v>
@@ -1853,80 +1853,80 @@
         <v>3</v>
       </c>
       <c r="E17" t="n">
-        <v>5121</v>
+        <v>5191</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>COMPANHIA ENERGÉTICA DE MINAS GERAIS - CEMIG HOLDING</t>
+          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>9995</v>
+        <v>9796</v>
       </c>
       <c r="H17" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I17" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J17" t="n">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="K17" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L17" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M17" t="n">
-        <v>3012</v>
+        <v>6011</v>
       </c>
       <c r="N17" t="n">
-        <v>629198369</v>
+        <v>670000</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL - PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R17" t="n">
-        <v>4512</v>
+        <v>4817</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>SOCIEDADES COLIGADAS</t>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
         </is>
       </c>
       <c r="T17" t="n">
-        <v>12100</v>
+        <v>51000</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>OUTRAS ENTIDADES - CEMIG</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL - PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS CEMIG</t>
+          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B18" t="n">
         <v>1220</v>
@@ -1940,80 +1940,80 @@
         <v>3</v>
       </c>
       <c r="E18" t="n">
-        <v>5131</v>
+        <v>5191</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>INSTITUTO DE DESENVOLVIMENTO INTEGRADO DE MINAS GERAIS - INDI</t>
+          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>9723</v>
+        <v>10513</v>
       </c>
       <c r="H18" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="I18" t="n">
         <v>122</v>
       </c>
       <c r="J18" t="n">
-        <v>142</v>
+        <v>24</v>
       </c>
       <c r="K18" t="n">
         <v>6</v>
       </c>
       <c r="L18" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="M18" t="n">
-        <v>6008</v>
+        <v>6002</v>
       </c>
       <c r="N18" t="n">
-        <v>500000</v>
+        <v>1000</v>
       </c>
       <c r="O18" t="n">
         <v>0</v>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DO INDI</t>
+          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R18" t="n">
-        <v>4614</v>
+        <v>4819</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T18" t="n">
-        <v>51000</v>
+        <v>11101</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DO INDI</t>
+          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL - INDI</t>
+          <t>DESENVOLVIMENTO SOCIOECONÔMICO</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B19" t="n">
         <v>1220</v>
@@ -2027,43 +2027,43 @@
         <v>3</v>
       </c>
       <c r="E19" t="n">
-        <v>5201</v>
+        <v>5191</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
+          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>9087</v>
+        <v>10513</v>
       </c>
       <c r="H19" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="I19" t="n">
         <v>122</v>
       </c>
       <c r="J19" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="K19" t="n">
         <v>6</v>
       </c>
       <c r="L19" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M19" t="n">
-        <v>6004</v>
+        <v>6002</v>
       </c>
       <c r="N19" t="n">
-        <v>21267000</v>
+        <v>186000</v>
       </c>
       <c r="O19" t="n">
         <v>0</v>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
+          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -2072,35 +2072,35 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>4813</v>
+        <v>4819</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>INTANGÍVEIS E OUTROS INVESTIMENTOS</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T19" t="n">
-        <v>12400</v>
+        <v>51000</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>OUTRAS ENTIDADES - BDMG</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
+          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>INVESTIMENTO NA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
+          <t>DESENVOLVIMENTO SOCIOECONÔMICO</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B20" t="n">
         <v>1220</v>
@@ -2114,80 +2114,80 @@
         <v>3</v>
       </c>
       <c r="E20" t="n">
-        <v>5251</v>
+        <v>5191</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>COMPANHIA DE GÁS DE MINAS GERAIS - GASMIG</t>
+          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>9629</v>
+        <v>9058</v>
       </c>
       <c r="H20" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I20" t="n">
-        <v>451</v>
+        <v>123</v>
       </c>
       <c r="J20" t="n">
-        <v>66</v>
+        <v>13</v>
       </c>
       <c r="K20" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>8003</v>
+        <v>6001</v>
       </c>
       <c r="N20" t="n">
-        <v>244358023</v>
+        <v>1000</v>
       </c>
       <c r="O20" t="n">
         <v>0</v>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
+          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R20" t="n">
-        <v>4613</v>
+        <v>4511</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T20" t="n">
-        <v>12900</v>
+        <v>51000</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>OUTRAS ENTIDADES - OUTRAS</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
+          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>#VEMPRAMINAS - ATRAÇÃO DE INVESTIMENTOS</t>
+          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B21" t="n">
         <v>1220</v>
@@ -2201,80 +2201,80 @@
         <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>5391</v>
+        <v>5201</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>9420</v>
+        <v>9087</v>
       </c>
       <c r="H21" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I21" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J21" t="n">
-        <v>92</v>
+        <v>17</v>
       </c>
       <c r="K21" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L21" t="n">
         <v>4</v>
       </c>
       <c r="M21" t="n">
-        <v>3004</v>
+        <v>6004</v>
       </c>
       <c r="N21" t="n">
-        <v>308709015</v>
+        <v>23908160</v>
       </c>
       <c r="O21" t="n">
         <v>0</v>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R21" t="n">
-        <v>4613</v>
+        <v>4813</v>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>INTANGÍVEIS E OUTROS INVESTIMENTOS</t>
         </is>
       </c>
       <c r="T21" t="n">
-        <v>51000</v>
+        <v>12400</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OUTRAS ENTIDADES - BDMG</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
+          <t>INVESTIMENTO NA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B22" t="n">
         <v>1220</v>
@@ -2288,80 +2288,80 @@
         <v>3</v>
       </c>
       <c r="E22" t="n">
-        <v>5391</v>
+        <v>5201</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>9421</v>
+        <v>10991</v>
       </c>
       <c r="H22" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I22" t="n">
-        <v>752</v>
+        <v>694</v>
       </c>
       <c r="J22" t="n">
-        <v>92</v>
+        <v>171</v>
       </c>
       <c r="K22" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M22" t="n">
-        <v>3005</v>
+        <v>8006</v>
       </c>
       <c r="N22" t="n">
-        <v>120452442</v>
+        <v>600000000</v>
       </c>
       <c r="O22" t="n">
         <v>0</v>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
+          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R22" t="n">
-        <v>4613</v>
+        <v>4819</v>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T22" t="n">
-        <v>51000</v>
+        <v>12400</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OUTRAS ENTIDADES - BDMG</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
+          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
+          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B23" t="n">
         <v>1220</v>
@@ -2375,43 +2375,43 @@
         <v>3</v>
       </c>
       <c r="E23" t="n">
-        <v>5391</v>
+        <v>5251</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>COMPANHIA DE GÁS DE MINAS GERAIS - GASMIG</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>9430</v>
+        <v>11027</v>
       </c>
       <c r="H23" t="n">
         <v>25</v>
       </c>
       <c r="I23" t="n">
-        <v>752</v>
+        <v>121</v>
       </c>
       <c r="J23" t="n">
-        <v>92</v>
+        <v>133</v>
       </c>
       <c r="K23" t="n">
         <v>3</v>
       </c>
       <c r="L23" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="M23" t="n">
-        <v>3006</v>
+        <v>3018</v>
       </c>
       <c r="N23" t="n">
-        <v>4693805</v>
+        <v>409881263</v>
       </c>
       <c r="O23" t="n">
         <v>0</v>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
+          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -2428,27 +2428,27 @@
         </is>
       </c>
       <c r="T23" t="n">
-        <v>51000</v>
+        <v>61000</v>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OUTRAS ORIGENS</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
+          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
+          <t>MINAS GERAÇÃO DE VALOR</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B24" t="n">
         <v>1220</v>
@@ -2462,43 +2462,43 @@
         <v>3</v>
       </c>
       <c r="E24" t="n">
-        <v>5391</v>
+        <v>5381</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>10062</v>
+        <v>9239</v>
       </c>
       <c r="H24" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J24" t="n">
-        <v>94</v>
+        <v>57</v>
       </c>
       <c r="K24" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M24" t="n">
-        <v>3001</v>
+        <v>8002</v>
       </c>
       <c r="N24" t="n">
-        <v>1880000000</v>
+        <v>4300000</v>
       </c>
       <c r="O24" t="n">
         <v>0</v>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -2507,11 +2507,11 @@
         </is>
       </c>
       <c r="R24" t="n">
-        <v>4613</v>
+        <v>4614</v>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T24" t="n">
@@ -2524,18 +2524,18 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B25" t="n">
         <v>1220</v>
@@ -2549,43 +2549,43 @@
         <v>3</v>
       </c>
       <c r="E25" t="n">
-        <v>5391</v>
+        <v>5381</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>9440</v>
+        <v>9239</v>
       </c>
       <c r="H25" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I25" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J25" t="n">
-        <v>94</v>
+        <v>57</v>
       </c>
       <c r="K25" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L25" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="M25" t="n">
-        <v>3007</v>
+        <v>8002</v>
       </c>
       <c r="N25" t="n">
-        <v>17888000</v>
+        <v>200000</v>
       </c>
       <c r="O25" t="n">
         <v>0</v>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -2594,11 +2594,11 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>4614</v>
+        <v>4615</v>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>MÓVEIS E UTENSÍLIOS</t>
         </is>
       </c>
       <c r="T25" t="n">
@@ -2611,18 +2611,18 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B26" t="n">
         <v>1220</v>
@@ -2636,56 +2636,56 @@
         <v>3</v>
       </c>
       <c r="E26" t="n">
-        <v>5391</v>
+        <v>5381</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>9450</v>
+        <v>9239</v>
       </c>
       <c r="H26" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I26" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J26" t="n">
-        <v>94</v>
+        <v>57</v>
       </c>
       <c r="K26" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L26" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="M26" t="n">
-        <v>3008</v>
+        <v>8002</v>
       </c>
       <c r="N26" t="n">
-        <v>15165514</v>
+        <v>4000000</v>
       </c>
       <c r="O26" t="n">
         <v>0</v>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R26" t="n">
-        <v>4614</v>
+        <v>4817</v>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
         </is>
       </c>
       <c r="T26" t="n">
@@ -2698,18 +2698,18 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B27" t="n">
         <v>1220</v>
@@ -2723,80 +2723,80 @@
         <v>3</v>
       </c>
       <c r="E27" t="n">
-        <v>5391</v>
+        <v>5381</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>10161</v>
+        <v>9239</v>
       </c>
       <c r="H27" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I27" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J27" t="n">
-        <v>94</v>
+        <v>57</v>
       </c>
       <c r="K27" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L27" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="M27" t="n">
-        <v>3009</v>
+        <v>8002</v>
       </c>
       <c r="N27" t="n">
-        <v>12241405</v>
+        <v>1000</v>
       </c>
       <c r="O27" t="n">
         <v>0</v>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL - PARTICIPAÇÕES SOCIETÁRIAS CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R27" t="n">
-        <v>4511</v>
+        <v>4819</v>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T27" t="n">
-        <v>12100</v>
+        <v>11101</v>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>OUTRAS ENTIDADES - CEMIG</t>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL - PARTICIPAÇÕES SOCIETÁRIAS CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B28" t="n">
         <v>1220</v>
@@ -2810,15 +2810,15 @@
         <v>3</v>
       </c>
       <c r="E28" t="n">
-        <v>5401</v>
+        <v>5391</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>9332</v>
+        <v>9420</v>
       </c>
       <c r="H28" t="n">
         <v>25</v>
@@ -2827,26 +2827,26 @@
         <v>752</v>
       </c>
       <c r="J28" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="K28" t="n">
         <v>3</v>
       </c>
       <c r="L28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M28" t="n">
-        <v>3002</v>
+        <v>3004</v>
       </c>
       <c r="N28" t="n">
-        <v>2901796000</v>
+        <v>198940203</v>
       </c>
       <c r="O28" t="n">
         <v>0</v>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
+          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -2872,18 +2872,18 @@
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
+          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B29" t="n">
         <v>1220</v>
@@ -2897,15 +2897,15 @@
         <v>3</v>
       </c>
       <c r="E29" t="n">
-        <v>5401</v>
+        <v>5391</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>9408</v>
+        <v>9421</v>
       </c>
       <c r="H29" t="n">
         <v>25</v>
@@ -2914,26 +2914,26 @@
         <v>752</v>
       </c>
       <c r="J29" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="K29" t="n">
         <v>3</v>
       </c>
       <c r="L29" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M29" t="n">
-        <v>3003</v>
+        <v>3005</v>
       </c>
       <c r="N29" t="n">
-        <v>162092993</v>
+        <v>241821909</v>
       </c>
       <c r="O29" t="n">
         <v>0</v>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
+          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -2942,11 +2942,11 @@
         </is>
       </c>
       <c r="R29" t="n">
-        <v>4614</v>
+        <v>4613</v>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T29" t="n">
@@ -2959,18 +2959,18 @@
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
+          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B30" t="n">
         <v>1220</v>
@@ -2984,43 +2984,43 @@
         <v>3</v>
       </c>
       <c r="E30" t="n">
-        <v>5511</v>
+        <v>5391</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>9899</v>
+        <v>9430</v>
       </c>
       <c r="H30" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I30" t="n">
-        <v>512</v>
+        <v>752</v>
       </c>
       <c r="J30" t="n">
-        <v>120</v>
+        <v>92</v>
       </c>
       <c r="K30" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L30" t="n">
         <v>6</v>
       </c>
       <c r="M30" t="n">
-        <v>8006</v>
+        <v>3006</v>
       </c>
       <c r="N30" t="n">
-        <v>45000000</v>
+        <v>30805275</v>
       </c>
       <c r="O30" t="n">
         <v>0</v>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPANOR</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -3029,11 +3029,11 @@
         </is>
       </c>
       <c r="R30" t="n">
-        <v>4613</v>
+        <v>4614</v>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T30" t="n">
@@ -3046,18 +3046,18 @@
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPANOR</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B31" t="n">
         <v>1220</v>
@@ -3071,43 +3071,43 @@
         <v>3</v>
       </c>
       <c r="E31" t="n">
-        <v>5511</v>
+        <v>5391</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>9900</v>
+        <v>10062</v>
       </c>
       <c r="H31" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I31" t="n">
-        <v>512</v>
+        <v>752</v>
       </c>
       <c r="J31" t="n">
-        <v>120</v>
+        <v>94</v>
       </c>
       <c r="K31" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L31" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>8007</v>
+        <v>3001</v>
       </c>
       <c r="N31" t="n">
-        <v>2000000</v>
+        <v>49096963</v>
       </c>
       <c r="O31" t="n">
         <v>0</v>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
+          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -3133,155 +3133,155 @@
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
+          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
         </is>
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>GESTÃO AMBIENTAL E SANEAMENTO</t>
+          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B32" t="n">
-        <v>1300</v>
+        <v>1220</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA E MOBILIDADE - SEINFRA</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D32" t="n">
         <v>3</v>
       </c>
       <c r="E32" t="n">
-        <v>5261</v>
+        <v>5391</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>TREM METROPOLITANO DE BELO HORIZONTE S.A - TREM METROPOLITANO</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>9927</v>
+        <v>9440</v>
       </c>
       <c r="H32" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I32" t="n">
-        <v>783</v>
+        <v>752</v>
       </c>
       <c r="J32" t="n">
-        <v>705</v>
+        <v>94</v>
       </c>
       <c r="K32" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L32" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="M32" t="n">
-        <v>8011</v>
+        <v>3007</v>
       </c>
       <c r="N32" t="n">
-        <v>1000</v>
+        <v>130600000</v>
       </c>
       <c r="O32" t="n">
         <v>0</v>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R32" t="n">
-        <v>4511</v>
+        <v>4614</v>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T32" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
         </is>
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
+          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B33" t="n">
-        <v>1480</v>
+        <v>1220</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO SOCIAL - SEDESE</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D33" t="n">
         <v>3</v>
       </c>
       <c r="E33" t="n">
-        <v>5071</v>
+        <v>5391</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>COMPANHIA DE HABITAÇÃO DO ESTADO DE MINAS GERAIS - COHAB</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>9775</v>
+        <v>9450</v>
       </c>
       <c r="H33" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I33" t="n">
-        <v>122</v>
+        <v>752</v>
       </c>
       <c r="J33" t="n">
-        <v>705</v>
+        <v>94</v>
       </c>
       <c r="K33" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L33" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="M33" t="n">
-        <v>6010</v>
+        <v>3008</v>
       </c>
       <c r="N33" t="n">
-        <v>120000</v>
+        <v>13194360</v>
       </c>
       <c r="O33" t="n">
         <v>0</v>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA - COHAB</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -3307,81 +3307,81 @@
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA - COHAB</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
         </is>
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
+          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B34" t="n">
-        <v>1500</v>
+        <v>1220</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D34" t="n">
         <v>3</v>
       </c>
       <c r="E34" t="n">
-        <v>5141</v>
+        <v>5391</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>9116</v>
+        <v>10677</v>
       </c>
       <c r="H34" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="I34" t="n">
-        <v>126</v>
+        <v>752</v>
       </c>
       <c r="J34" t="n">
-        <v>30</v>
+        <v>94</v>
       </c>
       <c r="K34" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L34" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="M34" t="n">
-        <v>8001</v>
+        <v>3014</v>
       </c>
       <c r="N34" t="n">
-        <v>45914908</v>
+        <v>508846661</v>
       </c>
       <c r="O34" t="n">
         <v>0</v>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R34" t="n">
-        <v>4817</v>
+        <v>4511</v>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>EQUIPAMENTOS E SOFTWARE</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T34" t="n">
@@ -3394,68 +3394,68 @@
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B35" t="n">
-        <v>1500</v>
+        <v>1220</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D35" t="n">
         <v>3</v>
       </c>
       <c r="E35" t="n">
-        <v>5381</v>
+        <v>5401</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
+          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>9239</v>
+        <v>9332</v>
       </c>
       <c r="H35" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="I35" t="n">
-        <v>122</v>
+        <v>752</v>
       </c>
       <c r="J35" t="n">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="K35" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L35" t="n">
         <v>2</v>
       </c>
       <c r="M35" t="n">
-        <v>8002</v>
+        <v>3002</v>
       </c>
       <c r="N35" t="n">
-        <v>3300000</v>
+        <v>3487433034</v>
       </c>
       <c r="O35" t="n">
         <v>0</v>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -3464,11 +3464,11 @@
         </is>
       </c>
       <c r="R35" t="n">
-        <v>4614</v>
+        <v>4613</v>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T35" t="n">
@@ -3481,68 +3481,68 @@
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
         </is>
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
+          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B36" t="n">
-        <v>1500</v>
+        <v>1220</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D36" t="n">
         <v>3</v>
       </c>
       <c r="E36" t="n">
-        <v>5381</v>
+        <v>5401</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
+          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>9239</v>
+        <v>9408</v>
       </c>
       <c r="H36" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="I36" t="n">
-        <v>122</v>
+        <v>752</v>
       </c>
       <c r="J36" t="n">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="K36" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M36" t="n">
-        <v>8002</v>
+        <v>3003</v>
       </c>
       <c r="N36" t="n">
-        <v>200000</v>
+        <v>247223810</v>
       </c>
       <c r="O36" t="n">
         <v>0</v>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -3551,11 +3551,11 @@
         </is>
       </c>
       <c r="R36" t="n">
-        <v>4615</v>
+        <v>4614</v>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>MÓVEIS E UTENSÍLIOS</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T36" t="n">
@@ -3568,81 +3568,81 @@
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
+          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B37" t="n">
-        <v>1500</v>
+        <v>1220</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D37" t="n">
         <v>3</v>
       </c>
       <c r="E37" t="n">
-        <v>5381</v>
+        <v>5511</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
+          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>9239</v>
+        <v>11024</v>
       </c>
       <c r="H37" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I37" t="n">
-        <v>122</v>
+        <v>512</v>
       </c>
       <c r="J37" t="n">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="K37" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L37" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="M37" t="n">
-        <v>8002</v>
+        <v>6012</v>
       </c>
       <c r="N37" t="n">
-        <v>4500000</v>
+        <v>2000000</v>
       </c>
       <c r="O37" t="n">
         <v>0</v>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R37" t="n">
-        <v>4817</v>
+        <v>4614</v>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>EQUIPAMENTOS E SOFTWARE</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T37" t="n">
@@ -3655,99 +3655,360 @@
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
         </is>
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B38" t="n">
-        <v>1500</v>
+        <v>1220</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D38" t="n">
         <v>3</v>
       </c>
       <c r="E38" t="n">
-        <v>5381</v>
+        <v>5511</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
+          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>9239</v>
+        <v>11026</v>
       </c>
       <c r="H38" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I38" t="n">
-        <v>122</v>
+        <v>512</v>
       </c>
       <c r="J38" t="n">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="K38" t="n">
         <v>8</v>
       </c>
       <c r="L38" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="M38" t="n">
-        <v>8002</v>
+        <v>8012</v>
       </c>
       <c r="N38" t="n">
-        <v>1000</v>
+        <v>45000000</v>
       </c>
       <c r="O38" t="n">
         <v>0</v>
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
+          <t>4610 - IMOBILIZAÇÕES</t>
+        </is>
+      </c>
+      <c r="R38" t="n">
+        <v>4613</v>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>OBRAS E INSTALAÇÕES</t>
+        </is>
+      </c>
+      <c r="T38" t="n">
+        <v>51000</v>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>RECURSOS PRÓPRIOS</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B39" t="n">
+        <v>1300</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA, MOBILIDADE E PARCERIA - SEINFRA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>3</v>
+      </c>
+      <c r="E39" t="n">
+        <v>5261</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>TREM METROPOLITANO DE BELO HORIZONTE S.A - TREM METROPOLITANO</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>9927</v>
+      </c>
+      <c r="H39" t="n">
+        <v>26</v>
+      </c>
+      <c r="I39" t="n">
+        <v>783</v>
+      </c>
+      <c r="J39" t="n">
+        <v>705</v>
+      </c>
+      <c r="K39" t="n">
+        <v>8</v>
+      </c>
+      <c r="L39" t="n">
+        <v>11</v>
+      </c>
+      <c r="M39" t="n">
+        <v>8011</v>
+      </c>
+      <c r="N39" t="n">
+        <v>1000</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+        </is>
+      </c>
+      <c r="R39" t="n">
+        <v>4511</v>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>SOCIEDADES CONTROLADAS</t>
+        </is>
+      </c>
+      <c r="T39" t="n">
+        <v>11101</v>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B40" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" t="n">
+        <v>5141</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>10882</v>
+      </c>
+      <c r="H40" t="n">
+        <v>4</v>
+      </c>
+      <c r="I40" t="n">
+        <v>126</v>
+      </c>
+      <c r="J40" t="n">
+        <v>30</v>
+      </c>
+      <c r="K40" t="n">
+        <v>6</v>
+      </c>
+      <c r="L40" t="n">
+        <v>6</v>
+      </c>
+      <c r="M40" t="n">
+        <v>6006</v>
+      </c>
+      <c r="N40" t="n">
+        <v>3280000</v>
+      </c>
+      <c r="O40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>4610 - IMOBILIZAÇÕES</t>
+        </is>
+      </c>
+      <c r="R40" t="n">
+        <v>4613</v>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>OBRAS E INSTALAÇÕES</t>
+        </is>
+      </c>
+      <c r="T40" t="n">
+        <v>51000</v>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>RECURSOS PRÓPRIOS</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B41" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" t="n">
+        <v>5141</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>9116</v>
+      </c>
+      <c r="H41" t="n">
+        <v>4</v>
+      </c>
+      <c r="I41" t="n">
+        <v>126</v>
+      </c>
+      <c r="J41" t="n">
+        <v>30</v>
+      </c>
+      <c r="K41" t="n">
+        <v>8</v>
+      </c>
+      <c r="L41" t="n">
+        <v>1</v>
+      </c>
+      <c r="M41" t="n">
+        <v>8001</v>
+      </c>
+      <c r="N41" t="n">
+        <v>35386354</v>
+      </c>
+      <c r="O41" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
           <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
-      <c r="R38" t="n">
-        <v>4819</v>
-      </c>
-      <c r="S38" t="inlineStr">
-        <is>
-          <t>OUTRAS APLICAÇÕES</t>
-        </is>
-      </c>
-      <c r="T38" t="n">
-        <v>11101</v>
-      </c>
-      <c r="U38" t="inlineStr">
-        <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
-        </is>
-      </c>
-      <c r="V38" t="inlineStr">
-        <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
-        </is>
-      </c>
-      <c r="W38" t="inlineStr">
-        <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
+      <c r="R41" t="n">
+        <v>4817</v>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
+        </is>
+      </c>
+      <c r="T41" t="n">
+        <v>51000</v>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>RECURSOS PRÓPRIOS</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
atualiza dados com bases producao 2025
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_QDD_INVESTIMENTO.xlsx
+++ b/bancos/SISOR/BASE_QDD_INVESTIMENTO.xlsx
@@ -534,7 +534,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B2" t="n">
         <v>1220</v>
@@ -621,7 +621,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B3" t="n">
         <v>1220</v>
@@ -639,7 +639,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>COMPANHIA DE DESENVOLVIMENTO DE MINAS GERAIS - CODEMG</t>
+          <t>COMPANHIA DE DESENVOLVIMENTO DE MINAS GERAIS - CODEMGE</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -664,7 +664,7 @@
         <v>3015</v>
       </c>
       <c r="N3" t="n">
-        <v>12580000</v>
+        <v>6380000</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -708,7 +708,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B4" t="n">
         <v>1220</v>
@@ -722,43 +722,43 @@
         <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>5071</v>
+        <v>5031</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>COMPANHIA DE HABITAÇÃO DO ESTADO DE MINAS GERAIS - COHAB</t>
+          <t>COMPANHIA DE DESENVOLVIMENTO DE MINAS GERAIS - CODEMGE</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>9775</v>
+        <v>10927</v>
       </c>
       <c r="H4" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="I4" t="n">
-        <v>122</v>
+        <v>572</v>
       </c>
       <c r="J4" t="n">
-        <v>705</v>
+        <v>133</v>
       </c>
       <c r="K4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L4" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="M4" t="n">
-        <v>6010</v>
+        <v>3015</v>
       </c>
       <c r="N4" t="n">
-        <v>120000</v>
+        <v>6240000</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA - COHAB</t>
+          <t>GESTÃO DE INFRAESTRUTURA, CONSÓRCIOS E EQUIPAMENTOS CULTURAIS E TURÍSTICOS</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -784,18 +784,18 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA - COHAB</t>
+          <t>GESTÃO DE INFRAESTRUTURA, CONSÓRCIOS E EQUIPAMENTOS CULTURAIS E TURÍSTICOS</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
+          <t>MINAS GERAÇÃO DE VALOR</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B5" t="n">
         <v>1220</v>
@@ -809,43 +809,43 @@
         <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>5081</v>
+        <v>5071</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
+          <t>COMPANHIA DE HABITAÇÃO DO ESTADO DE MINAS GERAIS - COHAB</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>11021</v>
+        <v>9775</v>
       </c>
       <c r="H5" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I5" t="n">
-        <v>512</v>
+        <v>122</v>
       </c>
       <c r="J5" t="n">
-        <v>21</v>
+        <v>705</v>
       </c>
       <c r="K5" t="n">
         <v>6</v>
       </c>
       <c r="L5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M5" t="n">
-        <v>6009</v>
+        <v>6010</v>
       </c>
       <c r="N5" t="n">
-        <v>50000000</v>
+        <v>120000</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA - COHAB</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -862,27 +862,27 @@
         </is>
       </c>
       <c r="T5" t="n">
-        <v>22199</v>
+        <v>51000</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA - COHAB</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
+          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B6" t="n">
         <v>1220</v>
@@ -949,11 +949,11 @@
         </is>
       </c>
       <c r="T6" t="n">
-        <v>51000</v>
+        <v>22199</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -969,7 +969,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B7" t="n">
         <v>1220</v>
@@ -991,7 +991,7 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>11022</v>
+        <v>11021</v>
       </c>
       <c r="H7" t="n">
         <v>17</v>
@@ -1003,23 +1003,23 @@
         <v>21</v>
       </c>
       <c r="K7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M7" t="n">
-        <v>8008</v>
+        <v>6009</v>
       </c>
       <c r="N7" t="n">
-        <v>100000000</v>
+        <v>50000000</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
+          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1028,11 +1028,11 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>4611</v>
+        <v>4614</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>TERRENOS</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T7" t="n">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
+          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
@@ -1056,7 +1056,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B8" t="n">
         <v>1220</v>
@@ -1099,7 +1099,7 @@
         <v>8008</v>
       </c>
       <c r="N8" t="n">
-        <v>250000000</v>
+        <v>100000000</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
@@ -1115,19 +1115,19 @@
         </is>
       </c>
       <c r="R8" t="n">
-        <v>4613</v>
+        <v>4611</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>TERRENOS</t>
         </is>
       </c>
       <c r="T8" t="n">
-        <v>21204</v>
+        <v>51000</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>OP CRÉD CONTRAT EXTERNA - KFW</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1143,7 +1143,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B9" t="n">
         <v>1220</v>
@@ -1186,7 +1186,7 @@
         <v>8008</v>
       </c>
       <c r="N9" t="n">
-        <v>1062500000</v>
+        <v>350000000</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
@@ -1210,11 +1210,11 @@
         </is>
       </c>
       <c r="T9" t="n">
-        <v>22199</v>
+        <v>21204</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
+          <t>OP CRÉD CONTRAT EXTERNA - KFW</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1230,7 +1230,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B10" t="n">
         <v>1220</v>
@@ -1273,7 +1273,7 @@
         <v>8008</v>
       </c>
       <c r="N10" t="n">
-        <v>97500000</v>
+        <v>983250000</v>
       </c>
       <c r="O10" t="n">
         <v>0</v>
@@ -1297,11 +1297,11 @@
         </is>
       </c>
       <c r="T10" t="n">
-        <v>51000</v>
+        <v>22199</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1317,7 +1317,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B11" t="n">
         <v>1220</v>
@@ -1360,7 +1360,7 @@
         <v>8008</v>
       </c>
       <c r="N11" t="n">
-        <v>40000000</v>
+        <v>54750000</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
@@ -1376,19 +1376,19 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>4614</v>
+        <v>4613</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T11" t="n">
-        <v>22199</v>
+        <v>51000</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -1404,7 +1404,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B12" t="n">
         <v>1220</v>
@@ -1426,7 +1426,7 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>11023</v>
+        <v>11022</v>
       </c>
       <c r="H12" t="n">
         <v>17</v>
@@ -1441,20 +1441,20 @@
         <v>8</v>
       </c>
       <c r="L12" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M12" t="n">
-        <v>8009</v>
+        <v>8008</v>
       </c>
       <c r="N12" t="n">
-        <v>45752420</v>
+        <v>40000000</v>
       </c>
       <c r="O12" t="n">
         <v>0</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>PPP SISTEMA ADUTOR RIO MANSO</t>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -1463,24 +1463,24 @@
         </is>
       </c>
       <c r="R12" t="n">
-        <v>4613</v>
+        <v>4614</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T12" t="n">
-        <v>51000</v>
+        <v>22199</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>PPP SISTEMA ADUTOR RIO MANSO</t>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
@@ -1491,7 +1491,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B13" t="n">
         <v>1220</v>
@@ -1505,56 +1505,56 @@
         <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>5121</v>
+        <v>5081</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>COMPANHIA ENERGÉTICA DE MINAS GERAIS - CEMIG HOLDING</t>
+          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>10542</v>
+        <v>11023</v>
       </c>
       <c r="H13" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="I13" t="n">
-        <v>752</v>
+        <v>512</v>
       </c>
       <c r="J13" t="n">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="K13" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L13" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="M13" t="n">
-        <v>3010</v>
+        <v>8009</v>
       </c>
       <c r="N13" t="n">
-        <v>344720630</v>
+        <v>48428689</v>
       </c>
       <c r="O13" t="n">
         <v>0</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
+          <t>PPP SISTEMA ADUTOR RIO MANSO</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>4511</v>
+        <v>4613</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T13" t="n">
@@ -1567,18 +1567,18 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
+          <t>PPP SISTEMA ADUTOR RIO MANSO</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS CEMIG</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B14" t="n">
         <v>1220</v>
@@ -1600,7 +1600,7 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>9994</v>
+        <v>10542</v>
       </c>
       <c r="H14" t="n">
         <v>25</v>
@@ -1615,33 +1615,33 @@
         <v>3</v>
       </c>
       <c r="L14" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="M14" t="n">
-        <v>3011</v>
+        <v>3010</v>
       </c>
       <c r="N14" t="n">
-        <v>40000</v>
+        <v>259985809</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R14" t="n">
-        <v>4817</v>
+        <v>4511</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>EQUIPAMENTOS E SOFTWARE</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T14" t="n">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
@@ -1665,7 +1665,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B15" t="n">
         <v>1220</v>
@@ -1679,43 +1679,43 @@
         <v>3</v>
       </c>
       <c r="E15" t="n">
-        <v>5131</v>
+        <v>5121</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>AGÊNCIA DE PROMOÇÃO DE INVESTIMENTOS DE MINAS GERAIS - INVEST MINAS</t>
+          <t>COMPANHIA ENERGÉTICA DE MINAS GERAIS - CEMIG HOLDING</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>9723</v>
+        <v>9994</v>
       </c>
       <c r="H15" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I15" t="n">
-        <v>122</v>
+        <v>752</v>
       </c>
       <c r="J15" t="n">
-        <v>142</v>
+        <v>35</v>
       </c>
       <c r="K15" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L15" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="M15" t="n">
-        <v>6008</v>
+        <v>3011</v>
       </c>
       <c r="N15" t="n">
-        <v>500000</v>
+        <v>4440000</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -1741,18 +1741,18 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL - INVEST MINAS</t>
+          <t>INVESTIMENTOS CEMIG</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B16" t="n">
         <v>1220</v>
@@ -1766,56 +1766,56 @@
         <v>3</v>
       </c>
       <c r="E16" t="n">
-        <v>5191</v>
+        <v>5131</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
+          <t>AGÊNCIA DE PROMOÇÃO DE INVESTIMENTOS DE MINAS GERAIS - INVEST MINAS</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>9796</v>
+        <v>9723</v>
       </c>
       <c r="H16" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="I16" t="n">
         <v>122</v>
       </c>
       <c r="J16" t="n">
-        <v>13</v>
+        <v>142</v>
       </c>
       <c r="K16" t="n">
         <v>6</v>
       </c>
       <c r="L16" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="M16" t="n">
-        <v>6011</v>
+        <v>6008</v>
       </c>
       <c r="N16" t="n">
-        <v>670000</v>
+        <v>500000</v>
       </c>
       <c r="O16" t="n">
         <v>0</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R16" t="n">
-        <v>4817</v>
+        <v>4614</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>EQUIPAMENTOS E SOFTWARE</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T16" t="n">
@@ -1828,18 +1828,18 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL - INVEST MINAS</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B17" t="n">
         <v>1220</v>
@@ -1861,7 +1861,7 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>10513</v>
+        <v>9796</v>
       </c>
       <c r="H17" t="n">
         <v>4</v>
@@ -1870,26 +1870,26 @@
         <v>122</v>
       </c>
       <c r="J17" t="n">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="K17" t="n">
         <v>6</v>
       </c>
       <c r="L17" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="M17" t="n">
-        <v>6002</v>
+        <v>6011</v>
       </c>
       <c r="N17" t="n">
-        <v>1000</v>
+        <v>243000</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -1898,35 +1898,35 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>4819</v>
+        <v>4817</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
         </is>
       </c>
       <c r="T17" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>DESENVOLVIMENTO SOCIOECONÔMICO</t>
+          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B18" t="n">
         <v>1220</v>
@@ -1948,7 +1948,7 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>10513</v>
+        <v>11036</v>
       </c>
       <c r="H18" t="n">
         <v>4</v>
@@ -1957,19 +1957,19 @@
         <v>122</v>
       </c>
       <c r="J18" t="n">
-        <v>24</v>
+        <v>119</v>
       </c>
       <c r="K18" t="n">
         <v>6</v>
       </c>
       <c r="L18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M18" t="n">
-        <v>6002</v>
+        <v>6003</v>
       </c>
       <c r="N18" t="n">
-        <v>186000</v>
+        <v>1000</v>
       </c>
       <c r="O18" t="n">
         <v>0</v>
@@ -1993,11 +1993,11 @@
         </is>
       </c>
       <c r="T18" t="n">
-        <v>51000</v>
+        <v>11101</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
@@ -2007,13 +2007,13 @@
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>DESENVOLVIMENTO SOCIOECONÔMICO</t>
+          <t>APOIO AO DESENVOLVIMENTO MUNICIPAL E À COORDENAÇÃO DAS TRANSFERÊNCIAS ESTADUAIS DE RECURSOS FINANCEIROS</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B19" t="n">
         <v>1220</v>
@@ -2035,48 +2035,48 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>9058</v>
+        <v>11036</v>
       </c>
       <c r="H19" t="n">
         <v>4</v>
       </c>
       <c r="I19" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J19" t="n">
-        <v>13</v>
+        <v>119</v>
       </c>
       <c r="K19" t="n">
         <v>6</v>
       </c>
       <c r="L19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M19" t="n">
-        <v>6001</v>
+        <v>6003</v>
       </c>
       <c r="N19" t="n">
-        <v>1000</v>
+        <v>9256395</v>
       </c>
       <c r="O19" t="n">
         <v>0</v>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R19" t="n">
-        <v>4511</v>
+        <v>4819</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T19" t="n">
@@ -2089,18 +2089,18 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>APOIO AO DESENVOLVIMENTO MUNICIPAL E À COORDENAÇÃO DAS TRANSFERÊNCIAS ESTADUAIS DE RECURSOS FINANCEIROS</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B20" t="n">
         <v>1220</v>
@@ -2114,80 +2114,80 @@
         <v>3</v>
       </c>
       <c r="E20" t="n">
-        <v>5201</v>
+        <v>5191</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
+          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>9087</v>
+        <v>9058</v>
       </c>
       <c r="H20" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="I20" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J20" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="K20" t="n">
         <v>6</v>
       </c>
       <c r="L20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>6004</v>
+        <v>6001</v>
       </c>
       <c r="N20" t="n">
-        <v>23908160</v>
+        <v>1000</v>
       </c>
       <c r="O20" t="n">
         <v>0</v>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
+          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R20" t="n">
-        <v>4813</v>
+        <v>4511</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>INTANGÍVEIS E OUTROS INVESTIMENTOS</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T20" t="n">
-        <v>12400</v>
+        <v>11101</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>OUTRAS ENTIDADES - BDMG</t>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
+          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>INVESTIMENTO NA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
+          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B21" t="n">
         <v>1220</v>
@@ -2201,80 +2201,80 @@
         <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>5201</v>
+        <v>5191</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
+          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>10991</v>
+        <v>9058</v>
       </c>
       <c r="H21" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="I21" t="n">
-        <v>694</v>
+        <v>123</v>
       </c>
       <c r="J21" t="n">
-        <v>171</v>
+        <v>13</v>
       </c>
       <c r="K21" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L21" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>8006</v>
+        <v>6001</v>
       </c>
       <c r="N21" t="n">
-        <v>600000000</v>
+        <v>1000</v>
       </c>
       <c r="O21" t="n">
         <v>0</v>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
+          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R21" t="n">
-        <v>4819</v>
+        <v>4511</v>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T21" t="n">
-        <v>12400</v>
+        <v>51000</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>OUTRAS ENTIDADES - BDMG</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
+          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
+          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B22" t="n">
         <v>1220</v>
@@ -2288,80 +2288,80 @@
         <v>3</v>
       </c>
       <c r="E22" t="n">
-        <v>5251</v>
+        <v>5201</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>COMPANHIA DE GÁS DE MINAS GERAIS - GASMIG</t>
+          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>11027</v>
+        <v>9087</v>
       </c>
       <c r="H22" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I22" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J22" t="n">
-        <v>133</v>
+        <v>17</v>
       </c>
       <c r="K22" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L22" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="M22" t="n">
-        <v>3018</v>
+        <v>6004</v>
       </c>
       <c r="N22" t="n">
-        <v>409881263</v>
+        <v>26253389</v>
       </c>
       <c r="O22" t="n">
         <v>0</v>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R22" t="n">
-        <v>4613</v>
+        <v>4813</v>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>INTANGÍVEIS E OUTROS INVESTIMENTOS</t>
         </is>
       </c>
       <c r="T22" t="n">
-        <v>61000</v>
+        <v>12400</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>OUTRAS ORIGENS</t>
+          <t>OUTRAS ENTIDADES - BDMG</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>MINAS GERAÇÃO DE VALOR</t>
+          <t>INVESTIMENTO NA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B23" t="n">
         <v>1220</v>
@@ -2375,80 +2375,80 @@
         <v>3</v>
       </c>
       <c r="E23" t="n">
-        <v>5381</v>
+        <v>5201</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
+          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>9239</v>
+        <v>11046</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="I23" t="n">
-        <v>122</v>
+        <v>694</v>
       </c>
       <c r="J23" t="n">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="K23" t="n">
         <v>8</v>
       </c>
       <c r="L23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M23" t="n">
-        <v>8002</v>
+        <v>8003</v>
       </c>
       <c r="N23" t="n">
-        <v>4300000</v>
+        <v>250000000</v>
       </c>
       <c r="O23" t="n">
         <v>0</v>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R23" t="n">
-        <v>4614</v>
+        <v>4819</v>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T23" t="n">
-        <v>51000</v>
+        <v>12400</v>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OUTRAS ENTIDADES - BDMG</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
+          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B24" t="n">
         <v>1220</v>
@@ -2462,80 +2462,80 @@
         <v>3</v>
       </c>
       <c r="E24" t="n">
-        <v>5381</v>
+        <v>5201</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
+          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>9239</v>
+        <v>10991</v>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="I24" t="n">
-        <v>122</v>
+        <v>694</v>
       </c>
       <c r="J24" t="n">
-        <v>57</v>
+        <v>171</v>
       </c>
       <c r="K24" t="n">
         <v>8</v>
       </c>
       <c r="L24" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M24" t="n">
-        <v>8002</v>
+        <v>8006</v>
       </c>
       <c r="N24" t="n">
-        <v>200000</v>
+        <v>600000000</v>
       </c>
       <c r="O24" t="n">
         <v>0</v>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R24" t="n">
-        <v>4615</v>
+        <v>4819</v>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>MÓVEIS E UTENSÍLIOS</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T24" t="n">
-        <v>51000</v>
+        <v>12400</v>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OUTRAS ENTIDADES - BDMG</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
+          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B25" t="n">
         <v>1220</v>
@@ -2549,80 +2549,80 @@
         <v>3</v>
       </c>
       <c r="E25" t="n">
-        <v>5381</v>
+        <v>5251</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
+          <t>COMPANHIA DE GÁS DE MINAS GERAIS - GASMIG</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>9239</v>
+        <v>11027</v>
       </c>
       <c r="H25" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="I25" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="J25" t="n">
-        <v>57</v>
+        <v>133</v>
       </c>
       <c r="K25" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L25" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="M25" t="n">
-        <v>8002</v>
+        <v>3018</v>
       </c>
       <c r="N25" t="n">
-        <v>4000000</v>
+        <v>285487805</v>
       </c>
       <c r="O25" t="n">
         <v>0</v>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R25" t="n">
-        <v>4817</v>
+        <v>4613</v>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>EQUIPAMENTOS E SOFTWARE</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T25" t="n">
-        <v>51000</v>
+        <v>61000</v>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OUTRAS ORIGENS</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
+          <t>MINAS GERAÇÃO DE VALOR</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B26" t="n">
         <v>1220</v>
@@ -2665,7 +2665,7 @@
         <v>8002</v>
       </c>
       <c r="N26" t="n">
-        <v>1000</v>
+        <v>5450000</v>
       </c>
       <c r="O26" t="n">
         <v>0</v>
@@ -2677,23 +2677,23 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R26" t="n">
-        <v>4819</v>
+        <v>4614</v>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T26" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
@@ -2709,7 +2709,7 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B27" t="n">
         <v>1220</v>
@@ -2723,43 +2723,43 @@
         <v>3</v>
       </c>
       <c r="E27" t="n">
-        <v>5391</v>
+        <v>5381</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>9420</v>
+        <v>9239</v>
       </c>
       <c r="H27" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I27" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J27" t="n">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="K27" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L27" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M27" t="n">
-        <v>3004</v>
+        <v>8002</v>
       </c>
       <c r="N27" t="n">
-        <v>198940203</v>
+        <v>400000</v>
       </c>
       <c r="O27" t="n">
         <v>0</v>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -2768,11 +2768,11 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>4613</v>
+        <v>4615</v>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>MÓVEIS E UTENSÍLIOS</t>
         </is>
       </c>
       <c r="T27" t="n">
@@ -2785,18 +2785,18 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
+          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B28" t="n">
         <v>1220</v>
@@ -2810,56 +2810,56 @@
         <v>3</v>
       </c>
       <c r="E28" t="n">
-        <v>5391</v>
+        <v>5381</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>9421</v>
+        <v>9239</v>
       </c>
       <c r="H28" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I28" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J28" t="n">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="K28" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L28" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M28" t="n">
-        <v>3005</v>
+        <v>8002</v>
       </c>
       <c r="N28" t="n">
-        <v>241821909</v>
+        <v>4000000</v>
       </c>
       <c r="O28" t="n">
         <v>0</v>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R28" t="n">
-        <v>4613</v>
+        <v>4817</v>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
         </is>
       </c>
       <c r="T28" t="n">
@@ -2872,18 +2872,18 @@
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
+          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B29" t="n">
         <v>1220</v>
@@ -2897,80 +2897,80 @@
         <v>3</v>
       </c>
       <c r="E29" t="n">
-        <v>5391</v>
+        <v>5381</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>9430</v>
+        <v>9239</v>
       </c>
       <c r="H29" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I29" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J29" t="n">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="K29" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L29" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M29" t="n">
-        <v>3006</v>
+        <v>8002</v>
       </c>
       <c r="N29" t="n">
-        <v>30805275</v>
+        <v>1000</v>
       </c>
       <c r="O29" t="n">
         <v>0</v>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R29" t="n">
-        <v>4614</v>
+        <v>4819</v>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T29" t="n">
-        <v>51000</v>
+        <v>11101</v>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
+          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B30" t="n">
         <v>1220</v>
@@ -2992,7 +2992,7 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>10062</v>
+        <v>9420</v>
       </c>
       <c r="H30" t="n">
         <v>25</v>
@@ -3001,26 +3001,26 @@
         <v>752</v>
       </c>
       <c r="J30" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="K30" t="n">
         <v>3</v>
       </c>
       <c r="L30" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M30" t="n">
-        <v>3001</v>
+        <v>3004</v>
       </c>
       <c r="N30" t="n">
-        <v>49096963</v>
+        <v>231539977</v>
       </c>
       <c r="O30" t="n">
         <v>0</v>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
+          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -3046,18 +3046,18 @@
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
+          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B31" t="n">
         <v>1220</v>
@@ -3079,7 +3079,7 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>9440</v>
+        <v>9421</v>
       </c>
       <c r="H31" t="n">
         <v>25</v>
@@ -3088,26 +3088,26 @@
         <v>752</v>
       </c>
       <c r="J31" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="K31" t="n">
         <v>3</v>
       </c>
       <c r="L31" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M31" t="n">
-        <v>3007</v>
+        <v>3005</v>
       </c>
       <c r="N31" t="n">
-        <v>130600000</v>
+        <v>216613767</v>
       </c>
       <c r="O31" t="n">
         <v>0</v>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
+          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -3116,11 +3116,11 @@
         </is>
       </c>
       <c r="R31" t="n">
-        <v>4614</v>
+        <v>4613</v>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T31" t="n">
@@ -3133,18 +3133,18 @@
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
+          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B32" t="n">
         <v>1220</v>
@@ -3166,7 +3166,7 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>9450</v>
+        <v>9430</v>
       </c>
       <c r="H32" t="n">
         <v>25</v>
@@ -3175,26 +3175,26 @@
         <v>752</v>
       </c>
       <c r="J32" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="K32" t="n">
         <v>3</v>
       </c>
       <c r="L32" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M32" t="n">
-        <v>3008</v>
+        <v>3006</v>
       </c>
       <c r="N32" t="n">
-        <v>13194360</v>
+        <v>42479000</v>
       </c>
       <c r="O32" t="n">
         <v>0</v>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -3220,18 +3220,18 @@
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B33" t="n">
         <v>1220</v>
@@ -3253,7 +3253,7 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>10677</v>
+        <v>11134</v>
       </c>
       <c r="H33" t="n">
         <v>25</v>
@@ -3262,26 +3262,26 @@
         <v>752</v>
       </c>
       <c r="J33" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="K33" t="n">
         <v>3</v>
       </c>
       <c r="L33" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="M33" t="n">
-        <v>3014</v>
+        <v>3009</v>
       </c>
       <c r="N33" t="n">
-        <v>508846661</v>
+        <v>92271447</v>
       </c>
       <c r="O33" t="n">
         <v>0</v>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>INVESTIMENTOS PARTICIPAÇÕES SOCIETÁRIAS DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -3307,18 +3307,18 @@
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>INVESTIMENTOS PARTICIPAÇÕES SOCIETÁRIAS DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B34" t="n">
         <v>1220</v>
@@ -3332,15 +3332,15 @@
         <v>3</v>
       </c>
       <c r="E34" t="n">
-        <v>5401</v>
+        <v>5391</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>9332</v>
+        <v>10062</v>
       </c>
       <c r="H34" t="n">
         <v>25</v>
@@ -3349,26 +3349,26 @@
         <v>752</v>
       </c>
       <c r="J34" t="n">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="K34" t="n">
         <v>3</v>
       </c>
       <c r="L34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>3002</v>
+        <v>3001</v>
       </c>
       <c r="N34" t="n">
-        <v>3487433034</v>
+        <v>100000</v>
       </c>
       <c r="O34" t="n">
         <v>0</v>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
+          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -3394,18 +3394,18 @@
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
+          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
         </is>
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B35" t="n">
         <v>1220</v>
@@ -3419,15 +3419,15 @@
         <v>3</v>
       </c>
       <c r="E35" t="n">
-        <v>5401</v>
+        <v>5391</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>9408</v>
+        <v>9440</v>
       </c>
       <c r="H35" t="n">
         <v>25</v>
@@ -3436,26 +3436,26 @@
         <v>752</v>
       </c>
       <c r="J35" t="n">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="K35" t="n">
         <v>3</v>
       </c>
       <c r="L35" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="M35" t="n">
-        <v>3003</v>
+        <v>3007</v>
       </c>
       <c r="N35" t="n">
-        <v>247223810</v>
+        <v>96218712</v>
       </c>
       <c r="O35" t="n">
         <v>0</v>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
+          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -3481,18 +3481,18 @@
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
+          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
         </is>
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B36" t="n">
         <v>1220</v>
@@ -3506,43 +3506,43 @@
         <v>3</v>
       </c>
       <c r="E36" t="n">
-        <v>5511</v>
+        <v>5391</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>11024</v>
+        <v>9450</v>
       </c>
       <c r="H36" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I36" t="n">
-        <v>512</v>
+        <v>752</v>
       </c>
       <c r="J36" t="n">
-        <v>21</v>
+        <v>94</v>
       </c>
       <c r="K36" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L36" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="M36" t="n">
-        <v>6012</v>
+        <v>3008</v>
       </c>
       <c r="N36" t="n">
-        <v>2000000</v>
+        <v>18091000</v>
       </c>
       <c r="O36" t="n">
         <v>0</v>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -3568,18 +3568,18 @@
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
         </is>
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
+          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B37" t="n">
         <v>1220</v>
@@ -3593,56 +3593,56 @@
         <v>3</v>
       </c>
       <c r="E37" t="n">
-        <v>5511</v>
+        <v>5391</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>11026</v>
+        <v>10677</v>
       </c>
       <c r="H37" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I37" t="n">
-        <v>512</v>
+        <v>752</v>
       </c>
       <c r="J37" t="n">
-        <v>21</v>
+        <v>94</v>
       </c>
       <c r="K37" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L37" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="M37" t="n">
-        <v>8012</v>
+        <v>3014</v>
       </c>
       <c r="N37" t="n">
-        <v>45000000</v>
+        <v>190392082</v>
       </c>
       <c r="O37" t="n">
         <v>0</v>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS DA GERAÇÃO</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R37" t="n">
-        <v>4613</v>
+        <v>4511</v>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T37" t="n">
@@ -3655,155 +3655,155 @@
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS DA GERAÇÃO</t>
         </is>
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
+          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B38" t="n">
-        <v>1300</v>
+        <v>1220</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA, MOBILIDADE E PARCERIA - SEINFRA</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D38" t="n">
         <v>3</v>
       </c>
       <c r="E38" t="n">
-        <v>5261</v>
+        <v>5401</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>TREM METROPOLITANO DE BELO HORIZONTE S.A - TREM METROPOLITANO</t>
+          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>9927</v>
+        <v>9332</v>
       </c>
       <c r="H38" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I38" t="n">
-        <v>783</v>
+        <v>752</v>
       </c>
       <c r="J38" t="n">
-        <v>705</v>
+        <v>72</v>
       </c>
       <c r="K38" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L38" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="M38" t="n">
-        <v>8011</v>
+        <v>3002</v>
       </c>
       <c r="N38" t="n">
-        <v>1000</v>
+        <v>4721877188</v>
       </c>
       <c r="O38" t="n">
         <v>0</v>
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R38" t="n">
-        <v>4511</v>
+        <v>4613</v>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T38" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
         </is>
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
+          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B39" t="n">
-        <v>1500</v>
+        <v>1220</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D39" t="n">
         <v>3</v>
       </c>
       <c r="E39" t="n">
-        <v>5141</v>
+        <v>5401</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
         </is>
       </c>
       <c r="G39" t="n">
-        <v>10882</v>
+        <v>9408</v>
       </c>
       <c r="H39" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="I39" t="n">
-        <v>126</v>
+        <v>752</v>
       </c>
       <c r="J39" t="n">
-        <v>30</v>
+        <v>72</v>
       </c>
       <c r="K39" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L39" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M39" t="n">
-        <v>6006</v>
+        <v>3003</v>
       </c>
       <c r="N39" t="n">
-        <v>3280000</v>
+        <v>247976000</v>
       </c>
       <c r="O39" t="n">
         <v>0</v>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -3812,11 +3812,11 @@
         </is>
       </c>
       <c r="R39" t="n">
-        <v>4613</v>
+        <v>4614</v>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T39" t="n">
@@ -3829,81 +3829,81 @@
       </c>
       <c r="V39" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B40" t="n">
-        <v>1500</v>
+        <v>1220</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D40" t="n">
         <v>3</v>
       </c>
       <c r="E40" t="n">
-        <v>5141</v>
+        <v>5511</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>9116</v>
+        <v>11024</v>
       </c>
       <c r="H40" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I40" t="n">
-        <v>126</v>
+        <v>512</v>
       </c>
       <c r="J40" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="K40" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L40" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="M40" t="n">
-        <v>8001</v>
+        <v>6012</v>
       </c>
       <c r="N40" t="n">
-        <v>35386354</v>
+        <v>2000000</v>
       </c>
       <c r="O40" t="n">
         <v>0</v>
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R40" t="n">
-        <v>4817</v>
+        <v>4614</v>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>EQUIPAMENTOS E SOFTWARE</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T40" t="n">
@@ -3916,10 +3916,358 @@
       </c>
       <c r="V40" t="inlineStr">
         <is>
+          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B41" t="n">
+        <v>1220</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" t="n">
+        <v>5511</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>11026</v>
+      </c>
+      <c r="H41" t="n">
+        <v>17</v>
+      </c>
+      <c r="I41" t="n">
+        <v>512</v>
+      </c>
+      <c r="J41" t="n">
+        <v>21</v>
+      </c>
+      <c r="K41" t="n">
+        <v>8</v>
+      </c>
+      <c r="L41" t="n">
+        <v>12</v>
+      </c>
+      <c r="M41" t="n">
+        <v>8012</v>
+      </c>
+      <c r="N41" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="O41" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>4610 - IMOBILIZAÇÕES</t>
+        </is>
+      </c>
+      <c r="R41" t="n">
+        <v>4613</v>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>OBRAS E INSTALAÇÕES</t>
+        </is>
+      </c>
+      <c r="T41" t="n">
+        <v>51000</v>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>RECURSOS PRÓPRIOS</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B42" t="n">
+        <v>1300</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA, MOBILIDADE E PARCERIA - SEINFRA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>3</v>
+      </c>
+      <c r="E42" t="n">
+        <v>5261</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>TREM METROPOLITANO DE BELO HORIZONTE S.A - TREM METROPOLITANO</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>9927</v>
+      </c>
+      <c r="H42" t="n">
+        <v>26</v>
+      </c>
+      <c r="I42" t="n">
+        <v>783</v>
+      </c>
+      <c r="J42" t="n">
+        <v>705</v>
+      </c>
+      <c r="K42" t="n">
+        <v>8</v>
+      </c>
+      <c r="L42" t="n">
+        <v>11</v>
+      </c>
+      <c r="M42" t="n">
+        <v>8011</v>
+      </c>
+      <c r="N42" t="n">
+        <v>1000</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0</v>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+        </is>
+      </c>
+      <c r="R42" t="n">
+        <v>4511</v>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>SOCIEDADES CONTROLADAS</t>
+        </is>
+      </c>
+      <c r="T42" t="n">
+        <v>11101</v>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B43" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>3</v>
+      </c>
+      <c r="E43" t="n">
+        <v>5141</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>10882</v>
+      </c>
+      <c r="H43" t="n">
+        <v>4</v>
+      </c>
+      <c r="I43" t="n">
+        <v>126</v>
+      </c>
+      <c r="J43" t="n">
+        <v>30</v>
+      </c>
+      <c r="K43" t="n">
+        <v>6</v>
+      </c>
+      <c r="L43" t="n">
+        <v>6</v>
+      </c>
+      <c r="M43" t="n">
+        <v>6006</v>
+      </c>
+      <c r="N43" t="n">
+        <v>13233200</v>
+      </c>
+      <c r="O43" t="n">
+        <v>0</v>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>4610 - IMOBILIZAÇÕES</t>
+        </is>
+      </c>
+      <c r="R43" t="n">
+        <v>4613</v>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>OBRAS E INSTALAÇÕES</t>
+        </is>
+      </c>
+      <c r="T43" t="n">
+        <v>51000</v>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>RECURSOS PRÓPRIOS</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
+        </is>
+      </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B44" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>3</v>
+      </c>
+      <c r="E44" t="n">
+        <v>5141</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>9116</v>
+      </c>
+      <c r="H44" t="n">
+        <v>4</v>
+      </c>
+      <c r="I44" t="n">
+        <v>126</v>
+      </c>
+      <c r="J44" t="n">
+        <v>30</v>
+      </c>
+      <c r="K44" t="n">
+        <v>8</v>
+      </c>
+      <c r="L44" t="n">
+        <v>1</v>
+      </c>
+      <c r="M44" t="n">
+        <v>8001</v>
+      </c>
+      <c r="N44" t="n">
+        <v>38099783</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
           <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
         </is>
       </c>
-      <c r="W40" t="inlineStr">
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
+        </is>
+      </c>
+      <c r="R44" t="n">
+        <v>4817</v>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
+        </is>
+      </c>
+      <c r="T44" t="n">
+        <v>51000</v>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>RECURSOS PRÓPRIOS</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr">
         <is>
           <t>SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
         </is>

</xml_diff>

<commit_message>
chore(ploa2026): 1ª iteração dos volumes ploa.
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_QDD_INVESTIMENTO.xlsx
+++ b/bancos/SISOR/BASE_QDD_INVESTIMENTO.xlsx
@@ -534,7 +534,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B2" t="n">
         <v>1220</v>
@@ -621,7 +621,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B3" t="n">
         <v>1220</v>
@@ -664,7 +664,7 @@
         <v>3015</v>
       </c>
       <c r="N3" t="n">
-        <v>6380000</v>
+        <v>3500000</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -708,7 +708,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B4" t="n">
         <v>1220</v>
@@ -751,7 +751,7 @@
         <v>3015</v>
       </c>
       <c r="N4" t="n">
-        <v>6240000</v>
+        <v>4655000</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
@@ -795,7 +795,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B5" t="n">
         <v>1220</v>
@@ -882,7 +882,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B6" t="n">
         <v>1220</v>
@@ -904,35 +904,35 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>11021</v>
+        <v>11280</v>
       </c>
       <c r="H6" t="n">
         <v>17</v>
       </c>
       <c r="I6" t="n">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="J6" t="n">
-        <v>21</v>
+        <v>101</v>
       </c>
       <c r="K6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="M6" t="n">
-        <v>6009</v>
+        <v>3012</v>
       </c>
       <c r="N6" t="n">
-        <v>50000000</v>
+        <v>5000000</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
+          <t>DOAÇÃO DE MÓDULOS DE FOSSAS SÉPTICAS PARA MUNICÍPIOS SEM CONCESSÃO COPASA (CONVÊNIO DEFESA CIVIL)</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -949,27 +949,27 @@
         </is>
       </c>
       <c r="T6" t="n">
-        <v>22199</v>
+        <v>51000</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
+          <t>DOAÇÃO DE MÓDULOS DE FOSSAS SÉPTICAS PARA MUNICÍPIOS SEM CONCESSÃO COPASA (CONVÊNIO DEFESA CIVIL)</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
+          <t>PROGRAMA ENCONTRO DAS ÁGUAS</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B7" t="n">
         <v>1220</v>
@@ -1036,11 +1036,11 @@
         </is>
       </c>
       <c r="T7" t="n">
-        <v>51000</v>
+        <v>22199</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1056,7 +1056,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B8" t="n">
         <v>1220</v>
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>11022</v>
+        <v>11021</v>
       </c>
       <c r="H8" t="n">
         <v>17</v>
@@ -1090,23 +1090,23 @@
         <v>21</v>
       </c>
       <c r="K8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M8" t="n">
-        <v>8008</v>
+        <v>6009</v>
       </c>
       <c r="N8" t="n">
-        <v>100000000</v>
+        <v>50000000</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
+          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1115,11 +1115,11 @@
         </is>
       </c>
       <c r="R8" t="n">
-        <v>4611</v>
+        <v>4614</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>TERRENOS</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T8" t="n">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
+          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
@@ -1143,7 +1143,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B9" t="n">
         <v>1220</v>
@@ -1186,7 +1186,7 @@
         <v>8008</v>
       </c>
       <c r="N9" t="n">
-        <v>350000000</v>
+        <v>95000000</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
@@ -1202,19 +1202,19 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>4613</v>
+        <v>4611</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>TERRENOS</t>
         </is>
       </c>
       <c r="T9" t="n">
-        <v>21204</v>
+        <v>51000</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>OP CRÉD CONTRAT EXTERNA - KFW</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1230,7 +1230,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B10" t="n">
         <v>1220</v>
@@ -1273,7 +1273,7 @@
         <v>8008</v>
       </c>
       <c r="N10" t="n">
-        <v>983250000</v>
+        <v>350000000</v>
       </c>
       <c r="O10" t="n">
         <v>0</v>
@@ -1297,11 +1297,11 @@
         </is>
       </c>
       <c r="T10" t="n">
-        <v>22199</v>
+        <v>21204</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
+          <t>OP CRÉD CONTRAT EXTERNA - KFW</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1317,7 +1317,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B11" t="n">
         <v>1220</v>
@@ -1360,7 +1360,7 @@
         <v>8008</v>
       </c>
       <c r="N11" t="n">
-        <v>54750000</v>
+        <v>2510000000</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
@@ -1384,11 +1384,11 @@
         </is>
       </c>
       <c r="T11" t="n">
-        <v>51000</v>
+        <v>22199</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -1404,7 +1404,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B12" t="n">
         <v>1220</v>
@@ -1447,7 +1447,7 @@
         <v>8008</v>
       </c>
       <c r="N12" t="n">
-        <v>40000000</v>
+        <v>100000000</v>
       </c>
       <c r="O12" t="n">
         <v>0</v>
@@ -1463,19 +1463,19 @@
         </is>
       </c>
       <c r="R12" t="n">
-        <v>4614</v>
+        <v>4613</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T12" t="n">
-        <v>22199</v>
+        <v>51000</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
@@ -1491,7 +1491,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B13" t="n">
         <v>1220</v>
@@ -1513,7 +1513,7 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>11023</v>
+        <v>11022</v>
       </c>
       <c r="H13" t="n">
         <v>17</v>
@@ -1528,20 +1528,20 @@
         <v>8</v>
       </c>
       <c r="L13" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M13" t="n">
-        <v>8009</v>
+        <v>8008</v>
       </c>
       <c r="N13" t="n">
-        <v>48428689</v>
+        <v>40000000</v>
       </c>
       <c r="O13" t="n">
         <v>0</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>PPP SISTEMA ADUTOR RIO MANSO</t>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -1550,24 +1550,24 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>4613</v>
+        <v>4614</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T13" t="n">
-        <v>51000</v>
+        <v>22199</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>PPP SISTEMA ADUTOR RIO MANSO</t>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
@@ -1578,7 +1578,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B14" t="n">
         <v>1220</v>
@@ -1592,56 +1592,56 @@
         <v>3</v>
       </c>
       <c r="E14" t="n">
-        <v>5121</v>
+        <v>5081</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>COMPANHIA ENERGÉTICA DE MINAS GERAIS - CEMIG HOLDING</t>
+          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>10542</v>
+        <v>11023</v>
       </c>
       <c r="H14" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="I14" t="n">
-        <v>752</v>
+        <v>512</v>
       </c>
       <c r="J14" t="n">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="K14" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L14" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="M14" t="n">
-        <v>3010</v>
+        <v>8009</v>
       </c>
       <c r="N14" t="n">
-        <v>259985809</v>
+        <v>55500000</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
+          <t>PPP SISTEMA ADUTOR RIO MANSO</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R14" t="n">
-        <v>4511</v>
+        <v>4613</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T14" t="n">
@@ -1654,18 +1654,18 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
+          <t>PPP SISTEMA ADUTOR RIO MANSO</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS CEMIG</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B15" t="n">
         <v>1220</v>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>9994</v>
+        <v>10542</v>
       </c>
       <c r="H15" t="n">
         <v>25</v>
@@ -1702,33 +1702,33 @@
         <v>3</v>
       </c>
       <c r="L15" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="M15" t="n">
-        <v>3011</v>
+        <v>3010</v>
       </c>
       <c r="N15" t="n">
-        <v>4440000</v>
+        <v>70784312</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R15" t="n">
-        <v>4614</v>
+        <v>4511</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T15" t="n">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
@@ -1752,7 +1752,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B16" t="n">
         <v>1220</v>
@@ -1766,43 +1766,43 @@
         <v>3</v>
       </c>
       <c r="E16" t="n">
-        <v>5131</v>
+        <v>5121</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>AGÊNCIA DE PROMOÇÃO DE INVESTIMENTOS DE MINAS GERAIS - INVEST MINAS</t>
+          <t>COMPANHIA ENERGÉTICA DE MINAS GERAIS - CEMIG HOLDING</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>9723</v>
+        <v>9994</v>
       </c>
       <c r="H16" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I16" t="n">
-        <v>122</v>
+        <v>752</v>
       </c>
       <c r="J16" t="n">
-        <v>142</v>
+        <v>35</v>
       </c>
       <c r="K16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L16" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="M16" t="n">
-        <v>6008</v>
+        <v>3011</v>
       </c>
       <c r="N16" t="n">
-        <v>500000</v>
+        <v>2347000</v>
       </c>
       <c r="O16" t="n">
         <v>0</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1828,18 +1828,18 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL - INVEST MINAS</t>
+          <t>INVESTIMENTOS CEMIG</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B17" t="n">
         <v>1220</v>
@@ -1853,56 +1853,56 @@
         <v>3</v>
       </c>
       <c r="E17" t="n">
-        <v>5191</v>
+        <v>5131</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
+          <t>AGÊNCIA DE PROMOÇÃO DE INVESTIMENTOS DE MINAS GERAIS - INVEST MINAS</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>9796</v>
+        <v>9723</v>
       </c>
       <c r="H17" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="I17" t="n">
         <v>122</v>
       </c>
       <c r="J17" t="n">
-        <v>13</v>
+        <v>142</v>
       </c>
       <c r="K17" t="n">
         <v>6</v>
       </c>
       <c r="L17" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="M17" t="n">
-        <v>6011</v>
+        <v>6008</v>
       </c>
       <c r="N17" t="n">
-        <v>243000</v>
+        <v>250000</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R17" t="n">
-        <v>4817</v>
+        <v>4614</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>EQUIPAMENTOS E SOFTWARE</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T17" t="n">
@@ -1915,18 +1915,18 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL - INVEST MINAS</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B18" t="n">
         <v>1220</v>
@@ -1948,7 +1948,7 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>11036</v>
+        <v>9796</v>
       </c>
       <c r="H18" t="n">
         <v>4</v>
@@ -1957,26 +1957,26 @@
         <v>122</v>
       </c>
       <c r="J18" t="n">
-        <v>119</v>
+        <v>13</v>
       </c>
       <c r="K18" t="n">
         <v>6</v>
       </c>
       <c r="L18" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="M18" t="n">
-        <v>6003</v>
+        <v>6011</v>
       </c>
       <c r="N18" t="n">
-        <v>1000</v>
+        <v>240000</v>
       </c>
       <c r="O18" t="n">
         <v>0</v>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -1985,35 +1985,35 @@
         </is>
       </c>
       <c r="R18" t="n">
-        <v>4819</v>
+        <v>4817</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
         </is>
       </c>
       <c r="T18" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>APOIO AO DESENVOLVIMENTO MUNICIPAL E À COORDENAÇÃO DAS TRANSFERÊNCIAS ESTADUAIS DE RECURSOS FINANCEIROS</t>
+          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B19" t="n">
         <v>1220</v>
@@ -2056,7 +2056,7 @@
         <v>6003</v>
       </c>
       <c r="N19" t="n">
-        <v>9256395</v>
+        <v>1000</v>
       </c>
       <c r="O19" t="n">
         <v>0</v>
@@ -2080,11 +2080,11 @@
         </is>
       </c>
       <c r="T19" t="n">
-        <v>51000</v>
+        <v>11101</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
@@ -2100,7 +2100,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B20" t="n">
         <v>1220</v>
@@ -2122,72 +2122,72 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>9058</v>
+        <v>11036</v>
       </c>
       <c r="H20" t="n">
         <v>4</v>
       </c>
       <c r="I20" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J20" t="n">
-        <v>13</v>
+        <v>119</v>
       </c>
       <c r="K20" t="n">
         <v>6</v>
       </c>
       <c r="L20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M20" t="n">
-        <v>6001</v>
+        <v>6003</v>
       </c>
       <c r="N20" t="n">
-        <v>1000</v>
+        <v>1461000</v>
       </c>
       <c r="O20" t="n">
         <v>0</v>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R20" t="n">
-        <v>4511</v>
+        <v>4819</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T20" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>APOIO AO DESENVOLVIMENTO MUNICIPAL E À COORDENAÇÃO DAS TRANSFERÊNCIAS ESTADUAIS DE RECURSOS FINANCEIROS</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B21" t="n">
         <v>1220</v>
@@ -2254,11 +2254,11 @@
         </is>
       </c>
       <c r="T21" t="n">
-        <v>51000</v>
+        <v>11101</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
@@ -2274,7 +2274,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B22" t="n">
         <v>1220</v>
@@ -2288,80 +2288,80 @@
         <v>3</v>
       </c>
       <c r="E22" t="n">
-        <v>5201</v>
+        <v>5191</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
+          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>9087</v>
+        <v>9058</v>
       </c>
       <c r="H22" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="I22" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J22" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="K22" t="n">
         <v>6</v>
       </c>
       <c r="L22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>6004</v>
+        <v>6001</v>
       </c>
       <c r="N22" t="n">
-        <v>26253389</v>
+        <v>1000</v>
       </c>
       <c r="O22" t="n">
         <v>0</v>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
+          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R22" t="n">
-        <v>4813</v>
+        <v>4511</v>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>INTANGÍVEIS E OUTROS INVESTIMENTOS</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T22" t="n">
-        <v>12400</v>
+        <v>51000</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>OUTRAS ENTIDADES - BDMG</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
+          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>INVESTIMENTO NA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
+          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B23" t="n">
         <v>1220</v>
@@ -2383,35 +2383,35 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>11046</v>
+        <v>9087</v>
       </c>
       <c r="H23" t="n">
         <v>23</v>
       </c>
       <c r="I23" t="n">
-        <v>694</v>
+        <v>122</v>
       </c>
       <c r="J23" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="K23" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M23" t="n">
-        <v>8003</v>
+        <v>6004</v>
       </c>
       <c r="N23" t="n">
-        <v>250000000</v>
+        <v>30022403</v>
       </c>
       <c r="O23" t="n">
         <v>0</v>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -2420,11 +2420,11 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>4819</v>
+        <v>4813</v>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>INTANGÍVEIS E OUTROS INVESTIMENTOS</t>
         </is>
       </c>
       <c r="T23" t="n">
@@ -2437,18 +2437,18 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
+          <t>INVESTIMENTO NA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B24" t="n">
         <v>1220</v>
@@ -2470,7 +2470,7 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>10991</v>
+        <v>11046</v>
       </c>
       <c r="H24" t="n">
         <v>23</v>
@@ -2479,26 +2479,26 @@
         <v>694</v>
       </c>
       <c r="J24" t="n">
-        <v>171</v>
+        <v>14</v>
       </c>
       <c r="K24" t="n">
         <v>8</v>
       </c>
       <c r="L24" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M24" t="n">
-        <v>8006</v>
+        <v>8003</v>
       </c>
       <c r="N24" t="n">
-        <v>600000000</v>
+        <v>250000000</v>
       </c>
       <c r="O24" t="n">
         <v>0</v>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
+          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -2524,18 +2524,18 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
+          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
+          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B25" t="n">
         <v>1220</v>
@@ -2549,80 +2549,80 @@
         <v>3</v>
       </c>
       <c r="E25" t="n">
-        <v>5251</v>
+        <v>5201</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>COMPANHIA DE GÁS DE MINAS GERAIS - GASMIG</t>
+          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>11027</v>
+        <v>11249</v>
       </c>
       <c r="H25" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I25" t="n">
-        <v>121</v>
+        <v>694</v>
       </c>
       <c r="J25" t="n">
-        <v>133</v>
+        <v>107</v>
       </c>
       <c r="K25" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L25" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="M25" t="n">
-        <v>3018</v>
+        <v>8004</v>
       </c>
       <c r="N25" t="n">
-        <v>285487805</v>
+        <v>500000000</v>
       </c>
       <c r="O25" t="n">
         <v>0</v>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
+          <t>FINANCIAMENTO À SUSTENTABILIDADE E ÀS MICRO E PEQUENAS EMPRESAS DO ESTADO DE MINAS GERAIS ENTRE BDMG E BANCO EUROPEU DE INVESTIMENTO (BDMG SUSTENTABILIDADE E MPE)</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R25" t="n">
-        <v>4613</v>
+        <v>4819</v>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T25" t="n">
-        <v>61000</v>
+        <v>12400</v>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>OUTRAS ORIGENS</t>
+          <t>OUTRAS ENTIDADES - BDMG</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
+          <t>FINANCIAMENTO À SUSTENTABILIDADE E ÀS MICRO E PEQUENAS EMPRESAS DO ESTADO DE MINAS GERAIS ENTRE BDMG E BANCO EUROPEU DE INVESTIMENTO (BDMG SUSTENTABILIDADE E MPE)</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>MINAS GERAÇÃO DE VALOR</t>
+          <t>FINANCIAMENTO À SUSTENTABILIDADE E ÀS MICRO E PEQUENAS EMPRESAS DO ESTADO DE MINAS GERAIS ENTRE BDMG E BANCO EUROPEU DE INVESTIMENTO (BDMG SUSTENTABILIDADE E MPE)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B26" t="n">
         <v>1220</v>
@@ -2636,80 +2636,80 @@
         <v>3</v>
       </c>
       <c r="E26" t="n">
-        <v>5381</v>
+        <v>5201</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
+          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>9239</v>
+        <v>10991</v>
       </c>
       <c r="H26" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="I26" t="n">
-        <v>122</v>
+        <v>694</v>
       </c>
       <c r="J26" t="n">
-        <v>57</v>
+        <v>171</v>
       </c>
       <c r="K26" t="n">
         <v>8</v>
       </c>
       <c r="L26" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M26" t="n">
-        <v>8002</v>
+        <v>8006</v>
       </c>
       <c r="N26" t="n">
-        <v>5450000</v>
+        <v>600000000</v>
       </c>
       <c r="O26" t="n">
         <v>0</v>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R26" t="n">
-        <v>4614</v>
+        <v>4819</v>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T26" t="n">
-        <v>51000</v>
+        <v>12400</v>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OUTRAS ENTIDADES - BDMG</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
+          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B27" t="n">
         <v>1220</v>
@@ -2723,56 +2723,56 @@
         <v>3</v>
       </c>
       <c r="E27" t="n">
-        <v>5381</v>
+        <v>5251</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
+          <t>COMPANHIA DE GÁS DE MINAS GERAIS - GASMIG</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>9239</v>
+        <v>11027</v>
       </c>
       <c r="H27" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="I27" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="J27" t="n">
-        <v>57</v>
+        <v>133</v>
       </c>
       <c r="K27" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L27" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="M27" t="n">
-        <v>8002</v>
+        <v>3018</v>
       </c>
       <c r="N27" t="n">
-        <v>400000</v>
+        <v>191687487</v>
       </c>
       <c r="O27" t="n">
         <v>0</v>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R27" t="n">
-        <v>4615</v>
+        <v>4819</v>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>MÓVEIS E UTENSÍLIOS</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T27" t="n">
@@ -2785,18 +2785,18 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
         </is>
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
+          <t>MINAS GERAÇÃO DE VALOR</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B28" t="n">
         <v>1220</v>
@@ -2839,7 +2839,7 @@
         <v>8002</v>
       </c>
       <c r="N28" t="n">
-        <v>4000000</v>
+        <v>9152200</v>
       </c>
       <c r="O28" t="n">
         <v>0</v>
@@ -2851,15 +2851,15 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R28" t="n">
-        <v>4817</v>
+        <v>4614</v>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>EQUIPAMENTOS E SOFTWARE</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T28" t="n">
@@ -2883,7 +2883,7 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B29" t="n">
         <v>1220</v>
@@ -2926,7 +2926,7 @@
         <v>8002</v>
       </c>
       <c r="N29" t="n">
-        <v>1000</v>
+        <v>522300</v>
       </c>
       <c r="O29" t="n">
         <v>0</v>
@@ -2938,23 +2938,23 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R29" t="n">
-        <v>4819</v>
+        <v>4615</v>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>MÓVEIS E UTENSÍLIOS</t>
         </is>
       </c>
       <c r="T29" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
@@ -2970,7 +2970,7 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B30" t="n">
         <v>1220</v>
@@ -2984,56 +2984,56 @@
         <v>3</v>
       </c>
       <c r="E30" t="n">
-        <v>5391</v>
+        <v>5381</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>9420</v>
+        <v>9239</v>
       </c>
       <c r="H30" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I30" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J30" t="n">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="K30" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L30" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M30" t="n">
-        <v>3004</v>
+        <v>8002</v>
       </c>
       <c r="N30" t="n">
-        <v>231539977</v>
+        <v>12880000</v>
       </c>
       <c r="O30" t="n">
         <v>0</v>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R30" t="n">
-        <v>4613</v>
+        <v>4817</v>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
         </is>
       </c>
       <c r="T30" t="n">
@@ -3046,18 +3046,18 @@
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
+          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B31" t="n">
         <v>1220</v>
@@ -3071,80 +3071,80 @@
         <v>3</v>
       </c>
       <c r="E31" t="n">
-        <v>5391</v>
+        <v>5381</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>9421</v>
+        <v>9239</v>
       </c>
       <c r="H31" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I31" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J31" t="n">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="K31" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L31" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M31" t="n">
-        <v>3005</v>
+        <v>8002</v>
       </c>
       <c r="N31" t="n">
-        <v>216613767</v>
+        <v>1000</v>
       </c>
       <c r="O31" t="n">
         <v>0</v>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R31" t="n">
-        <v>4613</v>
+        <v>4819</v>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T31" t="n">
-        <v>51000</v>
+        <v>11101</v>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
+          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B32" t="n">
         <v>1220</v>
@@ -3166,7 +3166,7 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>9430</v>
+        <v>9420</v>
       </c>
       <c r="H32" t="n">
         <v>25</v>
@@ -3181,20 +3181,20 @@
         <v>3</v>
       </c>
       <c r="L32" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M32" t="n">
-        <v>3006</v>
+        <v>3004</v>
       </c>
       <c r="N32" t="n">
-        <v>42479000</v>
+        <v>343756125</v>
       </c>
       <c r="O32" t="n">
         <v>0</v>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
+          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -3203,11 +3203,11 @@
         </is>
       </c>
       <c r="R32" t="n">
-        <v>4614</v>
+        <v>4613</v>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T32" t="n">
@@ -3220,7 +3220,7 @@
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
+          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W32" t="inlineStr">
@@ -3231,7 +3231,7 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B33" t="n">
         <v>1220</v>
@@ -3253,7 +3253,7 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>11134</v>
+        <v>9421</v>
       </c>
       <c r="H33" t="n">
         <v>25</v>
@@ -3268,33 +3268,33 @@
         <v>3</v>
       </c>
       <c r="L33" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="M33" t="n">
-        <v>3009</v>
+        <v>3005</v>
       </c>
       <c r="N33" t="n">
-        <v>92271447</v>
+        <v>285714873</v>
       </c>
       <c r="O33" t="n">
         <v>0</v>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS PARTICIPAÇÕES SOCIETÁRIAS DA TRANSMISSÃO</t>
+          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R33" t="n">
-        <v>4511</v>
+        <v>4613</v>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T33" t="n">
@@ -3307,7 +3307,7 @@
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS PARTICIPAÇÕES SOCIETÁRIAS DA TRANSMISSÃO</t>
+          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W33" t="inlineStr">
@@ -3318,7 +3318,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B34" t="n">
         <v>1220</v>
@@ -3340,7 +3340,7 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>10062</v>
+        <v>9430</v>
       </c>
       <c r="H34" t="n">
         <v>25</v>
@@ -3349,26 +3349,26 @@
         <v>752</v>
       </c>
       <c r="J34" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="K34" t="n">
         <v>3</v>
       </c>
       <c r="L34" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="M34" t="n">
-        <v>3001</v>
+        <v>3006</v>
       </c>
       <c r="N34" t="n">
-        <v>100000</v>
+        <v>65874000</v>
       </c>
       <c r="O34" t="n">
         <v>0</v>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -3377,11 +3377,11 @@
         </is>
       </c>
       <c r="R34" t="n">
-        <v>4613</v>
+        <v>4614</v>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T34" t="n">
@@ -3394,18 +3394,18 @@
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B35" t="n">
         <v>1220</v>
@@ -3427,7 +3427,7 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>9440</v>
+        <v>11134</v>
       </c>
       <c r="H35" t="n">
         <v>25</v>
@@ -3436,39 +3436,39 @@
         <v>752</v>
       </c>
       <c r="J35" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="K35" t="n">
         <v>3</v>
       </c>
       <c r="L35" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M35" t="n">
-        <v>3007</v>
+        <v>3009</v>
       </c>
       <c r="N35" t="n">
-        <v>96218712</v>
+        <v>8146743</v>
       </c>
       <c r="O35" t="n">
         <v>0</v>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
+          <t>INVESTIMENTOS PARTICIPAÇÕES SOCIETÁRIAS DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R35" t="n">
-        <v>4614</v>
+        <v>4511</v>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T35" t="n">
@@ -3481,18 +3481,18 @@
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
+          <t>INVESTIMENTOS PARTICIPAÇÕES SOCIETÁRIAS DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B36" t="n">
         <v>1220</v>
@@ -3514,7 +3514,7 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>9450</v>
+        <v>10062</v>
       </c>
       <c r="H36" t="n">
         <v>25</v>
@@ -3529,20 +3529,20 @@
         <v>3</v>
       </c>
       <c r="L36" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>3008</v>
+        <v>3001</v>
       </c>
       <c r="N36" t="n">
-        <v>18091000</v>
+        <v>1</v>
       </c>
       <c r="O36" t="n">
         <v>0</v>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
+          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -3551,11 +3551,11 @@
         </is>
       </c>
       <c r="R36" t="n">
-        <v>4614</v>
+        <v>4613</v>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T36" t="n">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
+          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
         </is>
       </c>
       <c r="W36" t="inlineStr">
@@ -3579,7 +3579,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B37" t="n">
         <v>1220</v>
@@ -3601,7 +3601,7 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>10677</v>
+        <v>9440</v>
       </c>
       <c r="H37" t="n">
         <v>25</v>
@@ -3616,33 +3616,33 @@
         <v>3</v>
       </c>
       <c r="L37" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="M37" t="n">
-        <v>3014</v>
+        <v>3007</v>
       </c>
       <c r="N37" t="n">
-        <v>190392082</v>
+        <v>65661789</v>
       </c>
       <c r="O37" t="n">
         <v>0</v>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS DA GERAÇÃO</t>
+          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R37" t="n">
-        <v>4511</v>
+        <v>4614</v>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T37" t="n">
@@ -3655,7 +3655,7 @@
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS DA GERAÇÃO</t>
+          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
         </is>
       </c>
       <c r="W37" t="inlineStr">
@@ -3666,7 +3666,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B38" t="n">
         <v>1220</v>
@@ -3680,15 +3680,15 @@
         <v>3</v>
       </c>
       <c r="E38" t="n">
-        <v>5401</v>
+        <v>5391</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>9332</v>
+        <v>9450</v>
       </c>
       <c r="H38" t="n">
         <v>25</v>
@@ -3697,26 +3697,26 @@
         <v>752</v>
       </c>
       <c r="J38" t="n">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="K38" t="n">
         <v>3</v>
       </c>
       <c r="L38" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="M38" t="n">
-        <v>3002</v>
+        <v>3008</v>
       </c>
       <c r="N38" t="n">
-        <v>4721877188</v>
+        <v>42279000</v>
       </c>
       <c r="O38" t="n">
         <v>0</v>
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
@@ -3725,11 +3725,11 @@
         </is>
       </c>
       <c r="R38" t="n">
-        <v>4613</v>
+        <v>4614</v>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T38" t="n">
@@ -3742,18 +3742,18 @@
       </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
         </is>
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B39" t="n">
         <v>1220</v>
@@ -3767,15 +3767,15 @@
         <v>3</v>
       </c>
       <c r="E39" t="n">
-        <v>5401</v>
+        <v>5391</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G39" t="n">
-        <v>9408</v>
+        <v>10677</v>
       </c>
       <c r="H39" t="n">
         <v>25</v>
@@ -3784,39 +3784,39 @@
         <v>752</v>
       </c>
       <c r="J39" t="n">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="K39" t="n">
         <v>3</v>
       </c>
       <c r="L39" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="M39" t="n">
-        <v>3003</v>
+        <v>3014</v>
       </c>
       <c r="N39" t="n">
-        <v>247976000</v>
+        <v>116689303</v>
       </c>
       <c r="O39" t="n">
         <v>0</v>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS DA GERAÇÃO</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R39" t="n">
-        <v>4614</v>
+        <v>4511</v>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T39" t="n">
@@ -3829,18 +3829,18 @@
       </c>
       <c r="V39" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS DA GERAÇÃO</t>
         </is>
       </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B40" t="n">
         <v>1220</v>
@@ -3854,43 +3854,43 @@
         <v>3</v>
       </c>
       <c r="E40" t="n">
-        <v>5511</v>
+        <v>5401</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
+          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>11024</v>
+        <v>9332</v>
       </c>
       <c r="H40" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I40" t="n">
-        <v>512</v>
+        <v>752</v>
       </c>
       <c r="J40" t="n">
-        <v>21</v>
+        <v>72</v>
       </c>
       <c r="K40" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L40" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="M40" t="n">
-        <v>6012</v>
+        <v>3002</v>
       </c>
       <c r="N40" t="n">
-        <v>2000000</v>
+        <v>5072587386</v>
       </c>
       <c r="O40" t="n">
         <v>0</v>
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
+          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
@@ -3899,11 +3899,11 @@
         </is>
       </c>
       <c r="R40" t="n">
-        <v>4614</v>
+        <v>4613</v>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T40" t="n">
@@ -3916,18 +3916,18 @@
       </c>
       <c r="V40" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
+          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
         </is>
       </c>
       <c r="W40" t="inlineStr">
         <is>
-          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
+          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B41" t="n">
         <v>1220</v>
@@ -3941,43 +3941,43 @@
         <v>3</v>
       </c>
       <c r="E41" t="n">
-        <v>5511</v>
+        <v>5401</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
+          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>11026</v>
+        <v>9408</v>
       </c>
       <c r="H41" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I41" t="n">
-        <v>512</v>
+        <v>752</v>
       </c>
       <c r="J41" t="n">
-        <v>21</v>
+        <v>72</v>
       </c>
       <c r="K41" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L41" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="M41" t="n">
-        <v>8012</v>
+        <v>3003</v>
       </c>
       <c r="N41" t="n">
-        <v>45000000</v>
+        <v>233275000</v>
       </c>
       <c r="O41" t="n">
         <v>0</v>
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
@@ -3986,11 +3986,11 @@
         </is>
       </c>
       <c r="R41" t="n">
-        <v>4613</v>
+        <v>4614</v>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T41" t="n">
@@ -4003,155 +4003,155 @@
       </c>
       <c r="V41" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="W41" t="inlineStr">
         <is>
-          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
+          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B42" t="n">
-        <v>1300</v>
+        <v>1220</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA, MOBILIDADE E PARCERIA - SEINFRA</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D42" t="n">
         <v>3</v>
       </c>
       <c r="E42" t="n">
-        <v>5261</v>
+        <v>5511</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>TREM METROPOLITANO DE BELO HORIZONTE S.A - TREM METROPOLITANO</t>
+          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
         </is>
       </c>
       <c r="G42" t="n">
-        <v>9927</v>
+        <v>11024</v>
       </c>
       <c r="H42" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="I42" t="n">
-        <v>783</v>
+        <v>512</v>
       </c>
       <c r="J42" t="n">
-        <v>705</v>
+        <v>21</v>
       </c>
       <c r="K42" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L42" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M42" t="n">
-        <v>8011</v>
+        <v>6012</v>
       </c>
       <c r="N42" t="n">
-        <v>1000</v>
+        <v>2500000</v>
       </c>
       <c r="O42" t="n">
         <v>0</v>
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R42" t="n">
-        <v>4511</v>
+        <v>4614</v>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T42" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V42" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
         </is>
       </c>
       <c r="W42" t="inlineStr">
         <is>
-          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B43" t="n">
-        <v>1500</v>
+        <v>1220</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D43" t="n">
         <v>3</v>
       </c>
       <c r="E43" t="n">
-        <v>5141</v>
+        <v>5511</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
         </is>
       </c>
       <c r="G43" t="n">
-        <v>10882</v>
+        <v>11026</v>
       </c>
       <c r="H43" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I43" t="n">
-        <v>126</v>
+        <v>512</v>
       </c>
       <c r="J43" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="K43" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L43" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="M43" t="n">
-        <v>6006</v>
+        <v>8012</v>
       </c>
       <c r="N43" t="n">
-        <v>13233200</v>
+        <v>10000000</v>
       </c>
       <c r="O43" t="n">
         <v>0</v>
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
@@ -4160,11 +4160,11 @@
         </is>
       </c>
       <c r="R43" t="n">
-        <v>4613</v>
+        <v>4611</v>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>TERRENOS</t>
         </is>
       </c>
       <c r="T43" t="n">
@@ -4177,81 +4177,81 @@
       </c>
       <c r="V43" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
         </is>
       </c>
       <c r="W43" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B44" t="n">
-        <v>1500</v>
+        <v>1220</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D44" t="n">
         <v>3</v>
       </c>
       <c r="E44" t="n">
-        <v>5141</v>
+        <v>5511</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
         </is>
       </c>
       <c r="G44" t="n">
-        <v>9116</v>
+        <v>11026</v>
       </c>
       <c r="H44" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I44" t="n">
-        <v>126</v>
+        <v>512</v>
       </c>
       <c r="J44" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="K44" t="n">
         <v>8</v>
       </c>
       <c r="L44" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="M44" t="n">
-        <v>8001</v>
+        <v>8012</v>
       </c>
       <c r="N44" t="n">
-        <v>38099783</v>
+        <v>30000000</v>
       </c>
       <c r="O44" t="n">
         <v>0</v>
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R44" t="n">
-        <v>4817</v>
+        <v>4613</v>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>EQUIPAMENTOS E SOFTWARE</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T44" t="n">
@@ -4264,10 +4264,358 @@
       </c>
       <c r="V44" t="inlineStr">
         <is>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B45" t="n">
+        <v>1220</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>3</v>
+      </c>
+      <c r="E45" t="n">
+        <v>5511</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>11026</v>
+      </c>
+      <c r="H45" t="n">
+        <v>17</v>
+      </c>
+      <c r="I45" t="n">
+        <v>512</v>
+      </c>
+      <c r="J45" t="n">
+        <v>21</v>
+      </c>
+      <c r="K45" t="n">
+        <v>8</v>
+      </c>
+      <c r="L45" t="n">
+        <v>12</v>
+      </c>
+      <c r="M45" t="n">
+        <v>8012</v>
+      </c>
+      <c r="N45" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>4610 - IMOBILIZAÇÕES</t>
+        </is>
+      </c>
+      <c r="R45" t="n">
+        <v>4614</v>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+        </is>
+      </c>
+      <c r="T45" t="n">
+        <v>51000</v>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>RECURSOS PRÓPRIOS</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B46" t="n">
+        <v>1300</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA, MOBILIDADE E PARCERIA - SEINFRA</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>3</v>
+      </c>
+      <c r="E46" t="n">
+        <v>5261</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>TREM METROPOLITANO DE BELO HORIZONTE S.A - TREM METROPOLITANO</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>9927</v>
+      </c>
+      <c r="H46" t="n">
+        <v>26</v>
+      </c>
+      <c r="I46" t="n">
+        <v>783</v>
+      </c>
+      <c r="J46" t="n">
+        <v>705</v>
+      </c>
+      <c r="K46" t="n">
+        <v>8</v>
+      </c>
+      <c r="L46" t="n">
+        <v>11</v>
+      </c>
+      <c r="M46" t="n">
+        <v>8011</v>
+      </c>
+      <c r="N46" t="n">
+        <v>1000</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+        </is>
+      </c>
+      <c r="R46" t="n">
+        <v>4511</v>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>SOCIEDADES CONTROLADAS</t>
+        </is>
+      </c>
+      <c r="T46" t="n">
+        <v>11101</v>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B47" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>3</v>
+      </c>
+      <c r="E47" t="n">
+        <v>5141</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>10882</v>
+      </c>
+      <c r="H47" t="n">
+        <v>4</v>
+      </c>
+      <c r="I47" t="n">
+        <v>126</v>
+      </c>
+      <c r="J47" t="n">
+        <v>30</v>
+      </c>
+      <c r="K47" t="n">
+        <v>6</v>
+      </c>
+      <c r="L47" t="n">
+        <v>6</v>
+      </c>
+      <c r="M47" t="n">
+        <v>6006</v>
+      </c>
+      <c r="N47" t="n">
+        <v>23614000</v>
+      </c>
+      <c r="O47" t="n">
+        <v>0</v>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>4610 - IMOBILIZAÇÕES</t>
+        </is>
+      </c>
+      <c r="R47" t="n">
+        <v>4613</v>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>OBRAS E INSTALAÇÕES</t>
+        </is>
+      </c>
+      <c r="T47" t="n">
+        <v>51000</v>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>RECURSOS PRÓPRIOS</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B48" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" t="n">
+        <v>5141</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>9116</v>
+      </c>
+      <c r="H48" t="n">
+        <v>4</v>
+      </c>
+      <c r="I48" t="n">
+        <v>126</v>
+      </c>
+      <c r="J48" t="n">
+        <v>30</v>
+      </c>
+      <c r="K48" t="n">
+        <v>8</v>
+      </c>
+      <c r="L48" t="n">
+        <v>1</v>
+      </c>
+      <c r="M48" t="n">
+        <v>8001</v>
+      </c>
+      <c r="N48" t="n">
+        <v>20445642</v>
+      </c>
+      <c r="O48" t="n">
+        <v>0</v>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
           <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
         </is>
       </c>
-      <c r="W44" t="inlineStr">
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
+        </is>
+      </c>
+      <c r="R48" t="n">
+        <v>4817</v>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
+        </is>
+      </c>
+      <c r="T48" t="n">
+        <v>51000</v>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>RECURSOS PRÓPRIOS</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
         <is>
           <t>SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
         </is>

</xml_diff>

<commit_message>
(dev) - gerando volumes ploa-2026
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_QDD_INVESTIMENTO.xlsx
+++ b/bancos/SISOR/BASE_QDD_INVESTIMENTO.xlsx
@@ -534,7 +534,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B2" t="n">
         <v>1220</v>
@@ -621,7 +621,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B3" t="n">
         <v>1220</v>
@@ -664,7 +664,7 @@
         <v>3015</v>
       </c>
       <c r="N3" t="n">
-        <v>6380000</v>
+        <v>3500000</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -708,7 +708,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B4" t="n">
         <v>1220</v>
@@ -751,7 +751,7 @@
         <v>3015</v>
       </c>
       <c r="N4" t="n">
-        <v>6240000</v>
+        <v>4655000</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
@@ -795,7 +795,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B5" t="n">
         <v>1220</v>
@@ -882,7 +882,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B6" t="n">
         <v>1220</v>
@@ -904,35 +904,35 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>11021</v>
+        <v>11280</v>
       </c>
       <c r="H6" t="n">
         <v>17</v>
       </c>
       <c r="I6" t="n">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="J6" t="n">
-        <v>21</v>
+        <v>101</v>
       </c>
       <c r="K6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="M6" t="n">
-        <v>6009</v>
+        <v>3012</v>
       </c>
       <c r="N6" t="n">
-        <v>50000000</v>
+        <v>5000000</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
+          <t>DOAÇÃO DE MÓDULOS DE FOSSAS SÉPTICAS PARA MUNICÍPIOS SEM CONCESSÃO COPASA (CONVÊNIO DEFESA CIVIL)</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -949,27 +949,27 @@
         </is>
       </c>
       <c r="T6" t="n">
-        <v>22199</v>
+        <v>51000</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
+          <t>DOAÇÃO DE MÓDULOS DE FOSSAS SÉPTICAS PARA MUNICÍPIOS SEM CONCESSÃO COPASA (CONVÊNIO DEFESA CIVIL)</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
+          <t>PROGRAMA ENCONTRO DAS ÁGUAS</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B7" t="n">
         <v>1220</v>
@@ -1036,11 +1036,11 @@
         </is>
       </c>
       <c r="T7" t="n">
-        <v>51000</v>
+        <v>22199</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1056,7 +1056,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B8" t="n">
         <v>1220</v>
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>11022</v>
+        <v>11021</v>
       </c>
       <c r="H8" t="n">
         <v>17</v>
@@ -1090,23 +1090,23 @@
         <v>21</v>
       </c>
       <c r="K8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M8" t="n">
-        <v>8008</v>
+        <v>6009</v>
       </c>
       <c r="N8" t="n">
-        <v>100000000</v>
+        <v>50000000</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
+          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1115,11 +1115,11 @@
         </is>
       </c>
       <c r="R8" t="n">
-        <v>4611</v>
+        <v>4614</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>TERRENOS</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T8" t="n">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
+          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
@@ -1143,7 +1143,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B9" t="n">
         <v>1220</v>
@@ -1186,7 +1186,7 @@
         <v>8008</v>
       </c>
       <c r="N9" t="n">
-        <v>350000000</v>
+        <v>95000000</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
@@ -1202,19 +1202,19 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>4613</v>
+        <v>4611</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>TERRENOS</t>
         </is>
       </c>
       <c r="T9" t="n">
-        <v>21204</v>
+        <v>51000</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>OP CRÉD CONTRAT EXTERNA - KFW</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1230,7 +1230,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B10" t="n">
         <v>1220</v>
@@ -1273,7 +1273,7 @@
         <v>8008</v>
       </c>
       <c r="N10" t="n">
-        <v>983250000</v>
+        <v>350000000</v>
       </c>
       <c r="O10" t="n">
         <v>0</v>
@@ -1297,11 +1297,11 @@
         </is>
       </c>
       <c r="T10" t="n">
-        <v>22199</v>
+        <v>21204</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
+          <t>OP CRÉD CONTRAT EXTERNA - KFW</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1317,7 +1317,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B11" t="n">
         <v>1220</v>
@@ -1360,7 +1360,7 @@
         <v>8008</v>
       </c>
       <c r="N11" t="n">
-        <v>54750000</v>
+        <v>2510000000</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
@@ -1384,11 +1384,11 @@
         </is>
       </c>
       <c r="T11" t="n">
-        <v>51000</v>
+        <v>22199</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -1404,7 +1404,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B12" t="n">
         <v>1220</v>
@@ -1447,7 +1447,7 @@
         <v>8008</v>
       </c>
       <c r="N12" t="n">
-        <v>40000000</v>
+        <v>100000000</v>
       </c>
       <c r="O12" t="n">
         <v>0</v>
@@ -1463,19 +1463,19 @@
         </is>
       </c>
       <c r="R12" t="n">
-        <v>4614</v>
+        <v>4613</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T12" t="n">
-        <v>22199</v>
+        <v>51000</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
@@ -1491,7 +1491,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B13" t="n">
         <v>1220</v>
@@ -1513,7 +1513,7 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>11023</v>
+        <v>11022</v>
       </c>
       <c r="H13" t="n">
         <v>17</v>
@@ -1528,20 +1528,20 @@
         <v>8</v>
       </c>
       <c r="L13" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M13" t="n">
-        <v>8009</v>
+        <v>8008</v>
       </c>
       <c r="N13" t="n">
-        <v>48428689</v>
+        <v>40000000</v>
       </c>
       <c r="O13" t="n">
         <v>0</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>PPP SISTEMA ADUTOR RIO MANSO</t>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -1550,24 +1550,24 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>4613</v>
+        <v>4614</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T13" t="n">
-        <v>51000</v>
+        <v>22199</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OP CRÉD A CONTRATAR INTERNA - OUTRAS</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>PPP SISTEMA ADUTOR RIO MANSO</t>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
@@ -1578,7 +1578,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B14" t="n">
         <v>1220</v>
@@ -1592,56 +1592,56 @@
         <v>3</v>
       </c>
       <c r="E14" t="n">
-        <v>5121</v>
+        <v>5081</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>COMPANHIA ENERGÉTICA DE MINAS GERAIS - CEMIG HOLDING</t>
+          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>10542</v>
+        <v>11023</v>
       </c>
       <c r="H14" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="I14" t="n">
-        <v>752</v>
+        <v>512</v>
       </c>
       <c r="J14" t="n">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="K14" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L14" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="M14" t="n">
-        <v>3010</v>
+        <v>8009</v>
       </c>
       <c r="N14" t="n">
-        <v>259985809</v>
+        <v>55500000</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
+          <t>PPP SISTEMA ADUTOR RIO MANSO</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R14" t="n">
-        <v>4511</v>
+        <v>4613</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T14" t="n">
@@ -1654,18 +1654,18 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
+          <t>PPP SISTEMA ADUTOR RIO MANSO</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS CEMIG</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B15" t="n">
         <v>1220</v>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>9994</v>
+        <v>10542</v>
       </c>
       <c r="H15" t="n">
         <v>25</v>
@@ -1702,33 +1702,33 @@
         <v>3</v>
       </c>
       <c r="L15" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="M15" t="n">
-        <v>3011</v>
+        <v>3010</v>
       </c>
       <c r="N15" t="n">
-        <v>4440000</v>
+        <v>70784312</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R15" t="n">
-        <v>4614</v>
+        <v>4511</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T15" t="n">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
@@ -1752,7 +1752,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B16" t="n">
         <v>1220</v>
@@ -1766,43 +1766,43 @@
         <v>3</v>
       </c>
       <c r="E16" t="n">
-        <v>5131</v>
+        <v>5121</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>AGÊNCIA DE PROMOÇÃO DE INVESTIMENTOS DE MINAS GERAIS - INVEST MINAS</t>
+          <t>COMPANHIA ENERGÉTICA DE MINAS GERAIS - CEMIG HOLDING</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>9723</v>
+        <v>9994</v>
       </c>
       <c r="H16" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I16" t="n">
-        <v>122</v>
+        <v>752</v>
       </c>
       <c r="J16" t="n">
-        <v>142</v>
+        <v>35</v>
       </c>
       <c r="K16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L16" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="M16" t="n">
-        <v>6008</v>
+        <v>3011</v>
       </c>
       <c r="N16" t="n">
-        <v>500000</v>
+        <v>2347000</v>
       </c>
       <c r="O16" t="n">
         <v>0</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1828,18 +1828,18 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL - INVEST MINAS</t>
+          <t>INVESTIMENTOS CEMIG</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B17" t="n">
         <v>1220</v>
@@ -1853,56 +1853,56 @@
         <v>3</v>
       </c>
       <c r="E17" t="n">
-        <v>5191</v>
+        <v>5131</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
+          <t>AGÊNCIA DE PROMOÇÃO DE INVESTIMENTOS DE MINAS GERAIS - INVEST MINAS</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>9796</v>
+        <v>9723</v>
       </c>
       <c r="H17" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="I17" t="n">
         <v>122</v>
       </c>
       <c r="J17" t="n">
-        <v>13</v>
+        <v>142</v>
       </c>
       <c r="K17" t="n">
         <v>6</v>
       </c>
       <c r="L17" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="M17" t="n">
-        <v>6011</v>
+        <v>6008</v>
       </c>
       <c r="N17" t="n">
-        <v>243000</v>
+        <v>250000</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R17" t="n">
-        <v>4817</v>
+        <v>4614</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>EQUIPAMENTOS E SOFTWARE</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T17" t="n">
@@ -1915,18 +1915,18 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL - INVEST MINAS</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B18" t="n">
         <v>1220</v>
@@ -1948,7 +1948,7 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>11036</v>
+        <v>9796</v>
       </c>
       <c r="H18" t="n">
         <v>4</v>
@@ -1957,26 +1957,26 @@
         <v>122</v>
       </c>
       <c r="J18" t="n">
-        <v>119</v>
+        <v>13</v>
       </c>
       <c r="K18" t="n">
         <v>6</v>
       </c>
       <c r="L18" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="M18" t="n">
-        <v>6003</v>
+        <v>6011</v>
       </c>
       <c r="N18" t="n">
-        <v>1000</v>
+        <v>240000</v>
       </c>
       <c r="O18" t="n">
         <v>0</v>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -1985,35 +1985,35 @@
         </is>
       </c>
       <c r="R18" t="n">
-        <v>4819</v>
+        <v>4817</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
         </is>
       </c>
       <c r="T18" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>APOIO AO DESENVOLVIMENTO MUNICIPAL E À COORDENAÇÃO DAS TRANSFERÊNCIAS ESTADUAIS DE RECURSOS FINANCEIROS</t>
+          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B19" t="n">
         <v>1220</v>
@@ -2056,7 +2056,7 @@
         <v>6003</v>
       </c>
       <c r="N19" t="n">
-        <v>9256395</v>
+        <v>1000</v>
       </c>
       <c r="O19" t="n">
         <v>0</v>
@@ -2080,11 +2080,11 @@
         </is>
       </c>
       <c r="T19" t="n">
-        <v>51000</v>
+        <v>11101</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
@@ -2100,7 +2100,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B20" t="n">
         <v>1220</v>
@@ -2122,72 +2122,72 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>9058</v>
+        <v>11036</v>
       </c>
       <c r="H20" t="n">
         <v>4</v>
       </c>
       <c r="I20" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J20" t="n">
-        <v>13</v>
+        <v>119</v>
       </c>
       <c r="K20" t="n">
         <v>6</v>
       </c>
       <c r="L20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M20" t="n">
-        <v>6001</v>
+        <v>6003</v>
       </c>
       <c r="N20" t="n">
-        <v>1000</v>
+        <v>1461000</v>
       </c>
       <c r="O20" t="n">
         <v>0</v>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R20" t="n">
-        <v>4511</v>
+        <v>4819</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T20" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
+          <t>APOIO AO DESENVOLVIMENTO MUNICIPAL E À COORDENAÇÃO DAS TRANSFERÊNCIAS ESTADUAIS DE RECURSOS FINANCEIROS</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B21" t="n">
         <v>1220</v>
@@ -2254,11 +2254,11 @@
         </is>
       </c>
       <c r="T21" t="n">
-        <v>51000</v>
+        <v>11101</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
@@ -2274,7 +2274,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B22" t="n">
         <v>1220</v>
@@ -2288,80 +2288,80 @@
         <v>3</v>
       </c>
       <c r="E22" t="n">
-        <v>5201</v>
+        <v>5191</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
+          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>9087</v>
+        <v>9058</v>
       </c>
       <c r="H22" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="I22" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J22" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="K22" t="n">
         <v>6</v>
       </c>
       <c r="L22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>6004</v>
+        <v>6001</v>
       </c>
       <c r="N22" t="n">
-        <v>26253389</v>
+        <v>1000</v>
       </c>
       <c r="O22" t="n">
         <v>0</v>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
+          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R22" t="n">
-        <v>4813</v>
+        <v>4511</v>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>INTANGÍVEIS E OUTROS INVESTIMENTOS</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T22" t="n">
-        <v>12400</v>
+        <v>51000</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>OUTRAS ENTIDADES - BDMG</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
+          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>INVESTIMENTO NA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
+          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B23" t="n">
         <v>1220</v>
@@ -2383,35 +2383,35 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>11046</v>
+        <v>9087</v>
       </c>
       <c r="H23" t="n">
         <v>23</v>
       </c>
       <c r="I23" t="n">
-        <v>694</v>
+        <v>122</v>
       </c>
       <c r="J23" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="K23" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M23" t="n">
-        <v>8003</v>
+        <v>6004</v>
       </c>
       <c r="N23" t="n">
-        <v>250000000</v>
+        <v>30022403</v>
       </c>
       <c r="O23" t="n">
         <v>0</v>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -2420,11 +2420,11 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>4819</v>
+        <v>4813</v>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>INTANGÍVEIS E OUTROS INVESTIMENTOS</t>
         </is>
       </c>
       <c r="T23" t="n">
@@ -2437,18 +2437,18 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
+          <t>INVESTIMENTO NA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B24" t="n">
         <v>1220</v>
@@ -2470,7 +2470,7 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>10991</v>
+        <v>11046</v>
       </c>
       <c r="H24" t="n">
         <v>23</v>
@@ -2479,26 +2479,26 @@
         <v>694</v>
       </c>
       <c r="J24" t="n">
-        <v>171</v>
+        <v>14</v>
       </c>
       <c r="K24" t="n">
         <v>8</v>
       </c>
       <c r="L24" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M24" t="n">
-        <v>8006</v>
+        <v>8003</v>
       </c>
       <c r="N24" t="n">
-        <v>600000000</v>
+        <v>250000000</v>
       </c>
       <c r="O24" t="n">
         <v>0</v>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
+          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -2524,18 +2524,18 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
+          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
+          <t>FINANCIAMENTO À DESCARBONIZAÇÃO E RESILIÊNCIA CLIMÁTICA ENTRE BDMG E BANCO INTERAMERICANO DE DESENVOLVIMENTO (BDMG PBR)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B25" t="n">
         <v>1220</v>
@@ -2549,80 +2549,80 @@
         <v>3</v>
       </c>
       <c r="E25" t="n">
-        <v>5251</v>
+        <v>5201</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>COMPANHIA DE GÁS DE MINAS GERAIS - GASMIG</t>
+          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>11027</v>
+        <v>11249</v>
       </c>
       <c r="H25" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I25" t="n">
-        <v>121</v>
+        <v>694</v>
       </c>
       <c r="J25" t="n">
-        <v>133</v>
+        <v>107</v>
       </c>
       <c r="K25" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L25" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="M25" t="n">
-        <v>3018</v>
+        <v>8004</v>
       </c>
       <c r="N25" t="n">
-        <v>285487805</v>
+        <v>500000000</v>
       </c>
       <c r="O25" t="n">
         <v>0</v>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
+          <t>FINANCIAMENTO À SUSTENTABILIDADE E ÀS MICRO E PEQUENAS EMPRESAS DO ESTADO DE MINAS GERAIS ENTRE BDMG E BANCO EUROPEU DE INVESTIMENTO (BDMG SUSTENTABILIDADE E MPE)</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R25" t="n">
-        <v>4613</v>
+        <v>4819</v>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T25" t="n">
-        <v>61000</v>
+        <v>12400</v>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>OUTRAS ORIGENS</t>
+          <t>OUTRAS ENTIDADES - BDMG</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
+          <t>FINANCIAMENTO À SUSTENTABILIDADE E ÀS MICRO E PEQUENAS EMPRESAS DO ESTADO DE MINAS GERAIS ENTRE BDMG E BANCO EUROPEU DE INVESTIMENTO (BDMG SUSTENTABILIDADE E MPE)</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>MINAS GERAÇÃO DE VALOR</t>
+          <t>FINANCIAMENTO À SUSTENTABILIDADE E ÀS MICRO E PEQUENAS EMPRESAS DO ESTADO DE MINAS GERAIS ENTRE BDMG E BANCO EUROPEU DE INVESTIMENTO (BDMG SUSTENTABILIDADE E MPE)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B26" t="n">
         <v>1220</v>
@@ -2636,80 +2636,80 @@
         <v>3</v>
       </c>
       <c r="E26" t="n">
-        <v>5381</v>
+        <v>5201</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
+          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>9239</v>
+        <v>10991</v>
       </c>
       <c r="H26" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="I26" t="n">
-        <v>122</v>
+        <v>694</v>
       </c>
       <c r="J26" t="n">
-        <v>57</v>
+        <v>171</v>
       </c>
       <c r="K26" t="n">
         <v>8</v>
       </c>
       <c r="L26" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M26" t="n">
-        <v>8002</v>
+        <v>8006</v>
       </c>
       <c r="N26" t="n">
-        <v>5450000</v>
+        <v>600000000</v>
       </c>
       <c r="O26" t="n">
         <v>0</v>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R26" t="n">
-        <v>4614</v>
+        <v>4819</v>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T26" t="n">
-        <v>51000</v>
+        <v>12400</v>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>OUTRAS ENTIDADES - BDMG</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
+          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B27" t="n">
         <v>1220</v>
@@ -2723,56 +2723,56 @@
         <v>3</v>
       </c>
       <c r="E27" t="n">
-        <v>5381</v>
+        <v>5251</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
+          <t>COMPANHIA DE GÁS DE MINAS GERAIS - GASMIG</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>9239</v>
+        <v>11027</v>
       </c>
       <c r="H27" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="I27" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="J27" t="n">
-        <v>57</v>
+        <v>133</v>
       </c>
       <c r="K27" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L27" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="M27" t="n">
-        <v>8002</v>
+        <v>3018</v>
       </c>
       <c r="N27" t="n">
-        <v>400000</v>
+        <v>191687487</v>
       </c>
       <c r="O27" t="n">
         <v>0</v>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R27" t="n">
-        <v>4615</v>
+        <v>4819</v>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>MÓVEIS E UTENSÍLIOS</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T27" t="n">
@@ -2785,18 +2785,18 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
         </is>
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
+          <t>MINAS GERAÇÃO DE VALOR</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B28" t="n">
         <v>1220</v>
@@ -2839,7 +2839,7 @@
         <v>8002</v>
       </c>
       <c r="N28" t="n">
-        <v>4000000</v>
+        <v>9152200</v>
       </c>
       <c r="O28" t="n">
         <v>0</v>
@@ -2851,15 +2851,15 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R28" t="n">
-        <v>4817</v>
+        <v>4614</v>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>EQUIPAMENTOS E SOFTWARE</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T28" t="n">
@@ -2883,7 +2883,7 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B29" t="n">
         <v>1220</v>
@@ -2926,7 +2926,7 @@
         <v>8002</v>
       </c>
       <c r="N29" t="n">
-        <v>1000</v>
+        <v>522300</v>
       </c>
       <c r="O29" t="n">
         <v>0</v>
@@ -2938,23 +2938,23 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R29" t="n">
-        <v>4819</v>
+        <v>4615</v>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>OUTRAS APLICAÇÕES</t>
+          <t>MÓVEIS E UTENSÍLIOS</t>
         </is>
       </c>
       <c r="T29" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
@@ -2970,7 +2970,7 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B30" t="n">
         <v>1220</v>
@@ -2984,56 +2984,56 @@
         <v>3</v>
       </c>
       <c r="E30" t="n">
-        <v>5391</v>
+        <v>5381</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>9420</v>
+        <v>9239</v>
       </c>
       <c r="H30" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I30" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J30" t="n">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="K30" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L30" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M30" t="n">
-        <v>3004</v>
+        <v>8002</v>
       </c>
       <c r="N30" t="n">
-        <v>231539977</v>
+        <v>12880000</v>
       </c>
       <c r="O30" t="n">
         <v>0</v>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R30" t="n">
-        <v>4613</v>
+        <v>4817</v>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
         </is>
       </c>
       <c r="T30" t="n">
@@ -3046,18 +3046,18 @@
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
+          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B31" t="n">
         <v>1220</v>
@@ -3071,80 +3071,80 @@
         <v>3</v>
       </c>
       <c r="E31" t="n">
-        <v>5391</v>
+        <v>5381</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>9421</v>
+        <v>9239</v>
       </c>
       <c r="H31" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I31" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J31" t="n">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="K31" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L31" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M31" t="n">
-        <v>3005</v>
+        <v>8002</v>
       </c>
       <c r="N31" t="n">
-        <v>216613767</v>
+        <v>1000</v>
       </c>
       <c r="O31" t="n">
         <v>0</v>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R31" t="n">
-        <v>4613</v>
+        <v>4819</v>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="T31" t="n">
-        <v>51000</v>
+        <v>11101</v>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
+          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B32" t="n">
         <v>1220</v>
@@ -3166,7 +3166,7 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>9430</v>
+        <v>9420</v>
       </c>
       <c r="H32" t="n">
         <v>25</v>
@@ -3181,20 +3181,20 @@
         <v>3</v>
       </c>
       <c r="L32" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M32" t="n">
-        <v>3006</v>
+        <v>3004</v>
       </c>
       <c r="N32" t="n">
-        <v>42479000</v>
+        <v>343756125</v>
       </c>
       <c r="O32" t="n">
         <v>0</v>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
+          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -3203,11 +3203,11 @@
         </is>
       </c>
       <c r="R32" t="n">
-        <v>4614</v>
+        <v>4613</v>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T32" t="n">
@@ -3220,7 +3220,7 @@
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
+          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W32" t="inlineStr">
@@ -3231,7 +3231,7 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B33" t="n">
         <v>1220</v>
@@ -3253,7 +3253,7 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>11134</v>
+        <v>9421</v>
       </c>
       <c r="H33" t="n">
         <v>25</v>
@@ -3268,33 +3268,33 @@
         <v>3</v>
       </c>
       <c r="L33" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="M33" t="n">
-        <v>3009</v>
+        <v>3005</v>
       </c>
       <c r="N33" t="n">
-        <v>92271447</v>
+        <v>285714873</v>
       </c>
       <c r="O33" t="n">
         <v>0</v>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS PARTICIPAÇÕES SOCIETÁRIAS DA TRANSMISSÃO</t>
+          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R33" t="n">
-        <v>4511</v>
+        <v>4613</v>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T33" t="n">
@@ -3307,7 +3307,7 @@
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS PARTICIPAÇÕES SOCIETÁRIAS DA TRANSMISSÃO</t>
+          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W33" t="inlineStr">
@@ -3318,7 +3318,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B34" t="n">
         <v>1220</v>
@@ -3340,7 +3340,7 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>10062</v>
+        <v>9430</v>
       </c>
       <c r="H34" t="n">
         <v>25</v>
@@ -3349,26 +3349,26 @@
         <v>752</v>
       </c>
       <c r="J34" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="K34" t="n">
         <v>3</v>
       </c>
       <c r="L34" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="M34" t="n">
-        <v>3001</v>
+        <v>3006</v>
       </c>
       <c r="N34" t="n">
-        <v>100000</v>
+        <v>65874000</v>
       </c>
       <c r="O34" t="n">
         <v>0</v>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -3377,11 +3377,11 @@
         </is>
       </c>
       <c r="R34" t="n">
-        <v>4613</v>
+        <v>4614</v>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T34" t="n">
@@ -3394,18 +3394,18 @@
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B35" t="n">
         <v>1220</v>
@@ -3427,7 +3427,7 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>9440</v>
+        <v>11134</v>
       </c>
       <c r="H35" t="n">
         <v>25</v>
@@ -3436,39 +3436,39 @@
         <v>752</v>
       </c>
       <c r="J35" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="K35" t="n">
         <v>3</v>
       </c>
       <c r="L35" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M35" t="n">
-        <v>3007</v>
+        <v>3009</v>
       </c>
       <c r="N35" t="n">
-        <v>96218712</v>
+        <v>8146743</v>
       </c>
       <c r="O35" t="n">
         <v>0</v>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
+          <t>INVESTIMENTOS PARTICIPAÇÕES SOCIETÁRIAS DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R35" t="n">
-        <v>4614</v>
+        <v>4511</v>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T35" t="n">
@@ -3481,18 +3481,18 @@
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
+          <t>INVESTIMENTOS PARTICIPAÇÕES SOCIETÁRIAS DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B36" t="n">
         <v>1220</v>
@@ -3514,7 +3514,7 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>9450</v>
+        <v>10062</v>
       </c>
       <c r="H36" t="n">
         <v>25</v>
@@ -3529,20 +3529,20 @@
         <v>3</v>
       </c>
       <c r="L36" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>3008</v>
+        <v>3001</v>
       </c>
       <c r="N36" t="n">
-        <v>18091000</v>
+        <v>1</v>
       </c>
       <c r="O36" t="n">
         <v>0</v>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
+          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -3551,11 +3551,11 @@
         </is>
       </c>
       <c r="R36" t="n">
-        <v>4614</v>
+        <v>4613</v>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T36" t="n">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
+          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
         </is>
       </c>
       <c r="W36" t="inlineStr">
@@ -3579,7 +3579,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B37" t="n">
         <v>1220</v>
@@ -3601,7 +3601,7 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>10677</v>
+        <v>9440</v>
       </c>
       <c r="H37" t="n">
         <v>25</v>
@@ -3616,33 +3616,33 @@
         <v>3</v>
       </c>
       <c r="L37" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="M37" t="n">
-        <v>3014</v>
+        <v>3007</v>
       </c>
       <c r="N37" t="n">
-        <v>190392082</v>
+        <v>65661789</v>
       </c>
       <c r="O37" t="n">
         <v>0</v>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS DA GERAÇÃO</t>
+          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R37" t="n">
-        <v>4511</v>
+        <v>4614</v>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T37" t="n">
@@ -3655,7 +3655,7 @@
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS DA GERAÇÃO</t>
+          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
         </is>
       </c>
       <c r="W37" t="inlineStr">
@@ -3666,7 +3666,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B38" t="n">
         <v>1220</v>
@@ -3680,15 +3680,15 @@
         <v>3</v>
       </c>
       <c r="E38" t="n">
-        <v>5401</v>
+        <v>5391</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>9332</v>
+        <v>9450</v>
       </c>
       <c r="H38" t="n">
         <v>25</v>
@@ -3697,26 +3697,26 @@
         <v>752</v>
       </c>
       <c r="J38" t="n">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="K38" t="n">
         <v>3</v>
       </c>
       <c r="L38" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="M38" t="n">
-        <v>3002</v>
+        <v>3008</v>
       </c>
       <c r="N38" t="n">
-        <v>4721877188</v>
+        <v>42279000</v>
       </c>
       <c r="O38" t="n">
         <v>0</v>
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
@@ -3725,11 +3725,11 @@
         </is>
       </c>
       <c r="R38" t="n">
-        <v>4613</v>
+        <v>4614</v>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T38" t="n">
@@ -3742,18 +3742,18 @@
       </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
         </is>
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B39" t="n">
         <v>1220</v>
@@ -3767,15 +3767,15 @@
         <v>3</v>
       </c>
       <c r="E39" t="n">
-        <v>5401</v>
+        <v>5391</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="G39" t="n">
-        <v>9408</v>
+        <v>10677</v>
       </c>
       <c r="H39" t="n">
         <v>25</v>
@@ -3784,39 +3784,39 @@
         <v>752</v>
       </c>
       <c r="J39" t="n">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="K39" t="n">
         <v>3</v>
       </c>
       <c r="L39" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="M39" t="n">
-        <v>3003</v>
+        <v>3014</v>
       </c>
       <c r="N39" t="n">
-        <v>247976000</v>
+        <v>116689303</v>
       </c>
       <c r="O39" t="n">
         <v>0</v>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS DA GERAÇÃO</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R39" t="n">
-        <v>4614</v>
+        <v>4511</v>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>SOCIEDADES CONTROLADAS</t>
         </is>
       </c>
       <c r="T39" t="n">
@@ -3829,18 +3829,18 @@
       </c>
       <c r="V39" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS DA GERAÇÃO</t>
         </is>
       </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
+          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B40" t="n">
         <v>1220</v>
@@ -3854,43 +3854,43 @@
         <v>3</v>
       </c>
       <c r="E40" t="n">
-        <v>5511</v>
+        <v>5401</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
+          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>11024</v>
+        <v>9332</v>
       </c>
       <c r="H40" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I40" t="n">
-        <v>512</v>
+        <v>752</v>
       </c>
       <c r="J40" t="n">
-        <v>21</v>
+        <v>72</v>
       </c>
       <c r="K40" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L40" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="M40" t="n">
-        <v>6012</v>
+        <v>3002</v>
       </c>
       <c r="N40" t="n">
-        <v>2000000</v>
+        <v>5072587386</v>
       </c>
       <c r="O40" t="n">
         <v>0</v>
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
+          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
@@ -3899,11 +3899,11 @@
         </is>
       </c>
       <c r="R40" t="n">
-        <v>4614</v>
+        <v>4613</v>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T40" t="n">
@@ -3916,18 +3916,18 @@
       </c>
       <c r="V40" t="inlineStr">
         <is>
-          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
+          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
         </is>
       </c>
       <c r="W40" t="inlineStr">
         <is>
-          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
+          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B41" t="n">
         <v>1220</v>
@@ -3941,43 +3941,43 @@
         <v>3</v>
       </c>
       <c r="E41" t="n">
-        <v>5511</v>
+        <v>5401</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
+          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>11026</v>
+        <v>9408</v>
       </c>
       <c r="H41" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I41" t="n">
-        <v>512</v>
+        <v>752</v>
       </c>
       <c r="J41" t="n">
-        <v>21</v>
+        <v>72</v>
       </c>
       <c r="K41" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L41" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="M41" t="n">
-        <v>8012</v>
+        <v>3003</v>
       </c>
       <c r="N41" t="n">
-        <v>45000000</v>
+        <v>233275000</v>
       </c>
       <c r="O41" t="n">
         <v>0</v>
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
@@ -3986,11 +3986,11 @@
         </is>
       </c>
       <c r="R41" t="n">
-        <v>4613</v>
+        <v>4614</v>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T41" t="n">
@@ -4003,155 +4003,155 @@
       </c>
       <c r="V41" t="inlineStr">
         <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="W41" t="inlineStr">
         <is>
-          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
+          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B42" t="n">
-        <v>1300</v>
+        <v>1220</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA, MOBILIDADE E PARCERIA - SEINFRA</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D42" t="n">
         <v>3</v>
       </c>
       <c r="E42" t="n">
-        <v>5261</v>
+        <v>5511</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>TREM METROPOLITANO DE BELO HORIZONTE S.A - TREM METROPOLITANO</t>
+          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
         </is>
       </c>
       <c r="G42" t="n">
-        <v>9927</v>
+        <v>11024</v>
       </c>
       <c r="H42" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="I42" t="n">
-        <v>783</v>
+        <v>512</v>
       </c>
       <c r="J42" t="n">
-        <v>705</v>
+        <v>21</v>
       </c>
       <c r="K42" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L42" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M42" t="n">
-        <v>8011</v>
+        <v>6012</v>
       </c>
       <c r="N42" t="n">
-        <v>1000</v>
+        <v>2500000</v>
       </c>
       <c r="O42" t="n">
         <v>0</v>
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R42" t="n">
-        <v>4511</v>
+        <v>4614</v>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>SOCIEDADES CONTROLADAS</t>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
         </is>
       </c>
       <c r="T42" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V42" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
         </is>
       </c>
       <c r="W42" t="inlineStr">
         <is>
-          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B43" t="n">
-        <v>1500</v>
+        <v>1220</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D43" t="n">
         <v>3</v>
       </c>
       <c r="E43" t="n">
-        <v>5141</v>
+        <v>5511</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
         </is>
       </c>
       <c r="G43" t="n">
-        <v>10882</v>
+        <v>11026</v>
       </c>
       <c r="H43" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I43" t="n">
-        <v>126</v>
+        <v>512</v>
       </c>
       <c r="J43" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="K43" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L43" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="M43" t="n">
-        <v>6006</v>
+        <v>8012</v>
       </c>
       <c r="N43" t="n">
-        <v>13233200</v>
+        <v>10000000</v>
       </c>
       <c r="O43" t="n">
         <v>0</v>
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
@@ -4160,11 +4160,11 @@
         </is>
       </c>
       <c r="R43" t="n">
-        <v>4613</v>
+        <v>4611</v>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>OBRAS E INSTALAÇÕES</t>
+          <t>TERRENOS</t>
         </is>
       </c>
       <c r="T43" t="n">
@@ -4177,81 +4177,81 @@
       </c>
       <c r="V43" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
         </is>
       </c>
       <c r="W43" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B44" t="n">
-        <v>1500</v>
+        <v>1220</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
         </is>
       </c>
       <c r="D44" t="n">
         <v>3</v>
       </c>
       <c r="E44" t="n">
-        <v>5141</v>
+        <v>5511</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
         </is>
       </c>
       <c r="G44" t="n">
-        <v>9116</v>
+        <v>11026</v>
       </c>
       <c r="H44" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I44" t="n">
-        <v>126</v>
+        <v>512</v>
       </c>
       <c r="J44" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="K44" t="n">
         <v>8</v>
       </c>
       <c r="L44" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="M44" t="n">
-        <v>8001</v>
+        <v>8012</v>
       </c>
       <c r="N44" t="n">
-        <v>38099783</v>
+        <v>30000000</v>
       </c>
       <c r="O44" t="n">
         <v>0</v>
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R44" t="n">
-        <v>4817</v>
+        <v>4613</v>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>EQUIPAMENTOS E SOFTWARE</t>
+          <t>OBRAS E INSTALAÇÕES</t>
         </is>
       </c>
       <c r="T44" t="n">
@@ -4264,10 +4264,358 @@
       </c>
       <c r="V44" t="inlineStr">
         <is>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B45" t="n">
+        <v>1220</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>3</v>
+      </c>
+      <c r="E45" t="n">
+        <v>5511</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>11026</v>
+      </c>
+      <c r="H45" t="n">
+        <v>17</v>
+      </c>
+      <c r="I45" t="n">
+        <v>512</v>
+      </c>
+      <c r="J45" t="n">
+        <v>21</v>
+      </c>
+      <c r="K45" t="n">
+        <v>8</v>
+      </c>
+      <c r="L45" t="n">
+        <v>12</v>
+      </c>
+      <c r="M45" t="n">
+        <v>8012</v>
+      </c>
+      <c r="N45" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>4610 - IMOBILIZAÇÕES</t>
+        </is>
+      </c>
+      <c r="R45" t="n">
+        <v>4614</v>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+        </is>
+      </c>
+      <c r="T45" t="n">
+        <v>51000</v>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>RECURSOS PRÓPRIOS</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B46" t="n">
+        <v>1300</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA, MOBILIDADE E PARCERIA - SEINFRA</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>3</v>
+      </c>
+      <c r="E46" t="n">
+        <v>5261</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>TREM METROPOLITANO DE BELO HORIZONTE S.A - TREM METROPOLITANO</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>9927</v>
+      </c>
+      <c r="H46" t="n">
+        <v>26</v>
+      </c>
+      <c r="I46" t="n">
+        <v>783</v>
+      </c>
+      <c r="J46" t="n">
+        <v>705</v>
+      </c>
+      <c r="K46" t="n">
+        <v>8</v>
+      </c>
+      <c r="L46" t="n">
+        <v>11</v>
+      </c>
+      <c r="M46" t="n">
+        <v>8011</v>
+      </c>
+      <c r="N46" t="n">
+        <v>1000</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
+        </is>
+      </c>
+      <c r="R46" t="n">
+        <v>4511</v>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>SOCIEDADES CONTROLADAS</t>
+        </is>
+      </c>
+      <c r="T46" t="n">
+        <v>11101</v>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B47" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>3</v>
+      </c>
+      <c r="E47" t="n">
+        <v>5141</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>10882</v>
+      </c>
+      <c r="H47" t="n">
+        <v>4</v>
+      </c>
+      <c r="I47" t="n">
+        <v>126</v>
+      </c>
+      <c r="J47" t="n">
+        <v>30</v>
+      </c>
+      <c r="K47" t="n">
+        <v>6</v>
+      </c>
+      <c r="L47" t="n">
+        <v>6</v>
+      </c>
+      <c r="M47" t="n">
+        <v>6006</v>
+      </c>
+      <c r="N47" t="n">
+        <v>23614000</v>
+      </c>
+      <c r="O47" t="n">
+        <v>0</v>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>4610 - IMOBILIZAÇÕES</t>
+        </is>
+      </c>
+      <c r="R47" t="n">
+        <v>4613</v>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>OBRAS E INSTALAÇÕES</t>
+        </is>
+      </c>
+      <c r="T47" t="n">
+        <v>51000</v>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>RECURSOS PRÓPRIOS</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B48" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" t="n">
+        <v>5141</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>9116</v>
+      </c>
+      <c r="H48" t="n">
+        <v>4</v>
+      </c>
+      <c r="I48" t="n">
+        <v>126</v>
+      </c>
+      <c r="J48" t="n">
+        <v>30</v>
+      </c>
+      <c r="K48" t="n">
+        <v>8</v>
+      </c>
+      <c r="L48" t="n">
+        <v>1</v>
+      </c>
+      <c r="M48" t="n">
+        <v>8001</v>
+      </c>
+      <c r="N48" t="n">
+        <v>20445642</v>
+      </c>
+      <c r="O48" t="n">
+        <v>0</v>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
           <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
         </is>
       </c>
-      <c r="W44" t="inlineStr">
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
+        </is>
+      </c>
+      <c r="R48" t="n">
+        <v>4817</v>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
+        </is>
+      </c>
+      <c r="T48" t="n">
+        <v>51000</v>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>RECURSOS PRÓPRIOS</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
         <is>
           <t>SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
         </is>

</xml_diff>

<commit_message>
atualiza volumes loa com ppo - 09092026
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_QDD_INVESTIMENTO.xlsx
+++ b/bancos/SISOR/BASE_QDD_INVESTIMENTO.xlsx
@@ -592,6 +592,11 @@
       <c r="R2" t="n">
         <v>4613</v>
       </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>OBRAS E INSTALAÇÕES</t>
+        </is>
+      </c>
       <c r="T2" t="n">
         <v>51000</v>
       </c>
@@ -671,6 +676,11 @@
       <c r="R3" t="n">
         <v>4614</v>
       </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+        </is>
+      </c>
       <c r="T3" t="n">
         <v>51000</v>
       </c>
@@ -750,6 +760,11 @@
       <c r="R4" t="n">
         <v>4613</v>
       </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>OBRAS E INSTALAÇÕES</t>
+        </is>
+      </c>
       <c r="T4" t="n">
         <v>51000</v>
       </c>
@@ -829,6 +844,11 @@
       <c r="R5" t="n">
         <v>4614</v>
       </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+        </is>
+      </c>
       <c r="T5" t="n">
         <v>51000</v>
       </c>
@@ -908,6 +928,11 @@
       <c r="R6" t="n">
         <v>4614</v>
       </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+        </is>
+      </c>
       <c r="T6" t="n">
         <v>51000</v>
       </c>
@@ -987,6 +1012,11 @@
       <c r="R7" t="n">
         <v>4614</v>
       </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+        </is>
+      </c>
       <c r="T7" t="n">
         <v>51000</v>
       </c>
@@ -1066,6 +1096,11 @@
       <c r="R8" t="n">
         <v>4610</v>
       </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>IMOBILIZAÇÕES</t>
+        </is>
+      </c>
       <c r="T8" t="n">
         <v>51000</v>
       </c>
@@ -1145,6 +1180,11 @@
       <c r="R9" t="n">
         <v>4613</v>
       </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>OBRAS E INSTALAÇÕES</t>
+        </is>
+      </c>
       <c r="T9" t="n">
         <v>51000</v>
       </c>
@@ -1224,6 +1264,11 @@
       <c r="R10" t="n">
         <v>4817</v>
       </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
+        </is>
+      </c>
       <c r="T10" t="n">
         <v>51000</v>
       </c>
@@ -1303,6 +1348,11 @@
       <c r="R11" t="n">
         <v>4511</v>
       </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>SOCIEDADES CONTROLADAS</t>
+        </is>
+      </c>
       <c r="T11" t="n">
         <v>11101</v>
       </c>
@@ -1382,6 +1432,11 @@
       <c r="R12" t="n">
         <v>4511</v>
       </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>SOCIEDADES CONTROLADAS</t>
+        </is>
+      </c>
       <c r="T12" t="n">
         <v>51000</v>
       </c>
@@ -1461,6 +1516,11 @@
       <c r="R13" t="n">
         <v>4817</v>
       </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
+        </is>
+      </c>
       <c r="T13" t="n">
         <v>51000</v>
       </c>
@@ -1540,6 +1600,11 @@
       <c r="R14" t="n">
         <v>4819</v>
       </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>OUTRAS APLICAÇÕES</t>
+        </is>
+      </c>
       <c r="T14" t="n">
         <v>11101</v>
       </c>
@@ -1619,6 +1684,11 @@
       <c r="R15" t="n">
         <v>4819</v>
       </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>OUTRAS APLICAÇÕES</t>
+        </is>
+      </c>
       <c r="T15" t="n">
         <v>51000</v>
       </c>
@@ -1698,6 +1768,11 @@
       <c r="R16" t="n">
         <v>4810</v>
       </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>OUTRAS APLICAÇÕES</t>
+        </is>
+      </c>
       <c r="T16" t="n">
         <v>12400</v>
       </c>
@@ -1777,6 +1852,11 @@
       <c r="R17" t="n">
         <v>4813</v>
       </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>INTANGÍVEIS E OUTROS INVESTIMENTOS</t>
+        </is>
+      </c>
       <c r="T17" t="n">
         <v>12400</v>
       </c>
@@ -1856,6 +1936,11 @@
       <c r="R18" t="n">
         <v>4810</v>
       </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>OUTRAS APLICAÇÕES</t>
+        </is>
+      </c>
       <c r="T18" t="n">
         <v>12400</v>
       </c>
@@ -1935,6 +2020,11 @@
       <c r="R19" t="n">
         <v>4613</v>
       </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>OBRAS E INSTALAÇÕES</t>
+        </is>
+      </c>
       <c r="T19" t="n">
         <v>51000</v>
       </c>
@@ -1959,77 +2049,82 @@
         <v>2027</v>
       </c>
       <c r="B20" t="n">
-        <v>1220</v>
+        <v>1300</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - MGS</t>
+          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA, MOBILIDADE E PARCERIA - TREM METROPOLITANO</t>
         </is>
       </c>
       <c r="D20" t="n">
         <v>3</v>
       </c>
       <c r="E20" t="n">
-        <v>5381</v>
+        <v>5261</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
+          <t>TREM METROPOLITANO DE BELO HORIZONTE S.A - TREM METROPOLITANO</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="I20" t="n">
-        <v>122</v>
+        <v>783</v>
       </c>
       <c r="J20" t="n">
-        <v>57</v>
+        <v>705</v>
       </c>
       <c r="K20" t="n">
         <v>8</v>
       </c>
       <c r="L20" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="M20" t="n">
-        <v>8002</v>
+        <v>8011</v>
       </c>
       <c r="N20" t="n">
-        <v>12650330</v>
+        <v>1000</v>
       </c>
       <c r="O20" t="n">
         <v>0</v>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4510 - PARTICIPAÇÃO SOCIETÁRIA</t>
         </is>
       </c>
       <c r="R20" t="n">
-        <v>4614</v>
+        <v>4511</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>SOCIEDADES CONTROLADAS</t>
+        </is>
       </c>
       <c r="T20" t="n">
-        <v>51000</v>
+        <v>11101</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
+          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
         </is>
       </c>
     </row>
@@ -2075,7 +2170,7 @@
         <v>8002</v>
       </c>
       <c r="N21" t="n">
-        <v>524600</v>
+        <v>12650330</v>
       </c>
       <c r="O21" t="n">
         <v>0</v>
@@ -2091,7 +2186,12 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>4615</v>
+        <v>4614</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+        </is>
       </c>
       <c r="T21" t="n">
         <v>51000</v>
@@ -2154,7 +2254,7 @@
         <v>8002</v>
       </c>
       <c r="N22" t="n">
-        <v>1000</v>
+        <v>524600</v>
       </c>
       <c r="O22" t="n">
         <v>0</v>
@@ -2166,18 +2266,23 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>4810 - OUTRAS APLICAÇÕES</t>
+          <t>4610 - IMOBILIZAÇÕES</t>
         </is>
       </c>
       <c r="R22" t="n">
-        <v>4810</v>
+        <v>4615</v>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>MÓVEIS E UTENSÍLIOS</t>
+        </is>
       </c>
       <c r="T22" t="n">
-        <v>11101</v>
+        <v>51000</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
+          <t>RECURSOS PRÓPRIOS</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
@@ -2233,7 +2338,7 @@
         <v>8002</v>
       </c>
       <c r="N23" t="n">
-        <v>4842500</v>
+        <v>1000</v>
       </c>
       <c r="O23" t="n">
         <v>0</v>
@@ -2249,14 +2354,19 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>4817</v>
+        <v>4810</v>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>OUTRAS APLICAÇÕES</t>
+        </is>
       </c>
       <c r="T23" t="n">
-        <v>51000</v>
+        <v>11101</v>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>RECURSOS PRÓPRIOS</t>
+          <t>TESOURO ORDINÁRIO - APLICAÇÃO LIVRE</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
@@ -2279,56 +2389,61 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - MGS</t>
         </is>
       </c>
       <c r="D24" t="n">
         <v>3</v>
       </c>
       <c r="E24" t="n">
-        <v>5391</v>
+        <v>5381</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>752</v>
+        <v>122</v>
       </c>
       <c r="J24" t="n">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="K24" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M24" t="n">
-        <v>3004</v>
+        <v>8002</v>
       </c>
       <c r="N24" t="n">
-        <v>228410975</v>
+        <v>4842500</v>
       </c>
       <c r="O24" t="n">
         <v>0</v>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>4610 - IMOBILIZAÇÕES</t>
+          <t>4810 - OUTRAS APLICAÇÕES</t>
         </is>
       </c>
       <c r="R24" t="n">
-        <v>4613</v>
+        <v>4817</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>EQUIPAMENTOS E SOFTWARE</t>
+        </is>
       </c>
       <c r="T24" t="n">
         <v>51000</v>
@@ -2340,12 +2455,12 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
+          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
+          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
         </is>
       </c>
     </row>
@@ -2385,20 +2500,20 @@
         <v>3</v>
       </c>
       <c r="L25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M25" t="n">
-        <v>3005</v>
+        <v>3004</v>
       </c>
       <c r="N25" t="n">
-        <v>426883823</v>
+        <v>228410975</v>
       </c>
       <c r="O25" t="n">
         <v>0</v>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t xml:space="preserve">REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO </t>
+          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -2409,6 +2524,11 @@
       <c r="R25" t="n">
         <v>4613</v>
       </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>OBRAS E INSTALAÇÕES</t>
+        </is>
+      </c>
       <c r="T25" t="n">
         <v>51000</v>
       </c>
@@ -2419,7 +2539,7 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t xml:space="preserve">REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO </t>
+          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
@@ -2464,20 +2584,20 @@
         <v>3</v>
       </c>
       <c r="L26" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M26" t="n">
-        <v>3006</v>
+        <v>3005</v>
       </c>
       <c r="N26" t="n">
-        <v>32235731</v>
+        <v>426883823</v>
       </c>
       <c r="O26" t="n">
         <v>0</v>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
+          <t xml:space="preserve">REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO </t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -2486,7 +2606,12 @@
         </is>
       </c>
       <c r="R26" t="n">
-        <v>4614</v>
+        <v>4613</v>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>OBRAS E INSTALAÇÕES</t>
+        </is>
       </c>
       <c r="T26" t="n">
         <v>51000</v>
@@ -2498,7 +2623,7 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
+          <t xml:space="preserve">REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO </t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
@@ -2543,20 +2668,20 @@
         <v>3</v>
       </c>
       <c r="L27" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="M27" t="n">
-        <v>3009</v>
+        <v>3006</v>
       </c>
       <c r="N27" t="n">
-        <v>56493213</v>
+        <v>32235731</v>
       </c>
       <c r="O27" t="n">
         <v>0</v>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t xml:space="preserve">INVESTIMENTOS PARTICIPAÇÕES SOCIETÁRIAS DA TRANSMISSÃO </t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -2567,6 +2692,11 @@
       <c r="R27" t="n">
         <v>4614</v>
       </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+        </is>
+      </c>
       <c r="T27" t="n">
         <v>51000</v>
       </c>
@@ -2577,7 +2707,7 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t xml:space="preserve">INVESTIMENTOS PARTICIPAÇÕES SOCIETÁRIAS DA TRANSMISSÃO </t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
         </is>
       </c>
       <c r="W27" t="inlineStr">
@@ -2616,26 +2746,26 @@
         <v>752</v>
       </c>
       <c r="J28" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="K28" t="n">
         <v>3</v>
       </c>
       <c r="L28" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="M28" t="n">
-        <v>3001</v>
+        <v>3009</v>
       </c>
       <c r="N28" t="n">
-        <v>1</v>
+        <v>56493213</v>
       </c>
       <c r="O28" t="n">
         <v>0</v>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
+          <t xml:space="preserve">INVESTIMENTOS PARTICIPAÇÕES SOCIETÁRIAS DA TRANSMISSÃO </t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -2644,7 +2774,12 @@
         </is>
       </c>
       <c r="R28" t="n">
-        <v>4613</v>
+        <v>4614</v>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+        </is>
       </c>
       <c r="T28" t="n">
         <v>51000</v>
@@ -2656,12 +2791,12 @@
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
+          <t xml:space="preserve">INVESTIMENTOS PARTICIPAÇÕES SOCIETÁRIAS DA TRANSMISSÃO </t>
         </is>
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t xml:space="preserve">GERAÇÃO DE ENERGIA ELÉTRICA </t>
+          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
         </is>
       </c>
     </row>
@@ -2701,20 +2836,20 @@
         <v>3</v>
       </c>
       <c r="L29" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>3007</v>
+        <v>3001</v>
       </c>
       <c r="N29" t="n">
-        <v>121588957</v>
+        <v>1</v>
       </c>
       <c r="O29" t="n">
         <v>0</v>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t xml:space="preserve"> REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
+          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -2723,7 +2858,12 @@
         </is>
       </c>
       <c r="R29" t="n">
-        <v>4614</v>
+        <v>4613</v>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>OBRAS E INSTALAÇÕES</t>
+        </is>
       </c>
       <c r="T29" t="n">
         <v>51000</v>
@@ -2735,7 +2875,7 @@
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t xml:space="preserve"> REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
+          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
         </is>
       </c>
       <c r="W29" t="inlineStr">
@@ -2780,20 +2920,20 @@
         <v>3</v>
       </c>
       <c r="L30" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M30" t="n">
-        <v>3008</v>
+        <v>3007</v>
       </c>
       <c r="N30" t="n">
-        <v>28627843</v>
+        <v>121588957</v>
       </c>
       <c r="O30" t="n">
         <v>0</v>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
+          <t xml:space="preserve"> REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -2804,6 +2944,11 @@
       <c r="R30" t="n">
         <v>4614</v>
       </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+        </is>
+      </c>
       <c r="T30" t="n">
         <v>51000</v>
       </c>
@@ -2814,7 +2959,7 @@
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
+          <t xml:space="preserve"> REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
         </is>
       </c>
       <c r="W30" t="inlineStr">
@@ -2859,20 +3004,20 @@
         <v>3</v>
       </c>
       <c r="L31" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="M31" t="n">
-        <v>3014</v>
+        <v>3008</v>
       </c>
       <c r="N31" t="n">
-        <v>1080197578</v>
+        <v>28627843</v>
       </c>
       <c r="O31" t="n">
         <v>0</v>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS DA GERAÇÃO</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -2883,6 +3028,11 @@
       <c r="R31" t="n">
         <v>4614</v>
       </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+        </is>
+      </c>
       <c r="T31" t="n">
         <v>51000</v>
       </c>
@@ -2893,7 +3043,7 @@
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS DA GERAÇÃO</t>
+          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
         </is>
       </c>
       <c r="W31" t="inlineStr">
@@ -2911,18 +3061,18 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - CEMIG DISTRIBUIDORA</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="D32" t="n">
         <v>3</v>
       </c>
       <c r="E32" t="n">
-        <v>5401</v>
+        <v>5391</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
+          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
         </is>
       </c>
       <c r="H32" t="n">
@@ -2932,26 +3082,26 @@
         <v>752</v>
       </c>
       <c r="J32" t="n">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="K32" t="n">
         <v>3</v>
       </c>
       <c r="L32" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="M32" t="n">
-        <v>3002</v>
+        <v>3014</v>
       </c>
       <c r="N32" t="n">
-        <v>5320034427</v>
+        <v>1080197578</v>
       </c>
       <c r="O32" t="n">
         <v>0</v>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t xml:space="preserve">EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD) </t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS DA GERAÇÃO</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -2962,6 +3112,11 @@
       <c r="R32" t="n">
         <v>4614</v>
       </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+        </is>
+      </c>
       <c r="T32" t="n">
         <v>51000</v>
       </c>
@@ -2972,12 +3127,12 @@
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t xml:space="preserve">EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD) </t>
+          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS DA GERAÇÃO</t>
         </is>
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
+          <t xml:space="preserve">GERAÇÃO DE ENERGIA ELÉTRICA </t>
         </is>
       </c>
     </row>
@@ -3017,20 +3172,20 @@
         <v>3</v>
       </c>
       <c r="L33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M33" t="n">
-        <v>3003</v>
+        <v>3002</v>
       </c>
       <c r="N33" t="n">
-        <v>250370467</v>
+        <v>5320034427</v>
       </c>
       <c r="O33" t="n">
         <v>0</v>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t xml:space="preserve">MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO </t>
+          <t xml:space="preserve">EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD) </t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -3041,6 +3196,11 @@
       <c r="R33" t="n">
         <v>4614</v>
       </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+        </is>
+      </c>
       <c r="T33" t="n">
         <v>51000</v>
       </c>
@@ -3051,10 +3211,94 @@
       </c>
       <c r="V33" t="inlineStr">
         <is>
+          <t xml:space="preserve">EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD) </t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B34" t="n">
+        <v>1220</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - CEMIG DISTRIBUIDORA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>3</v>
+      </c>
+      <c r="E34" t="n">
+        <v>5401</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>25</v>
+      </c>
+      <c r="I34" t="n">
+        <v>752</v>
+      </c>
+      <c r="J34" t="n">
+        <v>72</v>
+      </c>
+      <c r="K34" t="n">
+        <v>3</v>
+      </c>
+      <c r="L34" t="n">
+        <v>3</v>
+      </c>
+      <c r="M34" t="n">
+        <v>3003</v>
+      </c>
+      <c r="N34" t="n">
+        <v>250370467</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
           <t xml:space="preserve">MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO </t>
         </is>
       </c>
-      <c r="W33" t="inlineStr">
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>4610 - IMOBILIZAÇÕES</t>
+        </is>
+      </c>
+      <c r="R34" t="n">
+        <v>4614</v>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>MÁQUINAS, APARELHOS E EQUIPAMENTOS</t>
+        </is>
+      </c>
+      <c r="T34" t="n">
+        <v>51000</v>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>RECURSOS PRÓPRIOS</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO </t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
         <is>
           <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
         </is>

</xml_diff>